<commit_message>
Accept all 10 pending proposals (445 -> 455) [platform-engineering, ai-engineer, product-manager]
Graduated per the maintainer checklist: OPS-31 thinnest viable platform
scoping, OPS-32 cognitive-load management, SEC-18 guardrails & policy as
code (platform); SWE-10 AI-augmented development, AI-21 AI risk
governance (AI engineer); PM-15..19 discovery-craft cluster (product
manager - the PM domain now has 19 capabilities, all used by the role).
All 12 proposed placeholders re-pointed to real ids across role.yaml,
ladder.csv capability columns, and ladder.md link tables; renders
regenerated; contrib/ empty; domains.csv and README counts updated.
Fix: render_role_links.py now rewrites already-tabled cells whose links
still point into contrib/ once role.yaml carries the accepted id -
previously graduated cells stayed stale. Root workbook still lags (no
generator; holds 421 ids).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roles/ai-engineer/ladder.xlsx
+++ b/roles/ai-engineer/ladder.xlsx
@@ -1129,7 +1129,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>SWE-10</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>AI-21</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">

</xml_diff>

<commit_message>
feat(roles): derive sourced ai-engineer ladder
Retrofit roles/ai-engineer from schema-migrated-but-unsourced to fully
sourced derived rendering: every mapping now carries a bibliography
source and a per-competency, per-level why grounded in the mapped
capability's actual P1-P6 catalog text. All 43 anchors resolve to
existing bibliography keys (23 exact, 20 close catalog-adjacent
substitutes) with zero new bibliography rows. Evidence semantically
audited across all 258 cells; 24 rewritten (two self-sourced
capabilities where the catalog text was circularly distilled from this
role's own prior ladder, plus two more that paraphrased rather than
instantiated their bar), zero discarded.
</commit_message>
<xml_diff>
--- a/roles/ai-engineer/ladder.xlsx
+++ b/roles/ai-engineer/ladder.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Competency Matrix" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Rating Template" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sources" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sources &amp; Theory" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -696,20 +696,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="55" customWidth="1" min="8" max="8"/>
     <col width="55" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
     <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -735,35 +736,40 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Theory Anchor</t>
+          <t>What it covers</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Theory anchor &amp; why</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>E1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>E2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>E3</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>E4</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>E6</t>
         </is>
@@ -792,37 +798,42 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Kleppmann, *Designing Data-Intensive Applications* (2017)</t>
+          <t>Structures software — modules, boundaries, interfaces.</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Depth: explains the system's architecture in their own words and implements designs specified by others, asking when a boundary is unclear - including where model calls sit in the request path and why they are isolated behind interfaces. Scope: a task within an existing design.</t>
+          <t>Kleppmann, Designing Data-Intensive Applications: The Big Ideas Behind Reliable, Scalable, and Maintainable Systems (O'Reilly, 2017) — AI features live inside distributed systems; the data-flow and consistency trade-offs Kleppmann catalogs are the load-bearing design decisions, model calls included.</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Depth: designs a component and writes the short design note for it, naming at least one alternative considered; isolates model calls behind clear interfaces and uses established patterns correctly. Scope: a component and its immediate neighbors.</t>
+          <t>Depth: Implements designs specified by others; asks why, not just how. Evidenced by: Explains the system's architecture in their own words. Scope: task.</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Depth: selects patterns by trade-off in design docs that name the alternatives and failure modes, designing for evolution - swappable models, versioned prompts, isolated nondeterminism - and catches coupling and scaling problems in others' designs before build. Scope: owns architecture for an AI capability and runs its design reviews.</t>
+          <t>Depth: Designs sound components; understands coupling, cohesion, interface design. Evidenced by: Designs a component and writes the short design note for it. Scope: component.</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>Depth: writes the reference architectures other teams instantiate and arbitrates cross-team design disputes with written trade-off analysis. Scope: multiple teams build against their designs.</t>
+          <t>Depth: Designs systems for evolution: clean seams, versioned interfaces, replaceable parts. Evidenced by: Selects patterns by trade-off in design docs that name the alternatives and failure modes. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets the architectural direction for AI systems across the org, retiring dead-end patterns explicitly and removing the systemic obstacles that block the target state. Scope: organization.</t>
+          <t>Depth: Mastery of architecture for complex systems; sets patterns and prevents drift. Evidenced by: Writes the reference architectures other teams instantiate. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>Depth: defines the company's long-horizon technical bets for AI systems - build vs. buy, platform vs. product - in writing executives and engineers both act on. Scope: company.</t>
+          <t>Depth: Sets multi-year architecture direction across the org. Evidenced by: Sets the architectural direction for AI systems across the org. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Authoritative and externally credible; defines architectural approach others follow. Evidenced by: Defines the company's long-horizon technical bets for AI systems. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -849,37 +860,42 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Bloch, "How to Design a Good API and Why It Matters" (2006)</t>
+          <t>Designs clean, durable interfaces between systems.</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Depth: implements endpoints to an existing API contract, including error responses, and flags mismatches between spec and behavior. Scope: single endpoints.</t>
+          <t>Fielding, Architectural Styles and the Design of Network-based Software Architectures (PhD dissertation, University of California Irvine, 2000) — Bloch's original API-design essay has no bibliography entry; Fielding's REST dissertation is the foundational, catalog-sourced text SWE-07's own P1/P2 bars already cite for interface design, and AI features leak nondeterminism to consumers unless the contract deliberately contains it.</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Depth: designs the API surface for a component - versioning, streaming semantics, and explicit error shapes for model failures included - and documents it well enough that a consumer needs no walkthrough. Scope: a component's consumers.</t>
+          <t>Depth: Understands HTTP/REST and the deploy pipeline; makes guided changes. Evidenced by: Implements endpoints to an existing API contract, including error responses, and flags mismatches between spec and behavior. Scope: task.</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Depth: designs contracts that isolate consumers from model and provider changes - streaming, partial failure, and nondeterminism handled explicitly in the interface - and rejects designs that leak provider details or raw model output to callers. Scope: the APIs of a capability; reviews neighbors' contracts.</t>
+          <t>Depth: Designs clean APIs; understands rate limits, retries, timeouts, idempotency. Evidenced by: Designs the API surface for a component and documents it well enough that a consumer needs no walkthrough. Scope: component.</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets the API conventions multiple teams follow for model-backed services and retires inconsistent legacy surfaces with migration paths. Scope: multiple teams.</t>
+          <t>Depth: Designs services for scale and cost; understands distributed failure modes. Evidenced by: Designs contracts that isolate consumers from model and provider changes and rejects designs that leak provider details to callers. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>Depth: drives the org's interface strategy - which capabilities become shared platforms, and the deprecation policy that keeps the surface coherent. Scope: organization.</t>
+          <t>Depth: Expert in platform/service design (multi-tenancy, capacity, shared services). Evidenced by: Sets the API conventions multiple teams follow for model-backed services and retires inconsistent legacy surfaces with migration paths. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>Depth: shapes the company's external and partner-facing AI interfaces, balancing product commitments against provider volatility. Scope: company and ecosystem.</t>
+          <t>Depth: Sets interface standards used across the org. Evidenced by: Drives the org's interface strategy — which capabilities become shared platforms, and the deprecation policy that keeps the surface coherent. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines company-wide API approach; trusted with irreversible interface bets. Evidenced by: Shapes the company's external and partner-facing AI interfaces, balancing product commitments against provider volatility. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -906,37 +922,42 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>McConnell, *Code Complete* (2nd ed., 2004)</t>
+          <t>Produces correct, readable, idiomatic code.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Depth: writes working, readable code in the team's primary language and debugs their own changes to root cause before asking for help. Scope: small changes delivered with review and guidance.</t>
+          <t>McConnell, Code Complete: A Practical Handbook of Software Construction, 2nd Edition (Microsoft Press, 2004) — AI code is still code; McConnell's implementation discipline is the base layer the rest of the ladder stands on.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Depth: implements features of moderate complexity independently, handling error paths, async patterns, and concurrency basics correctly in idiomatic code. Scope: a component.</t>
+          <t>Depth: Writes working, readable code in the team's language; debugs own changes. Evidenced by: Implements the retry-with-backoff helper for a flaky provider call exactly to spec and finds the off-by-one in their own token-counting logic before it reaches review. Scope: task.</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Depth: writes code others use as the reference for the stack and debugs the hard problems - race conditions, memory pressure, nondeterministic failures - that stall teammates. Scope: raises implementation quality across a capability.</t>
+          <t>Depth: Proficient in the primary language/ecosystem; handles errors, async and concurrency basics correctly. Evidenced by: Ships the async job that reprocesses failed embedding batches, handling partial-batch failures and concurrent writes to the vector store without a teammate having to point them out. Scope: component.</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Depth: solves the implementation problems other teams can't, working across multiple stacks and paradigms, and lands the patterns they use as shared libraries. Scope: multiple teams.</t>
+          <t>Depth: Code is a reference others learn from; debugs the hard problems (races, memory, nondeterminism). Evidenced by: Writes the concurrent request-batching code newer engineers copy verbatim, and is the one who finds the race condition in the streaming-response handler that only shows up under load. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Depth: anticipates where implementations break at scale and shapes org-wide engineering practice through visible, load-bearing code. Scope: organization.</t>
+          <t>Depth: Mastery across multiple stacks/paradigms; solves problems others can't; sets implementation patterns. Evidenced by: Rewrites the team's Python retrieval service in Rust for a client with different concurrency guarantees, solving a memory-pressure bug in the vector index that stumped two other engineers. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Depth: authors foundational primitives used company-wide and is the benchmark for implementation depth. Scope: company.</t>
+          <t>Depth: Sets implementation standards adopted across the org; anticipates where code breaks at scale. Evidenced by: Sets the org's async-error-handling convention after a postmortem shows three teams' AI services failed the same way under provider timeout spikes. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Industry-level depth; authors foundational primitives and idioms others build on. Evidenced by: Writes the request-batching primitive now vendored into every AI service's client library company-wide, the reference implementation new hires study. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -963,37 +984,42 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Winters, Manshreck &amp; Wright, *Software Engineering at Google* (2020)</t>
+          <t>Keeps code healthy, modular and maintainable.</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Depth: submits small, reviewable changes that pass CI first try more often than not and responds to review feedback by fixing the pattern, not just the line. Scope: their own changes.</t>
+          <t>Winters, Manshreck &amp; Wright, Software Engineering at Google: Lessons Learned from Programming Over Time (O'Reilly, 2020) — Review is where a team's quality bar is actually enforced, and Winters, Manshreck &amp; Wright's account of code health at Google scale is written for exactly this discipline, with AI-generated code raising the volume it must absorb.</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Depth: reviews peers' changes with substantive comments - correctness, naming, missed edge cases - and keeps the code they touch consistently readable, separating prototype code from production paths without being told. Scope: a component's codebase.</t>
+          <t>Depth: Writes functional, readable code; uses version control correctly; responds well to review. Evidenced by: Submits small, reviewable changes that pass CI first try more often than not and responds to review feedback by fixing the pattern, not just the line. Scope: task.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Depth: holds the quality bar in review for a whole domain, including AI-generated code, articulating why a change is risky rather than just that it is, and pays down debt deliberately rather than opportunistically. Scope: a capability; the reviewer others request.</t>
+          <t>Depth: Writes clean, documented, modular code; gives useful review feedback. Evidenced by: Reviews peers' changes with substantive comments and keeps the code they touch consistently readable. Scope: component.</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Depth: codifies review and code-health standards multiple teams adopt - lint rules, prompt-versioning conventions, review norms - and measurably reduces defect escape in the areas they steward. Scope: multiple teams.</t>
+          <t>Depth: Designs for maintainability; leads refactors of problem areas; review feedback teaches. Evidenced by: Holds the quality bar in review for a whole domain, including AI-generated code, articulating why a change is risky rather than just that it is. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Depth: changes how the org reviews and maintains code - tooling, norms, and the standards for machine-authored changes. Scope: organization.</t>
+          <t>Depth: Expert in code health at scale (shared libraries, deprecations, large migrations). Evidenced by: Codifies review and code-health standards multiple teams adopt and measurably reduces defect escape in the areas they steward. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets the company's engineering quality bar, cited when quality trade-offs reach executive decisions. Scope: company.</t>
+          <t>Depth: Shapes org-wide engineering standards for long-lived codebases. Evidenced by: Changes how the org reviews and maintains code — tooling, norms, and the standards for machine-authored changes. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines what good engineering looks like company-wide; externally recognized. Evidenced by: Sets the company's engineering quality bar, cited when quality trade-offs reach executive decisions. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1020,37 +1046,42 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Agans, *Debugging: The 9 Indispensable Rules* (2002)</t>
+          <t>Diagnoses defects and anomalies methodically.</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Depth: reproduces a reported bug and bisects it to a candidate cause with guidance, reading logs and stack traces before asking for help. Scope: bugs in their own tasks.</t>
+          <t>Zeller, Why Programs Fail: A Guide to Systematic Debugging, 2nd Edition (Morgan Kaufmann, 2009) — Agans' rules have no bibliography entry; Zeller's systematic-debugging text is the catalog-sourced substitute SWE-06 already anchors on, and model-backed systems add nondeterminism on top of ordinary bugs, so disciplined fault isolation is what separates the two.</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Depth: isolates faults across service boundaries unaided, distinguishing deterministic code bugs from model-behavior variance before escalating. Scope: their component and its direct dependencies.</t>
+          <t>Depth: Debugs issues in own code with support; uses basic tooling. Evidenced by: Reproduces a reported bug and bisects it to a candidate cause with guidance, reading logs and stack traces before asking for help. Scope: task.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Depth: debugs the hardest failures in a capability, including intermittent model-dependent ones, and writes the reproduction others rerun. Scope: a capability; teammates bring them the stuck cases.</t>
+          <t>Depth: Independently diagnoses defects in own area systematically. Evidenced by: Isolates faults across service boundaries unaided, distinguishing deterministic code bugs from model-behavior variance before escalating. Scope: component.</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Depth: untangles cross-team failures where no single owner sees the whole path and leaves behind the instrumentation that makes the next one cheap. Scope: multiple teams' systems.</t>
+          <t>Depth: Leads diagnosis of hard, cross-cutting failures; root cause not symptoms. Evidenced by: Debugs the hardest failures in a capability, including intermittent model-dependent ones, and writes the reproduction others rerun. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Depth: spots systemic failure classes from incident patterns across the org and drives the architectural fixes. Scope: organization.</t>
+          <t>Depth: Expert at the rare/systemic failures; builds tooling that makes them visible. Evidenced by: Untangles cross-team failures where no single owner sees the whole path and leaves behind the instrumentation that makes the next one cheap. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Depth: is the debugger of last resort for company-critical AI incidents and turns each into a durable prevention mechanism. Scope: company.</t>
+          <t>Depth: The person called for the worst failures; sets diagnostic practice org-wide. Evidenced by: Spots systemic failure classes from incident patterns across the org and drives the architectural fixes. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Authority on diagnosis; advances the discipline. Evidenced by: Is the debugger of last resort for company-critical AI incidents and turns each into a durable prevention mechanism. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1077,37 +1108,42 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Vocke, "The Practical Test Pyramid" (martinfowler.com, 2018); Husain, "Your AI Product Needs Evals" (2024)</t>
+          <t>Designs tests that give real confidence to ship.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Depth: writes unit tests for the deterministic parts of a change - parsing, templating, tool schemas - and can say which behaviors are testable versus eval-able when asked. Scope: their task.</t>
+          <t>Cohn, Succeeding with Agile: Software Development Using Scrum (Addison-Wesley, 2009) — Vocke's blog post and Husain's article have no bibliography entries; Cohn's Succeeding with Agile is where the test pyramid this competency splits from evals actually originates, and LLM systems need two verification regimes that confusing breaks both.</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Depth: draws the test/eval boundary correctly for a component - mocks model calls in unit tests, routes behavioral claims to evals - and keeps CI fast and free of flaky model-dependent assertions. Scope: a component's test suite.</t>
+          <t>Depth: Writes unit tests with guidance; tests own changes before merging. Evidenced by: Writes unit tests for the deterministic parts of a change and can say which behaviors are testable versus eval-able when asked. Scope: task.</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Depth: designs the verification strategy for a capability - what runs in CI, what runs as evals, what only production monitoring can catch - and rejects flaky model-in-the-loop tests in review with a stated rule. Scope: a capability; the split they define is what teammates follow.</t>
+          <t>Depth: Applies the testing pyramid; everything shipped arrives tested; mocks dependencies sensibly. Evidenced by: Draws the test/eval boundary correctly for a component and keeps CI fast and free of flaky model-dependent assertions. Scope: component.</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Depth: standardizes the test-vs-eval discipline across teams with shared fixtures, replay harnesses, and CI policy for what may block a merge. Scope: multiple teams' pipelines.</t>
+          <t>Depth: Designs testable systems (contract, property-based, replay from prod); owns a test strategy. Evidenced by: Designs the verification strategy for a capability and rejects flaky model-in-the-loop tests in review with a stated rule. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the org's verification strategy for AI systems, funding the harnesses that make the right split cheap and killing the theater. Scope: organization.</t>
+          <t>Depth: Expert in test strategy at scale (test data, environments, deployment safety). Evidenced by: Standardizes the test-vs-eval discipline across teams with shared fixtures, replay harnesses, and CI policy for what may block a merge. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets company policy for what 'verified' means for AI products, traceable from CI to eval to production evidence. Scope: company.</t>
+          <t>Depth: Sets testing/verification discipline across the org. Evidenced by: Owns the org's verification strategy for AI systems, funding the harnesses that make the right split cheap and killing the theater. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes the company-wide quality culture; advances verification practice. Evidenced by: Sets company policy for what 'verified' means for AI products, traceable from CI to eval to production evidence. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1134,37 +1170,42 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>DORA, *Accelerate State of DevOps Report* (2024), AI adoption findings</t>
+          <t>Works effectively with AI coding tools and agents while remaining accountable for the output - calibrating what to delegate and what to hand-write, verifying generated changes with the same rigor as hand-written ones, and setting the review and provenance practices that keep quality intact.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Depth: uses AI coding tools with the output treated as a draft - reads every generated line, tests it, and can explain any part of the diff when asked. Scope: their own tasks.</t>
+          <t>DORA (Google Cloud), Accelerate State of DevOps Report 2024 (2024) — SWE-10's own catalog profile is written directly from DORA's 2024 AI-adoption findings: AI assistance boosts throughput but hurts stability without verification discipline, and DORA is the source that measured that trade-off.</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Depth: calibrates when generation helps and when it misleads - boilerplate yes, subtle invariants no - and catches plausible-but-wrong generated code before review; their AI-assisted diffs pass review at the same rate as hand-written ones. Scope: a component's workflow.</t>
+          <t>Depth: Uses AI coding tools with the output treated as a draft - reads every generated line, tests it, and can explain any part of the diff when asked. Evidenced by: Has the agent draft the schema-migration script, then reads and runs every line by hand and can walk a reviewer through why the down-migration is safe. Scope: task.</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets the norms for AI-assisted work on their capability - what may be delegated, what review it requires, how provenance shows up - and coaches others out of over-trust and under-use. Scope: a capability's development practice.</t>
+          <t>Depth: Calibrates when generation helps and when it misleads for the work at hand; catches plausible-but-wrong generated code before review, and their AI-assisted changes pass review at the same rate as hand-written ones. Evidenced by: Accepts the agent's generated boilerplate for a new API route unchanged but rewrites its generated cache-invalidation logic by hand after spotting a stale-read bug; their AI-assisted PRs land clean at the same rate as their hand-written ones. Scope: component.</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Depth: defines AI-assisted engineering practice across teams - where agents run in the delivery lifecycle, what gates their output - backed by throughput and defect data, not vendor claims. Scope: multiple teams.</t>
+          <t>Depth: Sets the norms for AI-assisted work in a domain - what may be delegated to agents, what verification it requires, how provenance is noted in review - and coaches others out of over-trust and under-use. Evidenced by: Writes the team's rule that agents may draft data-pipeline glue code unattended but never touch auth logic without a human diff review, and talks a skeptical teammate into trying agent-assisted refactors for mechanical renames instead of hand-editing forty files. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Depth: drives the org's AI-augmented engineering strategy, selecting tooling, measuring its effect on delivery outcomes, and adjusting policy from the data. Scope: organization.</t>
+          <t>Depth: Defines AI-assisted engineering practice across teams - where agents run in the delivery lifecycle, what gates their output - justified by throughput and defect data rather than vendor claims. Evidenced by: Decides, with six months of defect-escape data across three teams, which pipeline stages autonomous coding agents may run in unattended and which require a human gate before merge. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>Depth: shapes how the company builds software in the AI era and is the credible voice on what changes and what doesn't. Scope: company.</t>
+          <t>Depth: Drives an organization's AI-augmented engineering strategy - tooling selection, workflow redesign, skill expectations - and adjusts policy from measured delivery outcomes. Evidenced by: Picks the org's standard coding-agent tooling after a bake-off, redesigns the PR template around provenance tags, and walks back a workflow change once the data shows it slowed incident response. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes how software engineering itself changes with AI at company and industry level; a credible public voice on what changes and what doesn't. Evidenced by: Writes the engineering blog post other companies cite when re-tooling their own build process around agentic coding. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1191,37 +1232,42 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Anthropic and OpenAI prompt-engineering guides (2023-2025)</t>
+          <t>Builds reliable features on top of language models.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Depth: makes targeted edits to existing prompts and verifies the effect against known cases before committing, following the team's prompt-versioning convention. Scope: single prompts within a task.</t>
+          <t>Brown et al., Language Models are Few-Shot Learners, NeurIPS 2020 — Anthropic and OpenAI's prompt-engineering guides have no bibliography entries; Brown et al.'s GPT-3 paper is where few-shot prompting — the technique AI-01 P2 names directly — was first demonstrated, and prompts are load-bearing program text that versioned, tested iteration turns from folklore into engineering.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Depth: writes production prompts from scratch - role, constraints, output schema, few-shot examples - and iterates against a saved sample set rather than one lucky output. Scope: a component's prompts.</t>
+          <t>Depth: Understands LLM basics (tokens, context windows, temperature, system prompts); calls model APIs correctly. Evidenced by: Makes targeted edits to existing prompts and verifies the effect against known cases before committing, following the team's prompt-versioning convention. Scope: task.</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Depth: treats prompts as versioned, eval-gated artifacts; diagnoses failures to the responsible prompt section, documents why each instruction exists, and knows when the fix is retrieval or tooling, not wording. Scope: a capability; teammates adopt their prompt patterns.</t>
+          <t>Depth: Writes effective prompts; uses structured outputs, function calling and streaming; understands model differences and pricing. Evidenced by: Writes production prompts from scratch and iterates against a saved sample set rather than one lucky output. Scope: component.</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Depth: establishes prompt-engineering standards across teams - templates, review checklists, migration playbooks for model changes - and untangles the prompt failures others are stuck on. Scope: multiple teams.</t>
+          <t>Depth: Expert prompt/context design (few-shot, decomposition, chaining); knows when fine-tuning beats prompting (rarely); designs for model swappability. Evidenced by: Treats prompts as versioned, eval-gated artifacts and diagnoses failures to the responsible prompt section. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Depth: drives org-wide prompt and context craft, deciding where prompting ends and fine-tuning or tool-building begins, and re-baselining systematically when providers ship new models. Scope: organization.</t>
+          <t>Depth: Mastery of model behavior across providers and versions; designs upgrade-migration strategies; squeezes capability others can't. Evidenced by: Establishes prompt-engineering standards across teams and untangles the prompt failures others are stuck on. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>Depth: represents the state of the art to the company, resetting practice when model generations obsolete current techniques. Scope: company and industry.</t>
+          <t>Depth: Deep expertise; anticipates capability shifts (new modalities, reasoning models) and repositions ahead of them. Evidenced by: Drives org-wide prompt and context craft, deciding where prompting ends and fine-tuning or tool-building begins. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Authority on applied LLM engineering; may influence industry practice. Evidenced by: Represents the state of the art to the company, resetting practice when model generations obsolete current techniques. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1248,37 +1294,42 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Huyen, *AI Engineering* (2025)</t>
+          <t>Builds reliable features on top of language models.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Depth: integrates a specified model through the team's client layer - auth, retries, timeouts, streaming - per existing patterns. Scope: one integration point.</t>
+          <t>Bommasani et al., On the Opportunities and Risks of Foundation Models, Stanford CRFM (2021) — Huyen's AI Engineering (2025) has no bibliography entry; Bommasani et al.'s foundation-models survey is the catalog-adjacent source AI-01's own P4-P6 sourcing already draws on for cross-provider capability shifts, and model choice is an engineering trade-off across quality, latency, cost and provider risk, not a leaderboard beauty contest.</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Depth: runs a small structured comparison before picking a model for a feature - quality on real samples, latency, price - and records the result; handles provider quirks in code, not tribal knowledge. Scope: a component.</t>
+          <t>Depth: Understands LLM basics (tokens, context windows, temperature, system prompts); calls model APIs correctly. Evidenced by: Integrates a specified model through the team's client layer per existing patterns. Scope: task.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns model choice for a capability - including fine-tune vs. prompt vs. retrieval trade-offs - re-benchmarks when providers ship new models, and swaps models behind stable interfaces without consumer churn. Scope: a capability; their comparisons are reused by others.</t>
+          <t>Depth: Writes effective prompts; uses structured outputs, function calling and streaming; understands model differences and pricing. Evidenced by: Runs a small structured comparison before picking a model for a feature and records the result. Scope: component.</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Depth: defines the model-selection playbook and abstraction layers multiple teams use, making provider swaps routine instead of rewrites. Scope: multiple teams.</t>
+          <t>Depth: Expert prompt/context design (few-shot, decomposition, chaining); knows when fine-tuning beats prompting (rarely); designs for model swappability. Evidenced by: Owns model choice for a capability, re-benchmarks when providers ship new models, and swaps models behind stable interfaces without consumer churn. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets the org's model portfolio strategy - hosted vs. self-hosted, single vs. multi-provider - with cost and risk analysis leadership signs off on. Scope: organization.</t>
+          <t>Depth: Mastery of model behavior across providers and versions; designs upgrade-migration strategies; squeezes capability others can't. Evidenced by: Defines the model-selection playbook and abstraction layers multiple teams use, making provider swaps routine instead of rewrites. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the company's model-sourcing strategy and its biggest bets - build, fine-tune, or buy - and negotiates the strategic provider commitments behind them. Scope: company.</t>
+          <t>Depth: Deep expertise; anticipates capability shifts (new modalities, reasoning models) and repositions ahead of them. Evidenced by: Sets the org's model portfolio strategy with cost and risk analysis leadership signs off on. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Authority on applied LLM engineering; may influence industry practice. Evidenced by: Owns the company's model-sourcing strategy and its biggest bets and negotiates the strategic provider commitments behind them. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1305,37 +1356,42 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Schick et al., "Toolformer: Language Models Can Teach Themselves to Use Tools" (2023)</t>
+          <t>Validates untrusted data into precise types once at every system boundary (network, storage, configuration, third parties) and propagates a single source of type truth across client, server, and wire so contracts cannot silently drift.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Depth: validates model outputs against a given schema and handles rejects rather than trusting parses. Scope: one integration point.</t>
+          <t>King, Parse, Don't Validate (lexi-lambda.github.io, 2019) — Schick et al.'s Toolformer paper is about teaching models to call tools, not schema design as such; King's "Parse, Don't Validate" is SWE-09's own P1/P2 anchor and states the exact discipline this competency needs — validate once at the boundary and propagate a single source of type truth — since the schema is the contract between probabilistic text and deterministic code.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Depth: designs output schemas and tool signatures the model reliably satisfies, measuring parse and validation failure rates. Scope: a component's model I/O.</t>
+          <t>Depth: Uses the codebase's shared contract types and schema validators at boundaries rather than hand-casting external data, and can point to where a type is checked at runtime. Evidenced by: Validates model outputs against a given schema and handles rejects rather than trusting parses. Scope: task.</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the structured-I/O layer for a capability - schema evolution, repair strategies, when to constrain decoding versus post-validate - with failure rates on a dashboard. Scope: a capability; teams copy their schema patterns.</t>
+          <t>Depth: Puts runtime validation at every I/O boundary they touch — requests, messages, configuration — deriving static types from the runtime schemas so compile-time and runtime cannot drift. Evidenced by: Designs output schemas and tool signatures the model reliably satisfies, measuring parse and validation failure rates. Scope: component.</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets cross-team standards for tool definitions and output contracts, and audits integrations that skip them. Scope: multiple teams.</t>
+          <t>Depth: Designs end-to-end type integrity for a capability — schema-first contracts, generated clients, contract drift caught in continuous integration — and blocks unsound casts and unvalidated edges in review. Evidenced by: Owns the structured-I/O layer for a capability — schema evolution, repair strategies, when to constrain decoding versus post-validate. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the org's model-I/O reliability strategy, driving shared validation infrastructure. Scope: organization.</t>
+          <t>Depth: Builds the code-generation and contract-typing infrastructure multiple teams inherit, making boundary safety the default rather than a discipline, and resolves cross-team type drift at its source. Evidenced by: Sets cross-team standards for tool definitions and output contracts and audits integrations that skip them. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Depth: defines company-wide norms for machine-actionable model output, including what external partners may depend on. Scope: company.</t>
+          <t>Depth: Sets the organization's boundary-safety standard and the platform tooling that enforces it, with incident evidence showing the failure classes it removed. Evidenced by: Owns the org's model-I/O reliability strategy, driving shared validation infrastructure. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Owns contract-integrity strategy across products and external interfaces where a broken contract is a business event, and advances the state of practice publicly. Evidenced by: Defines company-wide norms for machine-actionable model output, including what external partners may depend on. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1362,37 +1418,42 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Lewis et al., "Retrieval-Augmented Generation for Knowledge-Intensive NLP Tasks" (NeurIPS 2020)</t>
+          <t>Grounds models in the right knowledge.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Depth: runs and modifies an existing ingestion/retrieval pipeline - chunking, embedding, indexing - and verifies retrieval hits by inspection. Scope: a task.</t>
+          <t>Lewis et al., Retrieval-Augmented Generation for Knowledge-Intensive NLP Tasks, NeurIPS 2020 — Lewis et al.'s RAG paper is where retrieval-augmented generation for knowledge-intensive tasks was introduced, and most production quality problems in knowledge features are retrieval problems wearing a model costume.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Depth: builds a retrieval pipeline for a corpus end to end and measures retrieval quality (recall on labeled queries) separately from answer quality. Scope: a component.</t>
+          <t>Depth: Understands embeddings, similarity search and why grounding reduces hallucination. Evidenced by: Runs and modifies an existing ingestion/retrieval pipeline and verifies retrieval hits by inspection. Scope: task.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Depth: diagnoses failures to the responsible stage - chunking, embedding, ranking, or synthesis - with evidence, and chooses hybrid, re-ranking, or structured-lookup strategies by measured trade-off, owning the ingestion, indexing, and freshness story. Scope: owns retrieval for a capability.</t>
+          <t>Depth: Builds standard RAG pipelines (chunking, embedding, retrieval, reranking); manages context budgets deliberately. Evidenced by: Builds a retrieval pipeline for a corpus end to end and measures retrieval quality separately from answer quality. Scope: component.</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Depth: designs the retrieval architecture several teams share - index topology, freshness SLAs, evaluation harness - and consolidates duplicated pipelines into shared infrastructure. Scope: multiple teams.</t>
+          <t>Depth: Designs retrieval quality systems (hybrid search, reranking, freshness, citation, memory for multi-turn). Evidenced by: Diagnoses failures to the responsible stage with evidence and chooses hybrid, re-ranking, or structured-lookup strategies by measured trade-off. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets the org's knowledge-grounding strategy - what corpora exist, who owns them, entitlement-aware access, and quality accountability. Scope: organization.</t>
+          <t>Depth: Expert in retrieval at scale (index strategy, multi-source federation, permission-aware retrieval). Evidenced by: Designs the retrieval architecture several teams share and consolidates duplicated pipelines into shared infrastructure. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>Depth: decides company-level grounding bets - proprietary-data moats, retrieval vs. long-context vs. fine-tuning - and owns that thesis with executives. Scope: company.</t>
+          <t>Depth: Deep expertise; anticipates how longer context and new architectures change retrieval economics. Evidenced by: Sets the org's knowledge-grounding strategy — what corpora exist, who owns them, entitlement-aware access, and quality accountability. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Mastery of the discipline; defines how AI systems access knowledge. Evidenced by: Decides company-level grounding bets — proprietary-data moats, retrieval vs. long-context vs. fine-tuning — and owns that thesis with executives. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1419,37 +1480,42 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Reimers &amp; Gurevych, "Sentence-BERT" (EMNLP 2019)</t>
+          <t>Grounds models in the right knowledge.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Depth: generates and stores embeddings using the team's pipeline and explains what an embedding represents in plain language. Scope: embedding tasks within a pipeline.</t>
+          <t>Johnson, Douze &amp; Jegou, Billion-Scale Similarity Search with GPUs, IEEE Transactions on Big Data (2019) — Reimers &amp; Gurevych's Sentence-BERT paper has no bibliography entry; Johnson, Douze &amp; Jegou's FAISS paper is the catalog-adjacent source behind AI-02's own P4 similarity-search-at-scale text, and embedding choices silently cap retrieval quality unless treated as tunable, evaluable components.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Depth: evaluates embedding models against the team's retrieval benchmarks and tunes similarity thresholds and index parameters with evidence. Scope: the embedding layer of a component.</t>
+          <t>Depth: Understands embeddings, similarity search and why grounding reduces hallucination. Evidenced by: Generates and stores embeddings using the team's pipeline and explains what an embedding represents in plain language. Scope: task.</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Depth: selects embedding models, dimensions, and index types by measured trade-off for a capability, and designs re-embedding and migration plans when models change. Scope: a capability's semantic-search layer.</t>
+          <t>Depth: Builds standard RAG pipelines (chunking, embedding, retrieval, reranking); manages context budgets deliberately. Evidenced by: Evaluates embedding models against the team's retrieval benchmarks and tunes similarity thresholds and index parameters with evidence. Scope: component.</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Depth: standardizes embedding infrastructure across teams - shared models, versioning, migration tooling - ending per-team drift. Scope: multiple teams.</t>
+          <t>Depth: Designs retrieval quality systems (hybrid search, reranking, freshness, citation, memory for multi-turn). Evidenced by: Selects embedding models, dimensions, and index types by measured trade-off for a capability and designs re-embedding and migration plans when models change. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Depth: drives the org's vector-infrastructure strategy, including build-vs-buy for vector stores and cost and scale planning. Scope: organization.</t>
+          <t>Depth: Expert in retrieval at scale (index strategy, multi-source federation, permission-aware retrieval). Evidenced by: Standardizes embedding infrastructure across teams — shared models, versioning, migration tooling — ending per-team drift. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Depth: anticipates representation-layer shifts - multimodal embeddings, new architectures - and positions the company ahead of them. Scope: company.</t>
+          <t>Depth: Deep expertise; anticipates how longer context and new architectures change retrieval economics. Evidenced by: Drives the org's vector-infrastructure strategy, including build-vs-buy for vector stores and cost and scale planning. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Mastery of the discipline; defines how AI systems access knowledge. Evidenced by: Anticipates representation-layer shifts — multimodal embeddings, new architectures — and positions the company ahead of them. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1476,37 +1542,42 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Liu et al., "Lost in the Middle: How Language Models Use Long Contexts" (TACL 2024)</t>
+          <t>Grounds models in the right knowledge.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Depth: keeps requests within the context budget, truncating per team rules, and notices when overflow or truncation silently degrades output. Scope: a task's context usage.</t>
+          <t>Gao et al., Retrieval-Augmented Generation for Large Language Models: A Survey (2023) — Liu et al.'s "Lost in the Middle" paper has no bibliography entry; Gao et al.'s RAG survey is the broadest catalog-adjacent source covering context and retrieval engineering together (it grounds AI-02's own P3/P5 text), and context windows are a scarce, position-sensitive resource that what enters, where, and what gets summarized away determines behavior.</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Depth: prioritizes what enters the window - system prompt, history, retrieved content - with explicit truncation rules, and tests the effect of dropping each element. Scope: a component's context assembly.</t>
+          <t>Depth: Understands embeddings, similarity search and why grounding reduces hallucination. Evidenced by: Keeps requests within the context budget, truncating per team rules, and notices when overflow or truncation silently degrades output. Scope: task.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Depth: designs the context-assembly strategy for a capability - token budgets per section, summarization versus omission, memory for long sessions, cache-friendly ordering - and shows with evals where added context stops paying. Scope: a capability; others reuse the assembly design.</t>
+          <t>Depth: Builds standard RAG pipelines (chunking, embedding, retrieval, reranking); manages context budgets deliberately. Evidenced by: Prioritizes what enters the window with explicit truncation rules and tests the effect of dropping each element. Scope: component.</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Depth: defines context-management patterns multiple teams reuse - shared memory stores, summarizers, compaction strategies - and audits high-cost windows for waste. Scope: multiple teams.</t>
+          <t>Depth: Designs retrieval quality systems (hybrid search, reranking, freshness, citation, memory for multi-turn). Evidenced by: Designs the context-assembly strategy for a capability and shows with evals where added context stops paying. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Depth: drives org-level context and memory architecture, deciding what user and org state is durable memory versus per-request context, with token-quality trade-offs measured at fleet level. Scope: organization.</t>
+          <t>Depth: Expert in retrieval at scale (index strategy, multi-source federation, permission-aware retrieval). Evidenced by: Defines context-management patterns multiple teams reuse and audits high-cost windows for waste. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>Depth: positions the company for context-regime shifts - window growth, pricing changes, memory architectures - before they invalidate current designs. Scope: company.</t>
+          <t>Depth: Deep expertise; anticipates how longer context and new architectures change retrieval economics. Evidenced by: Drives org-level context and memory architecture, deciding what user and org state is durable memory versus per-request context. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Mastery of the discipline; defines how AI systems access knowledge. Evidenced by: Positions the company for context-regime shifts before they invalidate current designs. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1533,37 +1604,42 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Anthropic, "Building Effective Agents" (2024)</t>
+          <t>Designs systems where models plan and act through tools.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Depth: traces an existing agent loop end to end - model call, tool call, state update - explaining why the agent took each step on a real transcript, and fixes defects in single steps. Scope: a task within an agent.</t>
+          <t>Yao et al., ReAct: Synergizing Reasoning and Acting in Language Models, ICLR 2023 — Anthropic's "Building Effective Agents" blog post has no bibliography entry; Yao et al.'s ReAct paper is where the plan-act-observe loop AI-03's own P1/P2 text names was formalized, and the central agentic decision is workflow vs. autonomous loop — over-agentifying is the field's dominant failure mode.</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Depth: builds single-agent workflows with a bounded tool set using the simplest pattern that works - chain, router, or loop - with explicit termination conditions and step limits by default. Scope: a component.</t>
+          <t>Depth: Understands tool calling and the agent loop (plan, act, observe); knows why agents need constraints. Evidenced by: Traces an existing agent loop end to end, explaining why the agent took each step on a real transcript, and fixes defects in single steps. Scope: task.</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Depth: chooses between workflow and autonomous-loop designs by failure-mode analysis, decomposing multi-step behavior so each step is independently observable and recoverable, and cuts autonomy when a simpler pipeline scores the same. Scope: owns agent architecture for a capability.</t>
+          <t>Depth: Designs good tool interfaces; builds single-agent workflows with sensible termination and confirmation points. Evidenced by: Builds single-agent workflows with a bounded tool set using the simplest pattern that works, with explicit termination conditions and step limits by default. Scope: component.</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets the agent-architecture patterns multiple teams follow - orchestration substrate, state and handoff conventions, delegation contracts - and kills over-engineered designs with evidence. Scope: multiple teams.</t>
+          <t>Depth: Designs reliable multi-step agents (state, recovery, sandboxing, permissions, human-in-the-loop); knows when an agent is the wrong answer. Evidenced by: Chooses between workflow and autonomous-loop designs by failure-mode analysis and cuts autonomy when a simpler pipeline scores the same. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the org's agentic-systems strategy, deciding where autonomy is worth its reliability cost and what the shared platform provides. Scope: organization.</t>
+          <t>Depth: Expert in complex orchestration (multi-agent, long-running workflows, MCP-style standards) and safe constraint at scale. Evidenced by: Sets the agent-architecture patterns multiple teams follow and kills over-engineered designs with evidence. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets company direction on agentic products - where agents act, where humans decide - informed by what current models can actually sustain. Scope: company.</t>
+          <t>Depth: Deep expertise; anticipates how increasing model autonomy changes system design. Evidenced by: Owns the org's agentic-systems strategy, deciding where autonomy is worth its reliability cost and what the shared platform provides. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Authority on agentic systems; may influence emerging industry standards. Evidenced by: Sets company direction on agentic products — where agents act, where humans decide — informed by what current models can actually sustain. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1590,37 +1666,42 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Anthropic, "Writing Effective Tools for Agents" (2025)</t>
+          <t>Designs systems where models plan and act through tools.</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Depth: implements a tool to a given schema with validation and error strings a model can act on, and tests it standalone before wiring it to a model. Scope: single tools within a task.</t>
+          <t>Anthropic, Model Context Protocol Specification (2025-11-25) — Anthropic's "Writing Effective Tools for Agents" post has no bibliography entry; Anthropic's own Model Context Protocol Specification is the catalog-adjacent source AI-03's own P4/P6 text cites for MCP-style tool standards, and agents fail at the tool boundary more than anywhere else — tool design is interface design for a non-human caller.</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Depth: designs tool schemas a model uses correctly on the first try - clear descriptions, tight parameters, informative error returns - and iterates on them against transcripts of real misuse. Scope: a component's tool set.</t>
+          <t>Depth: Understands tool calling and the agent loop (plan, act, observe); knows why agents need constraints. Evidenced by: Implements a tool to a given schema with validation and error strings a model can act on, and tests it standalone before wiring it to a model. Scope: task.</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Depth: curates the tool surface of a capability - right granularity, idempotency and side-effect discipline, permission boundaries - pruning overlapping tools that confuse routing and rewriting descriptions from observed call failures. Scope: a capability's tool ecosystem.</t>
+          <t>Depth: Designs good tool interfaces; builds single-agent workflows with sensible termination and confirmation points. Evidenced by: Designs tool schemas a model uses correctly on the first try and iterates on them against transcripts of real misuse. Scope: component.</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Depth: defines tool-design standards and shared registries multiple teams consume, with review gates for high-risk tools, killing near-duplicate tools across agents. Scope: multiple teams.</t>
+          <t>Depth: Designs reliable multi-step agents (state, recovery, sandboxing, permissions, human-in-the-loop); knows when an agent is the wrong answer. Evidenced by: Curates the tool surface of a capability — right granularity, idempotency and side-effect discipline, permission boundaries — pruning overlapping tools that confuse routing. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Depth: drives the org's tool and integration platform - registries, permissioning, audit requirements - deciding which internal systems get first-class tool interfaces. Scope: organization.</t>
+          <t>Depth: Expert in complex orchestration (multi-agent, long-running workflows, MCP-style standards) and safe constraint at scale. Evidenced by: Defines tool-design standards and shared registries multiple teams consume, with review gates for high-risk tools, killing near-duplicate tools across agents. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>Depth: shapes the company's external tool ecosystem posture - what third parties may plug in, what the company exposes - as a durable interface bet. Scope: company and partners.</t>
+          <t>Depth: Deep expertise; anticipates how increasing model autonomy changes system design. Evidenced by: Drives the org's tool and integration platform, deciding which internal systems get first-class tool interfaces. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Authority on agentic systems; may influence emerging industry standards. Evidenced by: Shapes the company's external tool ecosystem posture — what third parties may plug in, what the company exposes — as a durable interface bet. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1647,37 +1728,42 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>NIST AI Risk Management Framework 1.0 (2023)</t>
+          <t>Keeps AI behavior safe, honest and within bounds.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Depth: implements the approval and confirmation steps a design specifies - never bypassing a human checkpoint without sign-off - and states which of their feature's actions are reversible and which are not. Scope: a task's approval points.</t>
+          <t>NIST, Artificial Intelligence Risk Management Framework (AI RMF 1.0), NIST AI 100-1 (2023) — NIST's AI Risk Management Framework 1.0 is a real, exact bibliography match for the original citation: human oversight proportional to impact and reversibility is a designed control under NIST's GOVERN/MAP/MANAGE functions, not an afterthought.</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Depth: designs approval gates by reversibility and blast radius - auto-run the undoable, confirm the destructive - with dry-run modes, undo paths, and every escalation logged for audit. Scope: a component's autonomy rules.</t>
+          <t>Depth: Understands that models can be harmful, biased or confidently wrong; flags concerning behavior. Evidenced by: Implements the approval and confirmation steps a design specifies — never bypassing a human checkpoint without sign-off — and states which of their feature's actions are reversible. Scope: task.</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Depth: calibrates autonomy per action class for a capability - auto-execute, confirm, or escalate - from observed override and failure data rather than assumption, and pushes back with reasons when a design grants an agent more authority than its error rate supports. Scope: a capability's operating envelope.</t>
+          <t>Depth: Implements guardrails (filtering, refusal handling, grounding checks); designs honest UX. Evidenced by: Designs approval gates by reversibility and blast radius, with dry-run modes, undo paths, and every escalation logged for audit. Scope: component.</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Depth: standardizes autonomy tiers and approval mechanisms across teams, with shared approval UX and audit infrastructure, and reviews escalation designs for high-consequence actions. Scope: multiple teams.</t>
+          <t>Depth: Designs layered safety proportional to stakes; evaluates for bias/misuse before launch. Evidenced by: Calibrates autonomy per action class for a capability from observed override and failure data, and pushes back when a design grants an agent more authority than its error rate supports. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the org's policy for delegated agent authority, aligned with legal and security, including the evidence bar for widening autonomy. Scope: organization.</t>
+          <t>Depth: Expert in safety system design at scale; defines oversight and escalation frameworks. Evidenced by: Standardizes autonomy tiers and approval mechanisms across teams and reviews escalation designs for high-consequence actions. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>Depth: decides how much authority the company delegates to AI systems in its products and operations, and defends that line to regulators and customers. Scope: company.</t>
+          <t>Depth: Deep expertise balancing capability and safety under real product pressure. Evidenced by: Owns the org's policy for delegated agent authority, aligned with legal and security, including the evidence bar for widening autonomy. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Recognized authority; establishes responsible AI as a value; externally credible. Evidenced by: Decides how much authority the company delegates to AI systems in its products and operations and defends that line to regulators and customers. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1704,37 +1790,42 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Kapoor et al., "AI Agents That Matter" (2024)</t>
+          <t>Applies idempotency, retries, deduplication, and delivery guarantees to make operations safely repeatable.</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Depth: reproduces a failed agent run from its transcript and identifies the step where it went wrong - bad plan, bad tool result, lost state. Scope: task-level debugging.</t>
+          <t>Helland, Idempotence Is Not a Medical Condition, ACM Queue 10(4) (2012) — Kapoor et al.'s "AI Agents That Matter" has no bibliography entry; Helland's "Idempotence Is Not a Medical Condition" is BE-11's own catalog anchor at every level and states the exact engineering property — safely repeatable operations — that multi-step agents need once per-step error compounds across a run.</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Depth: builds checkpointing, retries, loop limits, and budget caps into agent steps so a wandering run halts cheaply and an interrupted run resumes or fails cleanly instead of duplicating side effects. Scope: a component's run lifecycle.</t>
+          <t>Depth: Applies provided idempotency and retry patterns for simple cases under review. Evidenced by: Reproduces a failed agent run from its transcript and identifies the step where it went wrong — bad plan, bad tool result, lost state. Scope: task.</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Depth: designs the state and containment model for an agentic capability - what persists across turns, blast-radius limits, compensating actions for tool side effects - quantifying compounded failure rates rather than trusting per-step accuracy, and proves recovery paths with fault injection. Scope: a capability's execution engine.</t>
+          <t>Depth: Implements standard reliability and retry handling independently. Evidenced by: Builds checkpointing, retries, loop limits, and budget caps into agent steps so a wandering run halts cheaply and an interrupted run resumes or fails cleanly. Scope: component.</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets durable-execution and recovery patterns multiple teams adopt - resumable run state, saga-style compensation - with adoption they can show. Scope: multiple teams' agent runtimes.</t>
+          <t>Depth: Designs idempotent, reliable flows autonomously; resolves duplicate and partial-failure cases. Evidenced by: Designs the state and containment model for an agentic capability, quantifying compounded failure rates rather than trusting per-step accuracy, and proves recovery paths with fault injection. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>Depth: drives the org's strategy for stateful, long-running AI execution, consolidating bespoke run-state code into platform, with reliability targets and failure drills. Scope: organization.</t>
+          <t>Depth: Defines reliability patterns teams adopt; solves the hardest exactly-once and recovery problems. Evidenced by: Sets durable-execution and recovery patterns multiple teams adopt — resumable run state, saga-style compensation — with adoption they can show. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets company reliability doctrine for autonomous systems, informing what the company will and won't promise customers. Scope: company.</t>
+          <t>Depth: Sets reliability and idempotency strategy across systems; anticipates evolving failure modes. Evidenced by: Drives the org's strategy for stateful, long-running AI execution, consolidating bespoke run-state code into platform, with reliability targets and failure drills. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines best practice for reliability patterns industrywide; shapes widely adopted approaches. Evidenced by: Sets company reliability doctrine for autonomous systems, informing what the company will and won't promise customers. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1761,37 +1852,42 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Nygard, *Release It!* (2nd ed., 2018), bulkheads</t>
+          <t>Designs systems where models plan and act through tools.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Depth: runs agents in the sandboxed environment provided and reports containment gaps they notice. Scope: their own agent runs.</t>
+          <t>Nygard, Release It!: Design and Deploy Production-Ready Software, 2nd Edition (Pragmatic Bookshelf, 2018) — An agent with tools is a failure amplifier; Nygard's Release It! bulkhead pattern is the exact containment discipline this competency instantiates for the agentic case, and containment must be engineered before autonomy is granted.</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Depth: scopes an agent's credentials and tool permissions to least privilege, and caps loops, spend, and side effects by construction. Scope: one agent's blast radius.</t>
+          <t>Depth: Understands tool calling and the agent loop (plan, act, observe); knows why agents need constraints. Evidenced by: Runs agents in the sandboxed environment provided and reports containment gaps they notice. Scope: task.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Depth: designs containment for a capability's agents - sandboxing, budget kill-switches, reversible-by-default actions - and red-teams their own boundaries before launch. Scope: a capability; their containment review gates agent launches.</t>
+          <t>Depth: Designs good tool interfaces; builds single-agent workflows with sensible termination and confirmation points. Evidenced by: Scopes an agent's credentials and tool permissions to least privilege, and caps loops, spend, and side effects by construction. Scope: component.</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Depth: builds containment infrastructure several teams inherit rather than reimplement, and audits exceptions. Scope: multiple teams.</t>
+          <t>Depth: Designs reliable multi-step agents (state, recovery, sandboxing, permissions, human-in-the-loop); knows when an agent is the wrong answer. Evidenced by: Designs containment for a capability's agents — sandboxing, budget kill-switches, reversible-by-default actions — and red-teams their own boundaries before launch. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets the org's containment standards for autonomous systems and verifies them through game days. Scope: organization.</t>
+          <t>Depth: Expert in complex orchestration (multi-agent, long-running workflows, MCP-style standards) and safe constraint at scale. Evidenced by: Builds containment infrastructure several teams inherit rather than reimplement, and audits exceptions. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the company's worst-case analysis for agentic products and the controls that bound it. Scope: company.</t>
+          <t>Depth: Deep expertise; anticipates how increasing model autonomy changes system design. Evidenced by: Sets the org's containment standards for autonomous systems and verifies them through game days. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Authority on agentic systems; may influence emerging industry standards. Evidenced by: Owns the company's worst-case analysis for agentic products and the controls that bound it. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1818,37 +1914,42 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Husain, "Your AI Product Needs Evals" (2024)</t>
+          <t>Assembles, labels, and curates representative datasets suitable for model training.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Depth: adds well-formed cases to an existing eval set - realistic input, unambiguous expected behavior - labeling edge cases consistently with the rubric and flagging ambiguous ones instead of guessing. Scope: eval cases for their task.</t>
+          <t>Sambasivan et al., "Everyone wants to do the model work, not the data work": Data Cascades in High-Stakes AI, CHI 2021 — Husain's "Your AI Product Needs Evals" article has no bibliography entry; Sambasivan et al.'s Data Cascades paper is AI-07's own catalog anchor and is the empirical case for why eval sets built by disciplined error analysis on real traces are the only ones that measure anything — sloppy data work cascades into every downstream quality claim.</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Depth: builds an eval set for a feature from production traces via error analysis, balancing common paths and hard cases, versioning golden data like code with documented inclusion criteria. Scope: a component's eval coverage.</t>
+          <t>Depth: Labels data to clear guidelines and flags ambiguities under review. Evidenced by: Adds well-formed cases to an existing eval set, labeling edge cases consistently with the rubric and flagging ambiguous ones instead of guessing. Scope: task.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the golden datasets of a capability - coverage mapped to known failure modes, refresh cadence, contamination and leakage checks - retiring stale cases and tracing every regression escape back to the missing case class. Scope: a capability; their sets gate teammates' merges.</t>
+          <t>Depth: Curates and labels routine datasets independently, applying consistent guidelines. Evidenced by: Builds an eval set for a feature from production traces via error analysis, versioning golden data like code with documented inclusion criteria. Scope: component.</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets eval-data standards multiple teams follow - sampling policy, labeling rubrics, inter-rater checks, dataset versioning - and audits suites whose numbers look too good. Scope: multiple teams.</t>
+          <t>Depth: Designs labeling schemes and resolves ambiguity and quality issues autonomously. Evidenced by: Owns the golden datasets of a capability, retiring stale cases and tracing every regression escape back to the missing case class. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Depth: drives the org's evaluation-data strategy - shared corpora, labeling operations, data governance for eval assets. Scope: organization.</t>
+          <t>Depth: Defines curation and annotation-quality standards others adopt. Evidenced by: Sets eval-data standards multiple teams follow and audits suites whose numbers look too good. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>Depth: defines how the company knows its AI works - the evidence doctrine cited in launch reviews and external claims. Scope: company.</t>
+          <t>Depth: Sets dataset strategy and anticipates shifts in labeling and curation practice. Evidenced by: Drives the org's evaluation-data strategy — shared corpora, labeling operations, data governance for eval assets. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines industry best practice for dataset curation and is externally credible. Evidenced by: Defines how the company knows its AI works — the evidence doctrine cited in launch reviews and external claims. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1875,37 +1976,42 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Zheng et al., "Judging LLM-as-a-Judge with MT-Bench and Chatbot Arena" (NeurIPS 2023); Shankar et al., "Who Validates the Validators?" (2024)</t>
+          <t>Proves AI behavior is good enough to ship.</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Depth: runs the eval harness and reads its reports correctly, distinguishing a real regression from noise with help and flagging results that look wrong instead of accepting them. Scope: their changes.</t>
+          <t>Zheng et al., Judging LLM-as-a-Judge with MT-Bench and Chatbot Arena, NeurIPS 2023 — Shankar et al.'s "Who Validates the Validators?" has no bibliography entry; Zheng et al.'s MT-Bench/Chatbot Arena paper is the exact bibliography match for the paired original citation and is AI-04's own P3/P5 anchor — judges are fallible instruments, and an unvalidated judge automates the wrong opinion at scale.</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Depth: chooses graders that fit the behavior under test - exact-match, rubric, pairwise, LLM-judge - and spot-checks judge agreement against their own labels before trusting it. Scope: a component's metrics.</t>
+          <t>Depth: Understands why 'it looked right in testing' is insufficient; runs existing evals and labels carefully. Evidenced by: Runs the eval harness and reads its reports correctly, distinguishing a real regression from noise with help and flagging results that look wrong instead of accepting them. Scope: task.</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Depth: designs the measurement itself for a capability - metrics that track user outcomes, judges validated against human ratings with quantified agreement and bias, significance limits stated before declaring a win. Scope: a capability; measure-before-ship is their default others copy.</t>
+          <t>Depth: Builds basic eval sets from real usage; measures changes before shipping prompt/model updates. Evidenced by: Chooses graders that fit the behavior under test and spot-checks judge agreement against their own labels before trusting it. Scope: component.</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Depth: standardizes eval methodology across teams, calibrating judge models centrally so scores are comparable, and arbitrates when two teams' numbers disagree about the same behavior. Scope: multiple teams.</t>
+          <t>Depth: Designs eval methodology (golden sets, LLM-as-judge with validation, human review, helpfulness/groundedness/safety metrics). Evidenced by: Designs the measurement itself for a capability — judges validated against human ratings with quantified agreement and bias, significance limits stated before declaring a win. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the org's measurement strategy for AI quality, connecting offline evals to online outcomes and killing metrics that don't predict. Scope: organization.</t>
+          <t>Depth: Expert in eval at scale (continuous eval, A/B testing AI features, drift detection). Evidenced by: Standardizes eval methodology across teams, calibrating judge models centrally so scores are comparable. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>Depth: defines what 'good' means for the company's AI products in measurable terms executives, customers, and regulators accept. Scope: company.</t>
+          <t>Depth: Deep expertise in measuring AI quality where ground truth is contested. Evidenced by: Owns the org's measurement strategy for AI quality, connecting offline evals to online outcomes and killing metrics that don't predict. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Mastery of the discipline; sets the bar for what 'proven to work' means. Evidenced by: Defines what 'good' means for the company's AI products in measurable terms executives, customers, and regulators accept. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1932,37 +2038,42 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Sculley et al., "Hidden Technical Debt in Machine Learning Systems" (NeurIPS 2015)</t>
+          <t>Integrating automated quality gates into build and deployment pipelines for fast feedback.</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Depth: runs the required evals before merging prompt or model changes and pastes results into the review, flagging regressions instead of explaining them away. Scope: their own changes.</t>
+          <t>Sculley et al., Hidden Technical Debt in Machine Learning Systems, NeurIPS 2015 — Sculley et al.'s Hidden Technical Debt paper is an exact bibliography match: unmeasured behavioral change is the dominant debt in model-backed systems, so ship decisions must rest on measured deltas, not demos.</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Depth: attaches eval deltas to every prompt, model, or retrieval change and blocks their own launches on regressions - shadow or A/B comparisons for risky changes - without being told. Scope: a component's releases.</t>
+          <t>Depth: Adds tests to existing pipeline stages following defined configuration, reviewed before merge. Evidenced by: Runs the required evals before merging prompt or model changes and pastes results into the review, flagging regressions instead of explaining them away. Scope: task.</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Depth: defines the ship gate for a capability - which evals block release, what regression tolerance is, when human review is required - and holds the line under deadline pressure with the reasoning in writing. Scope: a capability's ship decisions.</t>
+          <t>Depth: Integrates and maintains automated test stages independently within standard pipelines. Evidenced by: Attaches eval deltas to every prompt, model, or retrieval change and blocks their own launches on regressions without being told. Scope: component.</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Depth: installs measurement-gated release processes across teams - eval CI, canary analysis, staged rollouts teams actually use - and audits exceptions. Scope: multiple teams' pipelines.</t>
+          <t>Depth: Designs fast, reliable test gating for complex pipelines balancing speed and confidence. Evidenced by: Defines the ship gate for a capability — which evals block release, what regression tolerance is, when human review is required — and holds the line under deadline pressure with the reasoning in writing. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the org's ship/no-ship framework for AI behavior changes and arbitrates escalations where speed and evidence conflict. Scope: organization.</t>
+          <t>Depth: Defines continuous-testing patterns and gating strategy other teams adopt. Evidenced by: Installs measurement-gated release processes across teams — eval CI, canary analysis, staged rollouts teams actually use — and audits exceptions. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets company policy on the evidence required to ship AI behavior, balancing speed and risk explicitly. Scope: company.</t>
+          <t>Depth: Sets continuous-testing strategy and anticipates how quality gates must evolve with delivery. Evidenced by: Owns the org's ship/no-ship framework for AI behavior changes and arbitrates escalations where speed and evidence conflict. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines authoritative continuous-testing practice that shapes the discipline. Evidenced by: Sets company policy on the evidence required to ship AI behavior, balancing speed and risk explicitly. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1989,37 +2100,42 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>OpenTelemetry Generative AI semantic conventions (CNCF, 2024-2025)</t>
+          <t>Makes system behavior visible.</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Depth: uses existing traces to debug a failing request - walking prompt -&gt; retrieval -&gt; tool call -&gt; output - and adds a missing span when told what to capture. Scope: their tasks.</t>
+          <t>Sridharan, Distributed Systems Observability: A Guide to Building Robust Systems (O'Reilly, 2018) — The OpenTelemetry GenAI semantic conventions have no bibliography entry; Sridharan's Distributed Systems Observability is OPS-05's own catalog anchor at P1-P4, and nondeterministic multi-step systems cannot be debugged from logs alone — traces are the unit of truth.</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Depth: instruments a component end to end - prompts, completions, token counts, tool calls, latencies - as structured spans with the metadata (prompt version, model id) needed to reproduce any output later, with sampling and redaction applied correctly. Scope: a component's telemetry.</t>
+          <t>Depth: Understands logs/metrics/traces; reads existing dashboards. Evidenced by: Uses existing traces to debug a failing request — walking prompt to retrieval to tool call to output — and adds a missing span when told what to capture. Scope: task.</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Depth: designs the observability schema for a capability - what is captured, sampled, retained, and redacted - and builds the views that make failure clusters visible, answering 'why did this output happen' in minutes. Scope: a capability; their traces are where debugging starts.</t>
+          <t>Depth: Instruments their services; builds dashboards; tunes alerts to limit noise. Evidenced by: Instruments a component end to end as structured spans with the metadata needed to reproduce any output later, with sampling and redaction applied correctly. Scope: component.</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets tracing conventions multiple teams emit, aligning attributes so cross-service AI requests join up in one lens, and builds the views on-call engineers actually use. Scope: multiple teams.</t>
+          <t>Depth: Designs observability for complex systems (end-to-end traces, quality signals, cost attribution). Evidenced by: Designs the observability schema for a capability and builds the views that make failure clusters visible, answering 'why did this output happen' in minutes. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the org's AI observability platform strategy, including retention, privacy, and cost of trace data. Scope: organization.</t>
+          <t>Depth: Expert in instrumentation trade-offs at scale, incl. privacy-safe logging. Evidenced by: Sets tracing conventions multiple teams emit, aligning attributes so cross-service AI requests join up in one lens. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>Depth: ensures the company can answer 'why did the model do that?' for any production decision, as a matter of architecture. Scope: company.</t>
+          <t>Depth: Defines org observability strategy. Evidenced by: Owns the org's AI observability platform strategy, including retention, privacy, and cost of trace data. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes company-wide operational visibility; advances practice. Evidenced by: Ensures the company can answer 'why did the model do that?' for any production decision, as a matter of architecture. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2046,37 +2162,42 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Breck et al., "The ML Test Score" (2017)</t>
+          <t>Tracks live model quality and data drift to trigger retraining or rollback.</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Depth: watches the dashboards for their feature after deploys and escalates anomalies with the trace attached rather than assuming success. Scope: post-ship checks on their tasks.</t>
+          <t>Gama et al., A Survey on Concept Drift Adaptation, ACM Computing Surveys 46(4) (2014) — Breck et al.'s "The ML Test Score" has no bibliography entry; Gama et al.'s concept-drift survey is AI-17's own catalog anchor at every level, and model-backed quality decays silently as inputs, usage, and providers change, so monitoring must watch behavior, not just uptime.</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Depth: builds behavioral monitors for a component - refusal rate, format-break rate, user-feedback signals - with alert thresholds they can justify, promoting recurring failures into the eval set. Scope: a component's monitors.</t>
+          <t>Depth: Watches configured monitors and reports alerts under guidance. Evidenced by: Watches the dashboards for their feature after deploys and escalates anomalies with the trace attached rather than assuming success. Scope: task.</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Depth: detects silent degradation for a capability - baselines behavior, catches provider-side model changes and input-distribution drift, reruns evals on live samples on a schedule - and has caught a real regression no user reported. Scope: a capability in production.</t>
+          <t>Depth: Sets up standard performance and drift monitoring independently. Evidenced by: Builds behavioral monitors for a component with alert thresholds they can justify, promoting recurring failures into the eval set. Scope: component.</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Depth: standardizes behavioral monitoring and feedback-to-eval pipelines across teams, with shared metric definitions so numbers are comparable, correlating cross-product regressions to a common upstream cause. Scope: multiple teams.</t>
+          <t>Depth: Designs monitoring that catches subtle drift and degradation autonomously and triages causes. Evidenced by: Detects silent degradation for a capability — baselines behavior, catches provider-side model changes and input-distribution drift — and has caught a real regression no user reported. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the org's in-production AI quality picture, making drift review a routine practice with owners and SLAs, briefing leadership on trends rather than incidents. Scope: organization.</t>
+          <t>Depth: Defines monitoring and drift-detection patterns others adopt. Evidenced by: Standardizes behavioral monitoring and feedback-to-eval pipelines across teams, correlating cross-product regressions to a common upstream cause. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>Depth: makes behavioral health a company-level operational metric, reported alongside availability, defining how the company absorbs provider upgrades without quality surprises. Scope: company.</t>
+          <t>Depth: Sets monitoring strategy and anticipates advances in drift detection. Evidenced by: Owns the org's in-production AI quality picture, making drift review a routine practice with owners and SLAs. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines best practice for model monitoring and is externally credible. Evidenced by: Makes behavioral health a company-level operational metric, defining how the company absorbs provider upgrades without quality surprises. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2103,37 +2224,42 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Nygard, *Release It!* (2nd ed., 2018)</t>
+          <t>Keeps services healthy; designs for failure.</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Depth: implements the retry, timeout, and fallback behavior a design specifies and tests the failure path by forcing the failure, not just the happy path. Scope: their tasks.</t>
+          <t>Nygard, Release It!: Design and Deploy Production-Ready Software, 2nd Edition (Pragmatic Bookshelf, 2018) — Nygard's Release It! (2nd ed.) is an exact bibliography match: provider outages, rate limits, and malformed outputs are routine, and stability patterns are the designed defense OPS-04's own P2 text ("builds retries, timeouts and fallbacks") cites this book for directly.</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Depth: designs the degradation ladder for a component - retry budgets, circuit breaking on provider errors, cached or smaller-model fallbacks, an honest error - and makes each rung observable. Scope: a component's failure behavior.</t>
+          <t>Depth: Understands SLOs and common failure modes; keeps components healthy with guidance. Evidenced by: Implements the retry, timeout, and fallback behavior a design specifies and tests the failure path by forcing the failure, not just the happy path. Scope: task.</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns availability design for a capability across providers - failover routing, brownout modes, load shedding - with explicit SLOs that include behavioral quality, validated with game days rather than hope. Scope: a capability's reliability.</t>
+          <t>Depth: Builds retries, timeouts and fallbacks; understands blast radius. Evidenced by: Designs the degradation ladder for a component — retry budgets, circuit breaking on provider errors, cached or smaller-model fallbacks — and makes each rung observable. Scope: component.</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Depth: builds the shared resilience layer multiple teams depend on - gateway, routing, quota management - and reviews launches for shared-fate provider risk. Scope: multiple teams.</t>
+          <t>Depth: Designs for graceful degradation; defines SLOs; accountable for a domain's reliability. Evidenced by: Owns availability design for a capability across providers — failover routing, brownout modes, load shedding — validated with game days rather than hope. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns org-level continuity for provider failure - multi-provider posture, capacity reservations, tested playbooks. Scope: organization.</t>
+          <t>Depth: Expert in resilience and capacity planning at scale; drives down incidents systemically. Evidenced by: Builds the shared resilience layer multiple teams depend on and reviews launches for shared-fate provider risk. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>Depth: answers for company availability of AI products through provider incidents that make the news, setting the architecture doctrine behind the commitments. Scope: company.</t>
+          <t>Depth: Owns org-level reliability; fixes risk in process and org design. Evidenced by: Owns org-level continuity for provider failure — multi-provider posture, capacity reservations, tested playbooks. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Sets the company's reliability philosophy. Evidenced by: Answers for company availability of AI products through provider incidents that make the news, setting the architecture doctrine behind the commitments. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2160,37 +2286,42 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Beyer et al., *Site Reliability Engineering* (2016)</t>
+          <t>Responds to and learns from production incidents.</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Depth: follows the runbook during incidents, keeps the timeline updated, captures the traces responders need, and asks for help early. Scope: a participant in the response.</t>
+          <t>Beyer, Jones, Petoff &amp; Murphy (eds.), Site Reliability Engineering: How Google Runs Production Systems (O'Reilly/Google, 2016) — Beyer et al.'s Site Reliability Engineering is an exact bibliography match and OPS-06's own catalog anchor: AI incidents add novel failure classes — quality collapse, runaway cost, harmful output — to classic outage response.</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Depth: debugs live model-system incidents independently - distinguishing provider outage from prompt regression from data problem - and writes the postmortem with concrete actions. Scope: a component's on-call.</t>
+          <t>Depth: Responds to alerts with support; follows runbooks; escalates appropriately. Evidenced by: Follows the runbook during incidents, keeps the timeline updated, captures the traces responders need, and asks for help early. Scope: task.</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Depth: incident-commands for their capability, including quality and cost incidents that page no one by default; writes the runbooks for model rollback and prompt reversion others copy, and drives postmortems to systemic fixes. Scope: a capability's incident response.</t>
+          <t>Depth: Triages and resolves routine incidents; clear notes; takes on-call. Evidenced by: Debugs live model-system incidents independently — distinguishing provider outage from prompt regression from data problem — and writes the postmortem with concrete actions. Scope: component.</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Depth: raises operational maturity across teams - severity definitions that include model-quality events, game days for AI failure classes, readiness reviews before launches. Scope: multiple teams.</t>
+          <t>Depth: Leads response to complex failures; blameless postmortems; same failure never recurs. Evidenced by: Incident-commands for their capability, including quality and cost incidents that page no one by default, and drives postmortems to systemic fixes. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the org's incident-management standard for AI systems, reviewing the postmortems that cross team boundaries and closing systemic gaps. Scope: organization.</t>
+          <t>Depth: Expert in incident-management design (rotations, severity, escalation). Evidenced by: Raises operational maturity across teams — severity definitions that include model-quality events, game days for AI failure classes, readiness reviews before launches. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>Depth: is the company's senior technical responder in its worst AI incidents and changes company practice from what they reveal. Scope: company.</t>
+          <t>Depth: Commands the highest-severity incidents; sets incident process org-wide. Evidenced by: Owns the org's incident-management standard for AI systems, reviewing the postmortems that cross team boundaries and closing systemic gaps. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Sets the company's incident philosophy; calm authority in the worst moments. Evidenced by: Is the company's senior technical responder in its worst AI incidents and changes company practice from what they reveal. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2217,37 +2348,42 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Beyer et al., *Site Reliability Engineering* (2016), capacity planning</t>
+          <t>Forecasts demand and provisions compute, storage, and connection resources against budgets.</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Depth: monitors quota and rate-limit dashboards for their service and escalates approaching limits before they bite. Scope: awareness within a task.</t>
+          <t>Beyer, Jones, Petoff &amp; Murphy (eds.), Site Reliability Engineering: How Google Runs Production Systems (O'Reilly/Google, 2016) — A model provider is a tier-0 dependency the team doesn't operate; Beyer et al.'s SRE capacity-planning chapter, BE-19's own catalog anchor at every level, is where quota, deprecations and capacity being engineered around originates.</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Depth: implements rate limiting, request queuing, and backoff for a component and tracks provider deprecation notices that affect it. Scope: a component's capacity behavior.</t>
+          <t>Depth: Gathers usage metrics and applies simple capacity estimates under guidance. Evidenced by: Monitors quota and rate-limit dashboards for their service and escalates approaching limits before they bite. Scope: task.</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Depth: plans capacity for a capability - load forecasting, quota negotiation inputs, multi-region or multi-provider failover design - and runs model-version migrations without user-visible regression. Scope: a capability's provider posture.</t>
+          <t>Depth: Produces standard capacity forecasts and resource budgets independently. Evidenced by: Implements rate limiting, request queuing, and backoff for a component and tracks provider deprecation notices that affect it. Scope: component.</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Depth: runs cross-team capacity and migration programs - org-wide model deprecation moves, shared quota pooling - that land on schedule. Scope: multiple teams.</t>
+          <t>Depth: Plans capacity autonomously; models demand, headroom, and resource trade-offs. Evidenced by: Plans capacity for a capability — load forecasting, quota negotiation inputs, multi-region or multi-provider failover design — and runs model-version migrations without user-visible regression. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the org's provider risk management - concentration risk, contractual SLAs, burst capacity. Scope: organization.</t>
+          <t>Depth: Defines capacity-planning approaches teams adopt; solves hard forecasting and efficiency problems. Evidenced by: Runs cross-team capacity and migration programs — org-wide model deprecation moves, shared quota pooling — that land on schedule. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets company posture on model-supply resilience as a business-continuity matter leadership understands. Scope: company.</t>
+          <t>Depth: Sets capacity and resource-budgeting strategy across systems; anticipates long-term demand shifts. Evidenced by: Owns the org's provider risk management — concentration risk, contractual SLAs, burst capacity. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes industry practice for capacity planning; pioneers influential approaches to resource budgeting. Evidenced by: Sets company posture on model-supply resilience as a business-continuity matter leadership understands. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2274,37 +2410,42 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Chen et al., "FrugalGPT" (2023)</t>
+          <t>Keeps systems fast and economical.</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Depth: states what their feature costs per request, attributing spend to prompt size, output length, and call count correctly, and checks the dashboard after changes ship. Scope: their tasks' spend.</t>
+          <t>FinOps Foundation, FinOps Framework (accessed 2026-07) — Chen et al.'s FrugalGPT paper has no bibliography entry; the FinOps Framework is OPS-07's own catalog anchor at P1-P4 and is the cost-accountability discipline this competency's per-call marginal-cost engineering responsibility instantiates for LLM spend.</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Depth: cuts a component's cost with measured, quality-neutral levers - prompt trimming, caching, batching, output caps - and reports the before/after against any quality change. Scope: a component's unit economics.</t>
+          <t>Depth: Understands cost/latency drivers of what they build. Evidenced by: States what their feature costs per request, attributing spend to prompt size, output length, and call count correctly, and checks the dashboard after changes ship. Scope: task.</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the cost model of a capability - cost per request and per user action tracked against quality, budgets and anomaly alerts set, cost-quality trades explicit in design docs - and catches cost regressions in review before they ship. Scope: a capability's unit economics.</t>
+          <t>Depth: Applies standard optimizations; stays within cost/latency budgets. Evidenced by: Cuts a component's cost with measured, quality-neutral levers — prompt trimming, caching, batching, output caps — and reports the before/after against any quality change. Scope: component.</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Depth: finds the cross-team cost structure - shared caches, duplicated calls, misrouted traffic - and drives the fixes worth the most, with cost governance (attribution, budget reviews) teams adopt. Scope: multiple teams' spend.</t>
+          <t>Depth: Designs cost-aware architectures; defines and tracks unit economics for a domain. Evidenced by: Owns the cost model of a capability — cost per request and per user action tracked against quality, budgets and anomaly alerts set, cost-quality trades explicit in design docs. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the org's inference-spend strategy - forecasting at product scale, informing provider negotiations, deciding where cost work beats feature work. Scope: organization.</t>
+          <t>Depth: Expert in economics at scale (fleet optimization, build-vs-buy). Evidenced by: Finds the cross-team cost structure — shared caches, duplicated calls, misrouted traffic — and drives the fixes worth the most, with cost governance teams adopt. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>Depth: keeps AI gross margins viable at company level, shaping pricing and architecture together. Scope: company.</t>
+          <t>Depth: Owns org-level spend strategy; cost decisions change margins. Evidenced by: Owns the org's inference-spend strategy — forecasting at product scale, informing provider negotiations, deciding where cost work beats feature work. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes the company economics of the products. Evidenced by: Keeps AI gross margins viable at company level, shaping pricing and architecture together. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2331,37 +2472,42 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Huyen, *AI Engineering* (2025), inference-optimization chapters</t>
+          <t>Exposes models for low-latency, scalable inference across batch and real-time use.</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Depth: measures end-to-end latency for their feature - including time-to-first-token - and identifies the slowest stage from traces. Scope: their tasks.</t>
+          <t>Pope et al., Efficiently Scaling Transformer Inference (2022) — Huyen's AI Engineering has no bibliography entry; Pope et al.'s "Efficiently Scaling Transformer Inference" is AI-19's own catalog anchor at P3-P5 and is the exact-topic source for the claim that the smallest model meeting the quality bar is usually the right one, and someone has to prove which that is.</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Depth: applies standard latency levers independently - streaming, parallel calls, speculative work, caching - to hit a stated target, validated with p95, not averages. Scope: a component's latency budget.</t>
+          <t>Depth: Deploys models to a serving setup with given configs under review. Evidenced by: Measures end-to-end latency for their feature — including time-to-first-token — and identifies the slowest stage from traces. Scope: task.</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Depth: right-sizes models per task within a capability - proving with evals that the smaller, faster model holds the quality bar - designs routing that matches request difficulty to model tier, and defines latency SLOs users actually feel. Scope: a capability's performance envelope.</t>
+          <t>Depth: Serves models independently and applies standard latency and throughput tuning. Evidenced by: Applies standard latency levers independently — streaming, parallel calls, speculative work, caching — to hit a stated target, validated with p95, not averages. Scope: component.</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Depth: builds or mandates the routing and caching infrastructure multiple teams use to meet shared latency standards, and audits over-provisioned model use. Scope: multiple teams.</t>
+          <t>Depth: Optimizes serving for hard latency, scale, and cost constraints autonomously. Evidenced by: Right-sizes models per task within a capability — proving with evals that the smaller, faster model holds the quality bar — and defines latency SLOs users actually feel. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets the org's latency/quality/cost frontier and the serving investments (routing, caching, distillation, self-hosting) that move it. Scope: organization.</t>
+          <t>Depth: Defines serving and inference-optimization patterns others adopt. Evidenced by: Builds or mandates the routing and caching infrastructure multiple teams use to meet shared latency standards, and audits over-provisioned model use. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t>Depth: makes speed a company-level product advantage, deciding where the company competes on latency and the architectural commitments behind it. Scope: company.</t>
+          <t>Depth: Sets serving strategy and anticipates advances in inference efficiency. Evidenced by: Sets the org's latency/quality/cost frontier and the serving investments that move it. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines best practice for model serving across the discipline and is externally recognized. Evidenced by: Makes speed a company-level product advantage, deciding where the company competes on latency and the architectural commitments behind it. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2388,37 +2534,42 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>OWASP Top 10 for LLM Applications (2025) - LLM01 Prompt Injection</t>
+          <t>Builds secure-by-default systems.</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Depth: treats model output and retrieved content as untrusted - never executes, renders, or queries with it unescaped, never concatenates untrusted content into instructions - and can explain injection with a real example. Scope: their own code paths.</t>
+          <t>OWASP Foundation, OWASP Top 10 for Large Language Model Applications (2025) — OWASP's Top 10 for LLM Applications 2025 (LLM01 Prompt Injection) is an exact bibliography match: any content a model reads is a potential instruction channel, and agents with tools turn injection into action.</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Depth: builds injection defenses into a component - privilege separation between instructions and data, output validation, allowlisted tool arguments - and writes adversarial cases into its tests. Scope: a component's trust boundaries.</t>
+          <t>Depth: Understands core appsec; follows practices and flags concerns. Evidenced by: Treats model output and retrieved content as untrusted — never executes, renders, or queries with it unescaped — and can explain injection with a real example. Scope: task.</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Depth: threat-models a capability's model I/O paths end to end - including the untrusted-content, private-data, external-communication combination - designs least-privilege mitigations accepted by security review, and red-teams their own features before attackers do. Scope: a capability's attack surface; their threat model is reviewed, not re-derived, by others.</t>
+          <t>Depth: Applies least privilege; validates/sanitizes inputs; knows common attacks. Evidenced by: Builds injection defenses into a component — privilege separation between instructions and data, output validation, allowlisted tool arguments — and writes adversarial cases into its tests. Scope: component.</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets secure-by-default patterns for model I/O that multiple teams inherit from shared libraries - sanitization layers, tool-permission frameworks, injection suites in CI - and runs adversarial reviews of high-exposure launches. Scope: multiple teams.</t>
+          <t>Depth: Designs defense in depth; thinks in abuse cases; owns a domain's posture. Evidenced by: Threat-models a capability's model I/O paths end to end, designs least-privilege mitigations accepted by security review, and red-teams their own features before attackers do. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the org's LLM security program with the security org - threat models, red-team cadence, incident learnings folded back into platform defaults. Scope: organization.</t>
+          <t>Depth: Expert in securing systems at scale; leads red-teaming and remediation. Evidenced by: Sets secure-by-default patterns for model I/O that multiple teams inherit from shared libraries and runs adversarial reviews of high-exposure launches. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>Depth: is accountable for the company's AI attack surface - deciding what the company will and won't expose to untrusted input - and represents the posture to customers, auditors, and researchers. Scope: company.</t>
+          <t>Depth: Defines security strategy for the org's surface area. Evidenced by: Owns the org's LLM security program with the security org — threat models, red-team cadence, incident learnings folded back into platform defaults. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Company-level accountability; authority on the field. Evidenced by: Is accountable for the company's AI attack surface — deciding what the company will and won't expose to untrusted input — and represents the posture to customers, auditors, and researchers. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2445,37 +2596,42 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>NIST Privacy Framework (2020)</t>
+          <t>Bakes privacy, audit and regulatory controls into systems.</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Depth: follows the team's rules for what may enter prompts, logs, and eval data, and asks before sending a new data category to a model provider. Scope: data handling in their tasks.</t>
+          <t>NIST, NIST Privacy Framework: A Tool for Improving Privacy through Enterprise Risk Management, Version 1.0 (2020) — NIST's Privacy Framework is an exact bibliography match and OPS-09's own catalog anchor: prompts, traces, and eval sets are new copies of user data, and each is a leak path classic data governance doesn't automatically cover.</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>Depth: implements redaction and minimization in a component's pipelines - PII scrubbing before model calls, trace redaction, retention limits - and verifies with tests that sensitive fields don't leak into telemetry. Scope: a component's data flows.</t>
+          <t>Depth: Knows data handling has privacy implications; follows rules. Evidenced by: Follows the team's rules for what may enter prompts, logs, and eval data, and asks before sending a new data category to a model provider. Scope: task.</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the data-flow map of a capability end to end - what user data reaches which provider under what retention terms - designing minimization in rather than bolting it on, and catches new leak paths in design review. Scope: a capability's privacy posture.</t>
+          <t>Depth: Applies PII handling, redaction, residency and retention correctly. Evidenced by: Implements redaction and minimization in a component's pipelines and verifies with tests that sensitive fields don't leak into telemetry. Scope: component.</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Depth: standardizes privacy engineering for AI across teams - shared redaction tooling, review checklists, provider data-processing requirements - and audits the highest-sensitivity data flows. Scope: multiple teams.</t>
+          <t>Depth: Designs for compliance (consent, audit trails, regional rules); owns readiness for a domain. Evidenced by: Owns the data-flow map of a capability end to end — what user data reaches which provider under what retention terms — and catches new leak paths in design review. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the org's data posture toward model providers, partnering with legal on agreements, audits, and the hard cases like eval data versus deletion requests. Scope: organization.</t>
+          <t>Depth: Expert at translating regulation into controls; represents engineering in audits. Evidenced by: Standardizes privacy engineering for AI across teams — shared redaction tooling, review checklists, provider data-processing requirements — and audits the highest-sensitivity data flows. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>Depth: answers for the company's AI data-handling promises - what is committed to customers about their data, and the architecture that keeps it true. Scope: company.</t>
+          <t>Depth: Sets org compliance strategy; anticipates regulation. Evidenced by: Owns the org's data posture toward model providers, partnering with legal on agreements, audits, and the hard cases like eval data versus deletion requests. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Authoritative on the landscape; trusted interface to regulators. Evidenced by: Answers for the company's AI data-handling promises — what is committed to customers about their data, and the architecture that keeps it true. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2502,37 +2658,42 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Bai et al., "Constitutional AI: Harmlessness from AI Feedback" (2022)</t>
+          <t>Keeps AI behavior safe, honest and within bounds.</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Depth: wires existing guardrails into a feature - schema validation, content filters, refusal handling - verifies rejects follow the designed path, and escalates outputs that feel harmful rather than shipping past them. Scope: a task.</t>
+          <t>Bai et al., Constitutional AI: Harmlessness from AI Feedback, Anthropic (2022) — Bai et al.'s Constitutional AI paper is an exact bibliography match and one of AI-05's own catalog sources at P4: product-level safety is engineered in layers around the model, not delegated to it.</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Depth: implements layered guardrails for a component - input filters, output classifiers, safe-completion fallbacks - and measures their false-positive and false-negative rates instead of assuming they work. Scope: a component's safety layer.</t>
+          <t>Depth: Understands that models can be harmful, biased or confidently wrong; flags concerning behavior. Evidenced by: Wires existing guardrails into a feature, verifies rejects follow the designed path, and escalates outputs that feel harmful rather than shipping past them. Scope: task.</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>Depth: designs the control stack for a capability from a written risk analysis - which failures are prevented, detected, or accepted, and where each control lives (prompt, classifier, policy engine, UX) - testing guardrails adversarially before launch and owning the harm/annoyance trade explicitly. Scope: a capability's behavior boundaries.</t>
+          <t>Depth: Implements guardrails (filtering, refusal handling, grounding checks); designs honest UX. Evidenced by: Implements layered guardrails for a component and measures their false-positive and false-negative rates instead of assuming they work. Scope: component.</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Depth: standardizes guardrail patterns and shared safety infrastructure across teams - common classifiers, a policy taxonomy - with authority to block a ship on control gaps. Scope: multiple teams.</t>
+          <t>Depth: Designs layered safety proportional to stakes; evaluates for bias/misuse before launch. Evidenced by: Designs the control stack for a capability from a written risk analysis, testing guardrails adversarially before launch and owning the harm/annoyance trade explicitly. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the org's output-safety standards and red-teaming program, reporting residual risk honestly to leadership. Scope: organization.</t>
+          <t>Depth: Expert in safety system design at scale; defines oversight and escalation frameworks. Evidenced by: Standardizes guardrail patterns and shared safety infrastructure across teams, with authority to block a ship on control gaps. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>Depth: defines the company's safety bar for AI products - what its AI refuses, allows, and how that is defended publicly - including saying no to launches. Scope: company.</t>
+          <t>Depth: Deep expertise balancing capability and safety under real product pressure. Evidenced by: Owns the org's output-safety standards and red-teaming program, reporting residual risk honestly to leadership. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Recognized authority; establishes responsible AI as a value; externally credible. Evidenced by: Defines the company's safety bar for AI products — what its AI refuses, allows, and how that is defended publicly — including saying no to launches. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2559,37 +2720,42 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Weidinger et al., "Taxonomy of Risks Posed by Language Models" (FAccT 2022)</t>
+          <t>Investigates model errors and disparate outcomes to guide responsible improvement.</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Depth: recognizes and reports harmful or biased outputs found during development instead of shrugging them off as model quirks. Scope: their task.</t>
+          <t>Barocas, Hardt &amp; Narayanan, Fairness and Machine Learning: Limitations and Opportunities (MIT Press, 2023) — Weidinger et al.'s Taxonomy of Risks paper has no bibliography entry; Barocas, Hardt &amp; Narayanan's Fairness and Machine Learning is AI-15's own catalog anchor at P2-P5, and deployed models can produce harmful, biased, or overconfident output, so mitigation starts from a named harm profile, not a disclaimer.</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Depth: tests a component against the team's harm checklist - unsafe advice, bias probes across user groups, overconfident hallucination - and adds mitigations that measurably reduce hits. Scope: a component.</t>
+          <t>Depth: Runs prescribed bias and error checks under review. Evidenced by: Recognizes and reports harmful or biased outputs found during development instead of shrugging them off as model quirks. Scope: task.</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Depth: defines the harm profile for a capability - who can be hurt and how - ships mitigations (refusals, hedging, citations, escalation paths) with eval coverage per harm class, and makes a written ship/hold recommendation leadership can act on, escalating when asked to ship past a red line. Scope: a capability; launch reviews use their assessment.</t>
+          <t>Depth: Performs standard fairness and error analysis independently for routine models. Evidenced by: Tests a component against the team's harm checklist and adds mitigations that measurably reduce hits. Scope: component.</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets harm-analysis practice across teams and reviews launches with meaningful harm potential, arbitrating safety-vs-utility disputes with data. Scope: multiple teams.</t>
+          <t>Depth: Diagnoses subtle bias and failure modes in ambiguous cases and proposes remedies autonomously. Evidenced by: Defines the harm profile for a capability, ships mitigations with eval coverage per harm class, and makes a written ship/hold recommendation leadership can act on. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>Depth: operationalizes the org's responsible-AI commitments into engineering requirements teams can actually implement. Scope: organization.</t>
+          <t>Depth: Defines fairness and error-analysis frameworks others adopt. Evidenced by: Sets harm-analysis practice across teams and reviews launches with meaningful harm potential, arbitrating safety-vs-utility disputes with data. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>Depth: shapes the company's public safety posture and is accountable for it holding under scrutiny. Scope: company.</t>
+          <t>Depth: Sets fairness strategy and anticipates evolving ethical and regulatory expectations. Evidenced by: Operationalizes the org's responsible-AI commitments into engineering requirements teams can actually implement. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes industry practice for fairness and error analysis and is externally recognized. Evidenced by: Shapes the company's public safety posture and is accountable for it holding under scrutiny. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2616,37 +2782,42 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>NIST AI Risk Management Framework 1.0 (2023); EU AI Act (2024)</t>
+          <t>Assesses and governs the risk of AI systems through their lifecycle - classifying systems against recognized risk frameworks, converting findings into engineering requirements with owners, and keeping the evidence trail (evals, controls, incidents) audit-ready as systems and regulation change.</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Depth: completes the launch risk checklist for their change accurately - identifying who is affected if the model is wrong - and escalates anything the checklist doesn't cover. Scope: their task.</t>
+          <t>NIST, Artificial Intelligence Risk Management Framework (AI RMF 1.0), NIST AI 100-1 (2023) — Both original citations are exact bibliography matches — NIST's AI RMF 1.0 and the EU AI Act are AI-21's own catalog anchors (the EU AI Act appears explicitly in AI-21's P3/P5/P6 text) — and AI systems are entering a regulated era where classifying systems by risk and evidencing controls is table stakes for shipping.</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Depth: assesses a feature's failure impact before build - misuse, error harm, disparate performance - and documents residual risk and the design choices that reduce it, without being chased. Scope: a component's risk profile.</t>
+          <t>Depth: Completes the risk checklist for their change accurately - identifying who is affected if the model is wrong - and escalates anything the checklist doesn't cover. Evidenced by: Fills out the launch checklist noting that a wrong classification would misroute a customer's support ticket to the wrong queue, and flags to their lead that the checklist has no question covering non-English input. Scope: task.</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Depth: classifies a capability against the applicable risk framework, keeps its evidence pack (evals, controls, incidents) audit-ready, converts findings into engineering requirements with owners, and flags when a product change alters its risk class. Scope: a capability's risk register.</t>
+          <t>Depth: Assesses a feature's failure impact before build (misuse, error harm, disparate performance across user groups) and documents mitigations and residual risk unprompted. Evidenced by: Documents, before building a resume-screening feature, that the model underperforms on non-standard formats and adds a low-confidence-score fallback to human review without being asked. Scope: component.</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Depth: operates the cross-team AI risk-review process - fast enough that teams use it honestly, rigorous enough to catch real issues - and builds the governance tooling that makes compliance a byproduct of normal engineering. Scope: multiple teams' launches.</t>
+          <t>Depth: Classifies a domain against the applicable risk framework, keeps its evidence pack (evals, controls, incidents) audit-ready, converts findings into engineering requirements with owners, and flags when a product change alters the risk class. Evidenced by: Classifies the support-triage capability as limited-risk under the applicable framework, keeps its eval and incident log current for the quarterly audit, and flags to legal when a new use case would push it toward high-risk. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the org's AI governance program jointly with legal and risk, translating regulation into engineering requirements without freezing delivery. Scope: organization.</t>
+          <t>Depth: Operates a cross-team AI risk-review process - fast enough that teams use it honestly, rigorous enough to catch real issues - and builds governance tooling that makes compliance a byproduct of normal engineering. Evidenced by: Runs the weekly cross-team risk-review that every AI launch across four teams goes through, and ships the CI check that blocks a PR missing a risk classification before a human has to catch it. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>Depth: positions the company ahead of AI regulation, accountable to executives and boards for the risk posture and shaping its regulatory engagement. Scope: company.</t>
+          <t>Depth: Owns an organization's AI governance program jointly with legal and risk functions, translating regulation into engineering requirements without freezing delivery. Evidenced by: Co-owns the org's AI governance program with legal, turning a new regulation's high-risk-system obligations into a pre-launch checklist that ships features on schedule instead of stalling in review. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Positions a company ahead of AI regulation; accountable to executives, boards, and regulators for where the risk lines are drawn. Evidenced by: Briefs the board on where the company draws its AI risk lines before a regulator asks, and represents the company's position in an industry working group shaping upcoming AI-regulation guidance. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2673,37 +2844,42 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Zinkevich, "Rules of Machine Learning" (Google), Rule #1</t>
+          <t>Translates ambiguous business problems into well-posed, feasible ML approaches.</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Depth: states what user problem their task serves and raises it when a lookup table or heuristic would do what the ticket asks of a model. Scope: their tasks.</t>
+          <t>Zinkevich, Rules of Machine Learning: Best Practices for ML Engineering, Google (accessed 2026-07) — Zinkevich's Rules of Machine Learning is an exact bibliography match: the highest-leverage AI engineering decision is whether the problem needs a model at all, and Rule #1 ("don't be afraid to launch a product without machine learning") is this competency in one sentence.</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Depth: prototypes the simplest adequate approach first - rules, search, classical ML, or a model - and recommends the model only when it beats the baseline, with the comparison documented. Scope: a component's approach.</t>
+          <t>Depth: Translates a clearly scoped problem into a defined ML task under guidance. Evidenced by: States what user problem their task serves and raises it when a lookup table or heuristic would do what the ticket asks of a model. Scope: task.</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Depth: kills LLM-shaped solutions to non-LLM problems in design review with evidence, reframing vague 'add AI' asks into testable user outcomes product partners agree to, and matches technique to problem across a capability. Scope: a capability's problem space; PMs seek their framing early.</t>
+          <t>Depth: Frames routine problems as appropriate ML solutions independently. Evidenced by: Prototypes the simplest adequate approach first — rules, search, classical ML, or a model — and recommends the model only when it beats the baseline, with the comparison documented. Scope: component.</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Depth: installs solution-fit review in how multiple teams take on AI work, redirecting AI-for-its-own-sake proposals and unwinding the most expensive misfit projects. Scope: multiple teams' portfolios.</t>
+          <t>Depth: Frames ambiguous business problems into sound ML or non-ML approaches autonomously. Evidenced by: Kills LLM-shaped solutions to non-LLM problems in design review with evidence, reframing vague 'add AI' asks into testable user outcomes product partners agree to. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>Depth: shapes which problems the org points AI at, pairing with product leadership on where models genuinely change the offering and cancelling bets the evidence turns against. Scope: organization.</t>
+          <t>Depth: Defines solution-design patterns others adopt and reframes intractable problems. Evidenced by: Installs solution-fit review in how multiple teams take on AI work, redirecting AI-for-its-own-sake proposals and unwinding the most expensive misfit projects. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t>Depth: advises company leadership on what AI makes newly possible versus fashionable - and is right often enough to be believed. Scope: company.</t>
+          <t>Depth: Sets ML solution strategy and anticipates where applicable techniques are heading. Evidenced by: Shapes which problems the org points AI at, pairing with product leadership on where models genuinely change the offering and cancelling bets the evidence turns against. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Defines best practice for ML problem framing across the discipline and is externally recognized. Evidenced by: Advises company leadership on what AI makes newly possible versus fashionable — and is right often enough to be believed. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2730,37 +2906,42 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Forsgren, Humble &amp; Kim, *Accelerate* (2018)</t>
+          <t>Connects technical work to user and business value.</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Depth: states how their feature's success will be measured beyond 'it works' and checks the metric after launch rather than moving on. Scope: their features.</t>
+          <t>Forsgren, Humble &amp; Kim, Accelerate: The Science of Lean Software and DevOps (IT Revolution Press, 2018) — Forsgren, Humble &amp; Kim's Accelerate is an exact bibliography match: AI features are expensive per use, and proving they earn their cost with outcome metrics rather than delivery-throughput metrics alone is part of the job.</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Depth: defines success metrics with product partners before building and reports post-launch results honestly, including misses, reacting when product metrics and eval scores diverge. Scope: a component's outcomes.</t>
+          <t>Depth: Understands the capability they're building and who uses it. Evidenced by: States how their feature's success will be measured beyond 'it works' and checks the metric after launch rather than moving on. Scope: task.</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>Depth: connects a capability's engineering metrics to business outcomes - cost per outcome, retention, task completion - and recommends sunsetting features whose value evidence never arrives, with the data that justifies it. Scope: a capability's return on investment.</t>
+          <t>Depth: Frames own work in user/business outcomes, not just tasks. Evidenced by: Defines success metrics with product partners before building and reports post-launch results honestly, including misses. Scope: component.</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Depth: builds the value-measurement discipline multiple teams use for AI investments, surfacing which bets are and aren't paying off and reallocating effort when the numbers say so. Scope: multiple teams' portfolios.</t>
+          <t>Depth: Treats their area as a product; uses metrics to decide what to build for a domain. Evidenced by: Connects a capability's engineering metrics to business outcomes — cost per outcome, retention, task completion — and recommends sunsetting features whose value evidence never arrives. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns the org's account of AI value delivered, credible to finance and product alike, and reallocates engineering toward what the evidence supports. Scope: organization.</t>
+          <t>Depth: Expert at aligning technical bets with product strategy across teams. Evidenced by: Builds the value-measurement discipline multiple teams use for AI investments, surfacing which bets are and aren't paying off. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
-          <t>Depth: shapes how the company invests in AI based on demonstrated value, with numbers that survive diligence at board level. Scope: company.</t>
+          <t>Depth: Sets product direction for an org's technical surface. Evidenced by: Owns the org's account of AI value delivered, credible to finance and product alike, and reallocates engineering toward what the evidence supports. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes how the company creates value through technical products. Evidenced by: Shapes how the company invests in AI based on demonstrated value, with numbers that survive diligence at board level. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2787,37 +2968,42 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Yan et al., "What We Learned from a Year of Building with LLMs" (O'Reilly, 2024)</t>
+          <t>Forecasts and plans work credibly.</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Depth: breaks their work into small verifiable increments and flags early - with evidence - when the model can't do what the task assumed, instead of grinding silently. Scope: their tasks.</t>
+          <t>Cohn, Agile Estimating and Planning (Prentice Hall, 2005) — Yan et al.'s O'Reilly article has no bibliography entry; Cohn's Agile Estimating and Planning is PD-04's own catalog anchor at P1-P3 and is where the discipline of planning as a sequence that buys information before making promises originates — model capability being discovered, not specified, is the same problem at a different variance.</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Depth: plans feature work as a de-risking sequence - timeboxed feasibility spike, eval baseline, then build - giving estimates as ranges with stated confidence and re-planning visibly when the spike says no. Scope: a component's plan.</t>
+          <t>Depth: Learns to estimate; surfaces blockers; plans own tasks with guidance. Evidenced by: Breaks their work into small verifiable increments and flags early — with evidence — when the model can't do what the task assumed, instead of grinding silently. Scope: task.</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Depth: structures a capability's roadmap around its riskiest unknowns - feasibility gates before commitments, kill criteria stated before the spike starts and honored when triggered, a shippable fallback behind every model-dependent bet. Scope: a capability's roadmap; their spikes change roadmaps.</t>
+          <t>Depth: Estimates scoped work realistically; plans own 1-3 week projects. Evidenced by: Plans feature work as a de-risking sequence — timeboxed feasibility spike, eval baseline, then build — giving estimates as ranges with stated confidence. Scope: component.</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Depth: teaches teams to plan AI work honestly - separating engineering certainty from model uncertainty in commitments leaders can rely on - and de-risks the org's biggest AI commitments personally. Scope: multiple teams' planning.</t>
+          <t>Depth: Plans quarter-scale, multi-workstream efforts including dependencies. Evidenced by: Structures a capability's roadmap around its riskiest unknowns — feasibility gates before commitments, kill criteria stated before the spike starts and honored when triggered. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>Depth: shapes the org's portfolio of AI bets, balancing near-certain delivery against high-variance exploration and keeping leadership expectations calibrated to what evals actually show. Scope: organization.</t>
+          <t>Depth: Expert at planning large programs; anticipates risk early. Evidenced by: Teaches teams to plan AI work honestly — separating engineering certainty from model uncertainty in commitments leaders can rely on — and de-risks the org's biggest AI commitments personally. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t>Depth: times company bets against the model-capability curve - what to build now versus wait for - and is accountable for the calls. Scope: company.</t>
+          <t>Depth: Plans org-level programs across quarters/years. Evidenced by: Shapes the org's portfolio of AI bets, balancing near-certain delivery against high-variance exploration and keeping leadership expectations calibrated to what evals actually show. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes how the company plans major technical change. Evidenced by: Times company bets against the model-capability curve — what to build now versus wait for — and is accountable for the calls. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2844,37 +3030,42 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Humble &amp; Farley, *Continuous Delivery* (2010)</t>
+          <t>Manages how change reaches production safely — decoupling deploy from release with feature flags, staged and canary rollouts, rollback readiness, and migration sequencing that bounds the blast radius of every change.</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Depth: ships work in small reviewable increments behind flags as directed and rolls back their own change cleanly when asked. Scope: task-sized increments.</t>
+          <t>Humble &amp; Farley, Continuous Delivery: Reliable Software Releases through Build Test and Deployment Automation (Addison-Wesley, 2010) — Humble &amp; Farley's Continuous Delivery is an exact bibliography match and OPS-30's own catalog anchor at P1/P6: the safest way to ship nondeterministic behavior is in small, reversible, observable slices.</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Depth: designs a component's rollout as canary -&gt; percentage -&gt; full, watching evals and telemetry at each stage and rolling back on their own signal. Scope: a component's rollout.</t>
+          <t>Depth: Follows the release process exactly — flags, staged rollout steps, verification checklists — verifies their change in production, and rolls back with guidance. Evidenced by: Ships work in small reviewable increments behind flags as directed and rolls back their own change cleanly when asked. Scope: task.</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns progressive-delivery strategy for a capability - shadow modes for new models, reversible-by-design changes, automated rollback triggers - and their launches are uneventful. Scope: a capability's release engineering.</t>
+          <t>Depth: Ships behind flags with a rollback plan by default, monitors rollouts and reverts on their own judgment when signals degrade, and writes changes that tolerate both versions running during rollout. Evidenced by: Designs a component's rollout as canary -&gt; percentage -&gt; full, watching evals and telemetry at each stage and rolling back on their own signal. Scope: component.</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Depth: builds the progressive-delivery machinery multiple teams use for AI changes - flag conventions, automated rollback on eval regression. Scope: multiple teams.</t>
+          <t>Depth: Designs the rollout for risky changes — canary criteria, migration sequencing, flag lifecycle, kill switches — and reviews others' rollout plans for blast radius; the person teams ask how to ship something safely. Evidenced by: Owns progressive-delivery strategy for a capability — shadow modes for new models, reversible-by-design changes, automated rollback triggers — and their launches are uneventful. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets the org's release-engineering direction for AI products and its risk appetite per surface. Scope: organization.</t>
+          <t>Depth: Builds progressive-delivery machinery multiple teams release through (flag platforms, automated canary analysis, automated rollback), retiring deploy patterns that cause repeat incidents and measurably raising deploy frequency. Evidenced by: Builds the progressive-delivery machinery multiple teams use for AI changes — flag conventions, automated rollback on eval regression. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
-          <t>Depth: makes safe iteration speed a company capability competitors can't easily copy. Scope: company.</t>
+          <t>Depth: Owns release policy for an organization and its delivery metrics — rollout standards, freeze rules, environment strategy — dismantling ceremony that adds no safety. Evidenced by: Sets the org's release-engineering direction for AI products and its risk appetite per surface. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Sets how an entire company's software reaches customers — the risk posture products ship under — and defends it to executives, auditors, and regulators. Evidenced by: Makes safe iteration speed a company capability competitors can't easily copy. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2901,37 +3092,42 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>CircleCI Engineering Competency Matrix (progression.fyi/f/circle-ci)</t>
+          <t>Makes and keeps credible commitments.</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Depth: takes ownership of assigned tasks and communicates progress and blockers honestly, driving them to done without waiting to be asked. Scope: answerable for individual work items.</t>
+          <t>Willink &amp; Babin, Extreme Ownership: How U.S. Navy SEALs Lead and Win (St. Martin's Press, 2015) — The CircleCI Engineering Competency Matrix has no bibliography entry; Willink &amp; Babin's Extreme Ownership is PD-05's own catalog anchor at P2/P3/P4/P6 and is the source for the exact discipline this competency names — commitments made, kept, and renegotiated honestly, with no excuses.</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns components end to end and delivers committed work reliably, raising slips as soon as they are known. Scope: answerable for a component's quality and timeliness.</t>
+          <t>Depth: Takes ownership of assigned tasks; honest about progress and blockers. Evidenced by: Tells their lead two days early that the eval-harness ticket will slip because the golden dataset isn't ready, instead of going quiet until standup. Scope: task.</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns a capability and lands multi-week efforts without surprises, pushing back on unrealistic scope with reasons. Scope: others depend on their systems; answerable for the capability's outcomes.</t>
+          <t>Depth: Owns components end-to-end; delivers committed work reliably. Evidenced by: Delivers the retrieval-reranking component on the date they committed to, having flagged and absorbed a provider API change mid-sprint without missing the deadline. Scope: component.</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns cross-team initiatives, unblocking teams and killing failing approaches early. Scope: answerable to leadership for multi-team program outcomes.</t>
+          <t>Depth: Owns a domain; lands multi-week efforts without surprises; pushes back on unrealistic scope with reasons. Evidenced by: Owns the chatbot capability through a six-week model migration with no surprise regressions, and talks product out of a two-week scope add with a written cost estimate. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns an org-level portfolio of technical bets. Scope: answerable for org outcomes; sets direction others follow.</t>
+          <t>Depth: Owns cross-team initiatives; unblocks teams; kills failing approaches early. Evidenced by: Runs the cross-team migration off the deprecated embedding model, unblocking two teams stuck on the same provider quota issue and cutting a doomed fine-tuning effort before it burns another sprint. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>Depth: owns company-critical technical outcomes - leadership's go-to when something absolutely must land. Scope: company.</t>
+          <t>Depth: Owns an org-level portfolio of bets; sets direction others follow. Evidenced by: Owns the org's portfolio of AI reliability bets for the year, and three other teams plan their roadmaps around the sequencing they set. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Depth: The go-to when something company-critical must land. Evidenced by: Is who leadership calls in when the flagship AI feature's launch is at risk two weeks out, and lands it. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2958,37 +3154,42 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Larson, *Staff Engineer* (2021)</t>
+          <t>Conveys ideas clearly to the right audience.</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Depth: writes clear task updates, commit messages, and questions with enough context that responders don't have to ask for it, summarizing eval results without overstating them. Scope: their team's channels.</t>
+          <t>Larson, Staff Engineer: Leadership Beyond the Management Track (self-published, 2021) — AI systems are probabilistic and unfamiliar; Larson's Staff Engineer is CC-01's own catalog anchor at P3/P4 and argues the engineer who can explain them accurately shapes every decision around them.</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Depth: writes design notes and runbooks peers act on without follow-up questions, and explains model behavior and its limits to non-experts without jargon or overclaiming. Scope: a component's stakeholders.</t>
+          <t>Depth: Communicates status clearly; documentation is accurate. Evidenced by: Writes clear task updates, commit messages, and questions with enough context that responders don't have to ask for it, summarizing eval results without overstating them. Scope: task.</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Depth: writes the docs that settle decisions - options, evidence, recommendation - and translates eval results and AI trade-offs so accurately that product decisions built on their word hold up. Scope: a capability's decision record.</t>
+          <t>Depth: Writes clear design notes, runbooks and PRs; explains trade-offs without overselling. Evidenced by: Writes design notes and runbooks peers act on without follow-up questions, and explains model behavior and its limits to non-experts without jargon or overclaiming. Scope: component.</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Depth: aligns multiple teams through writing - RFCs, strategies, decision records cited months later as the reference - and presents AI capability and risk to leadership without dumbing it down. Scope: multiple teams.</t>
+          <t>Depth: Writes design docs that drive decisions; translates technical risk for non-technical stakeholders. Evidenced by: Writes the docs that settle decisions and translates eval results and AI trade-offs so accurately that product decisions built on their word hold up. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>Depth: communicates org-level technical direction upward and outward, translating between executive and engineering registers without loss, including bad news early. Scope: organization.</t>
+          <t>Depth: Expert at making complex capability/risk legible to executives without dumbing it down; RFCs align orgs. Evidenced by: Aligns multiple teams through writing — RFCs, strategies, decision records cited months later as the reference — and presents AI capability and risk to leadership without dumbing it down. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
-          <t>Depth: is the company's technical voice on AI internally and externally - talks, publications, customer and regulator conversations that move the company's position. Scope: company and industry.</t>
+          <t>Depth: Strategy memos leadership acts on; org-wide and external reach. Evidenced by: Communicates org-level technical direction upward and outward, translating between executive and engineering registers without loss, including bad news early. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>Depth: A clarifying voice at company scale; externally recognized. Evidenced by: Is the company's technical voice on AI internally and externally — talks, publications, customer and regulator conversations that move the company's position. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -3015,37 +3216,42 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>Skelton &amp; Pais, *Team Topologies* (2019)</t>
+          <t>Works productively with others toward shared goals.</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Depth: works effectively with designer and PM counterparts on task details, surfacing AI-specific constraints - latency, failure modes - early, and incorporates feedback without churn. Scope: their team.</t>
+          <t>Skelton &amp; Pais, Team Topologies (IT Revolution, 2019) — Skelton &amp; Pais's Team Topologies is an exact bibliography match and this ladder's convention for scope-vs-depth boundaries generally: AI features cut across product, design, data, legal, and security, and the seams are where they fail.</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Depth: partners with product and design on what the model can and can't support, involving them before the prompt is final and prototyping to resolve disagreements with evidence. Scope: a component's cross-functional loop.</t>
+          <t>Depth: Responsive to feedback; pairs willingly; asks for help appropriately. Evidenced by: Works effectively with designer and PM counterparts on task details, surfacing AI-specific constraints — latency, failure modes — early, and incorporates feedback without churn. Scope: task.</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>Depth: runs the cross-functional process for a capability - brings legal, security, and support in before launch, turns product intent into evaluable requirements - and resolves conflicts between functions without escalation. Scope: a capability's stakeholder set; peers in other functions seek them out.</t>
+          <t>Depth: Collaborates smoothly with adjacent functions; handles disagreement constructively. Evidenced by: Partners with product and design on what the model can and can't support, involving them before the prompt is final and prototyping to resolve disagreements with evidence. Scope: component.</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Depth: fixes broken cross-team interfaces - ownership gaps, handoff friction - building the review forums, interface agreements, and shared vocabularies several teams use. Scope: multiple teams' seams.</t>
+          <t>Depth: Builds strong cross-team relationships; resolves friction directly. Evidenced by: Runs the cross-functional process for a capability — brings legal, security, and support in before launch, turns product intent into evaluable requirements — and resolves conflicts between functions without escalation. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>Depth: builds the org's operating model between AI engineering and other functions - data, platform, trust, product - so work flows without heroics. Scope: organization.</t>
+          <t>Depth: Expert at aligning teams with competing priorities; mediates disputes between senior people. Evidenced by: Fixes broken cross-team interfaces — ownership gaps, handoff friction — building the review forums, interface agreements, and shared vocabularies several teams use. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>Depth: brokers company-level alignment on AI initiatives across executive functions with durable results. Scope: company.</t>
+          <t>Depth: Creates the forums and processes through which collaboration happens. Evidenced by: Builds the org's operating model between AI engineering and other functions — data, platform, trust, product — so work flows without heroics. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Builds coalitions at company scale and externally. Evidenced by: Brokers company-level alignment on AI initiatives across executive functions with durable results. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -3072,37 +3278,42 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Mitchell et al., "Model Cards for Model Reporting" (FAT* 2019)</t>
+          <t>Spreads understanding so others move faster.</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Depth: keeps the docs for what they build current - setup, known limits, gotchas - and files gaps they find in others'. Scope: their own work.</t>
+          <t>Gebru et al., Datasheets for Datasets, Communications of the ACM 64(12), 86-92 (2021) — Mitchell et al.'s Model Cards paper has no bibliography entry; Gebru et al.'s Datasheets for Datasets — Model Cards' own sister paper in the same responsible-AI-documentation research line — is the closest catalog-available source, and AI systems decay into folklore fast, so written behavior contracts are what survive team turnover.</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>Depth: documents a feature's behavior contract - intended use, eval results, failure modes, escalation paths - findable by the next engineer without asking. Scope: one component.</t>
+          <t>Depth: Shares what they learn; keeps their docs accurate. Evidenced by: Keeps the docs for what they build current — setup, known limits, gotchas — and files gaps they find in others'. Scope: task.</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>Depth: maintains the canonical documentation for a capability - architecture, prompt rationale, eval history, runbooks - and prunes stale docs as ruthlessly as stale code. Scope: a capability; new joiners onboard from their docs alone.</t>
+          <t>Depth: Documents their area well; proactively shares techniques with the team. Evidenced by: Documents a feature's behavior contract — intended use, eval results, failure modes, escalation paths — findable by the next engineer without asking. Scope: component.</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Depth: drives documentation standards for AI systems across teams - behavior cards, decision records - and reviews for compliance. Scope: multiple teams.</t>
+          <t>Depth: Creates documentation and forums that raise a whole domain's understanding. Evidenced by: Maintains the canonical documentation for a capability — architecture, prompt rationale, eval history, runbooks — and prunes stale docs as ruthlessly as stale code. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>Depth: builds the org's AI knowledge base as infrastructure, making internal expertise discoverable. Scope: organization.</t>
+          <t>Depth: Builds knowledge-sharing systems adopted across teams. Evidenced by: Drives documentation standards for AI systems across teams — behavior cards, decision records — and reviews for compliance. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
-          <t>Depth: externalizes company knowledge deliberately - publications, standards participation - where it compounds the company's position. Scope: company.</t>
+          <t>Depth: Defines how the org captures and spreads knowledge. Evidenced by: Builds the org's AI knowledge base as infrastructure, making internal expertise discoverable. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Shapes industry-facing knowledge practice. Evidenced by: Externalizes company knowledge deliberately — publications, standards participation — where it compounds the company's position. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -3129,37 +3340,42 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>Fournier, *The Manager's Path* (2017), mentoring chapters</t>
+          <t>Grows other people's capability.</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Depth: asks for help effectively and pays it forward, documenting what they learned where the next person will find it. Scope: their immediate peers.</t>
+          <t>Fournier, The Manager's Path (O'Reilly, 2017) — Fournier's The Manager's Path (mentoring chapters) is an exact bibliography match: AI engineering practice changes monthly, and teams that don't teach internally re-learn everything the hard way.</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>Depth: onboards new teammates onto the AI stack and pairs generously, turning their own review comments and repeated questions into reusable explanations. Scope: their team.</t>
+          <t>Depth: Receptive to mentoring; shares what they learn. Evidenced by: Asks for help effectively and pays it forward, documenting what they learned where the next person will find it. Scope: task.</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>Depth: mentors engineers deliberately - stretch tasks matched to gaps, feedback that names behavior and impact - and levels a team up on AI-specific craft (evals, prompting, agent design) it didn't have before; mentees ship independently sooner. Scope: a capability's engineers; the terminal-level expectation, sustainable indefinitely.</t>
+          <t>Depth: Helps onboard teammates; informally mentors juniors. Evidenced by: Onboards new teammates onto the AI stack and pairs generously, turning their own review comments and repeated questions into reusable explanations. Scope: component.</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Depth: grows senior engineers across teams, sponsoring others into leading work they would have led, and builds the guilds and curricula that scale beyond one-on-ones. Scope: multiple teams' talent.</t>
+          <t>Depth: Coaches engineers with growth-oriented feedback; measurably improves a team's skill. Evidenced by: Mentors engineers deliberately — stretch tasks matched to gaps, feedback that names behavior and impact — and levels a team up on AI-specific craft it didn't have before; mentees ship independently sooner. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>Depth: builds the org's AI-engineering bench - hiring bar, growth paths, promotion evidence, succession for critical systems. Scope: organization.</t>
+          <t>Depth: Develops future leads across teams; shapes hiring and onboarding. Evidenced by: Grows senior engineers across teams, sponsoring others into leading work they would have led, and builds the guilds and curricula that scale beyond one-on-ones. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
-          <t>Depth: develops the company's next generation of principal-level technical leaders, largely through others, and shapes how the company is known to candidates. Scope: company.</t>
+          <t>Depth: Develops senior engineers and leaders; builds culture deliberately. Evidenced by: Builds the org's AI-engineering bench — hiring bar, growth paths, promotion evidence, succession for critical systems. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Develops the next generation of top talent; legacy outlasts tenure. Evidenced by: Develops the company's next generation of principal-level technical leaders, largely through others, and shapes how the company is known to candidates. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -3186,37 +3402,42 @@
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Larson, *Staff Engineer* (2021) and StaffEng archetypes</t>
+          <t>Shapes technical direction beyond own work.</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Depth: volunteers for unglamorous work that unblocks others and raises risks early instead of waiting to be asked. Scope: their team's day-to-day.</t>
+          <t>Larson, Staff Engineer: Leadership Beyond the Management Track (self-published, 2021) — Larson's Staff Engineer and the StaffEng archetypes are an exact bibliography match and LI-03's own catalog anchor at P3-P5: past senior, direction-setting and alignment — not authority — are how technical outcomes land.</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>Depth: leads small technical efforts end to end - a migration, an integration - coordinating the people involved without formal authority or escalation. Scope: a component-sized effort.</t>
+          <t>Depth: Contributes informed opinions in technical discussions. Evidenced by: Volunteers for unglamorous work that unblocks others and raises risks early instead of waiting to be asked. Scope: task.</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets technical direction for a capability - making and documenting the contentious calls, taking responsibility when wrong - and is the engineer others seek out when an AI decision is stuck. Scope: a capability; the terminal-level leadership bar.</t>
+          <t>Depth: Influences component-level decisions through credibility. Evidenced by: Leads small technical efforts end to end — a migration, an integration — coordinating the people involved without formal authority or escalation. Scope: component.</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Depth: creates alignment across teams that don't report to them, landing multi-team initiatives - platform migrations, model transitions - through writing, relationships, and demonstrated judgment. Scope: multiple teams' roadmaps.</t>
+          <t>Depth: Sets technical direction for a domain; others align to their calls. Evidenced by: Sets technical direction for a capability — making and documenting the contentious calls, taking responsibility when wrong — and is the engineer others seek out when an AI decision is stuck. Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>Depth: drives the org's technical strategy for AI, choosing the few bets that matter and getting leadership and teams genuinely behind them. Scope: organization.</t>
+          <t>Depth: Shapes how multiple teams approach problems; trusted tiebreaker. Evidenced by: Creates alignment across teams that don't report to them, landing multi-team initiatives — platform migrations, model transitions — through writing, relationships, and demonstrated judgment. Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K44" s="4" t="inlineStr">
         <is>
-          <t>Depth: sets the company's long-term technical direction for AI, accountable for the bets years before they resolve. Scope: company.</t>
+          <t>Depth: Influences org-wide technical strategy. Evidenced by: Drives the org's technical strategy for AI, choosing the few bets that matter and getting leadership and teams genuinely behind them. Scope: organization.</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>Depth: Influences company strategic direction through insight. Evidenced by: Sets the company's long-term technical direction for AI, accountable for the bets years before they resolve. Scope: company.</t>
         </is>
       </c>
     </row>
@@ -5330,18 +5551,1296 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:D81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sources</t>
-        </is>
-      </c>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Grounds</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Encoding/serialization formats and schema evolution across storage and service boundaries</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Kleppmann, Designing Data-Intensive Applications: The Big Ideas Behind Reliable, Scalable, and Maintainable Systems (O'Reilly, 2017)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>System design &amp; architecture</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>https://dataintensive.net/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Origin of REST; underpins API design leveling</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Fielding, Architectural Styles and the Design of Network-based Software Architectures (PhD dissertation, University of California Irvine, 2000)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>API &amp; service design</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>https://roy.gbiv.com/pubs/dissertation/top.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Construction-discipline reference used to ground novice-to-competent coding levels</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>McConnell, Code Complete: A Practical Handbook of Software Construction, 2nd Edition (Microsoft Press, 2004)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Coding &amp; implementation</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>https://www.microsoftpressstore.com/store/code-complete-9780735619678</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Distinguishes programming from org-scale software engineering; anchors org-wide standard-setting levels</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Winters, Manshreck &amp; Wright, Software Engineering at Google: Lessons Learned from Programming Over Time (O'Reilly, 2020)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Code quality &amp; review</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>https://abseil.io/resources/swe-book</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Systematic-debugging-as-discipline framework</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Zeller, Why Programs Fail: A Guide to Systematic Debugging, 2nd Edition (Morgan Kaufmann, 2009)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Debugging &amp; systems diagnosis</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oreilly.com/library/view/why-programs-fail/9780123745156/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Origin of the test automation pyramid; verified by web search, no stable canonical URL for a direct citation</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Cohn, Succeeding with Agile: Software Development Using Scrum (Addison-Wesley, 2009)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Deterministic tests vs evals</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Empirical study of AI adoption's effect on delivery throughput/stability/productivity; anchors AI-augmented development leveling</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>DORA (Google Cloud), Accelerate State of DevOps Report 2024 (2024)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>AI-augmented development judgment</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>https://dora.dev/research/2024/dora-report/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>GPT-3; establishes in-context few-shot prompting as a technique</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Brown et al., Language Models are Few-Shot Learners, NeurIPS 2020</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Prompt design &amp; iteration</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2005.14165</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Cross-model foundation-model landscape, capability shifts and risk framing</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Bommasani et al., On the Opportunities and Risks of Foundation Models, Stanford CRFM (2021)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Model selection &amp; integration</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2108.07258</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Canonical articulation of type-driven boundary validation; anchors type-system and boundary-validation capabilities</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>King, Parse, Don't Validate (lexi-lambda.github.io, 2019)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Structured output &amp; schema design</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>https://lexi-lambda.github.io/blog/2019/11/05/parse-don-t-validate/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Origin of the retrieve-then-generate RAG architecture</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Lewis et al., Retrieval-Augmented Generation for Knowledge-Intensive NLP Tasks, NeurIPS 2020</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Retrieval &amp; grounding pipelines</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2005.11401</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>FAISS; index strategy and retrieval at scale</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Johnson, Douze &amp; Jegou, Billion-Scale Similarity Search with GPUs, IEEE Transactions on Big Data (2019)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Embeddings &amp; semantic search</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/1702.08734</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Survey of hybrid search, reranking and advanced RAG techniques beyond the base pipeline</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Gao et al., Retrieval-Augmented Generation for Large Language Models: A Survey (2023)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Context budget &amp; memory management</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2312.10997</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Formalizes the plan-act-observe agent loop</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Yao et al., ReAct: Synergizing Reasoning and Acting in Language Models, ICLR 2023</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Agent architecture &amp; orchestration</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2210.03629</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Open standard for tool/context interoperability across agentic systems</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Anthropic, Model Context Protocol Specification (2025-11-25)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Tool &amp; function design for agents</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>https://modelcontextprotocol.io/specification/2025-11-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>GOVERN/MAP/MEASURE/MANAGE functions for AI risk</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>NIST, Artificial Intelligence Risk Management Framework (AI RMF 1.0), NIST AI 100-1 (2023)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Human oversight &amp; autonomy boundaries</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nist.gov/publications/artificial-intelligence-risk-management-framework-ai-rmf-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Direct theory of idempotency and retry-safety for reliable messaging; link returns 403 to automated fetch but title/venue confirmed via web search</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Helland, Idempotence Is Not a Medical Condition, ACM Queue 10(4) (2012)</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Agent state &amp; failure recovery</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>https://queue.acm.org/detail.cfm?id=2187821</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Stability patterns: circuit breakers bulkheads blast-radius containment graceful degradation</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Nygard, Release It!: Design and Deploy Production-Ready Software, 2nd Edition (Pragmatic Bookshelf, 2018)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Agent containment &amp; blast-radius control</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>https://pragprog.com/titles/mnee2/release-it-second-edition/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Empirical study of data-quality failure cascades in production AI; link 403s but title/venue confirmed by web search</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Sambasivan et al., "Everyone wants to do the model work, not the data work": Data Cascades in High-Stakes AI, CHI 2021</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Eval sets &amp; golden data</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/doi/10.1145/3411764.3445518</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Validates and characterizes LLM-as-judge evaluation methodology</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Zheng et al., Judging LLM-as-a-Judge with MT-Bench and Chatbot Arena, NeurIPS 2023</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Eval metrics &amp; judge design</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2306.05685</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Names ML-specific technical debt patterns: entanglement, pipeline jungles, hidden feedback loops</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Sculley et al., Hidden Technical Debt in Machine Learning Systems, NeurIPS 2015</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Measurement-gated shipping</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>https://research.google/pubs/hidden-technical-debt-in-machine-learning-systems/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Three pillars of observability (logs metrics traces) and instrumentation challenges at scale -- link 403s to automated clients but title/publisher/year confirmed by WebSearch</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Sridharan, Distributed Systems Observability: A Guide to Building Robust Systems (O'Reilly, 2018)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Tracing &amp; instrumentation of AI systems</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oreilly.com/library/view/distributed-systems-observability/9781492033431/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Taxonomy of drift types and adaptation/detection strategies; link 403s but title/venue confirmed by web search</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Gama et al., A Survey on Concept Drift Adaptation, ACM Computing Surveys 46(4) (2014)</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Production monitoring &amp; drift detection</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>https://dl.acm.org/doi/10.1145/2523813</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Google's published postmortem/root-cause and diagnostic-tooling practice; anchors debugging leveling</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Beyer, Jones, Petoff &amp; Murphy (eds.), Site Reliability Engineering: How Google Runs Production Systems (O'Reilly/Google, 2016)</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Incident response for AI systems</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>https://sre.google/sre-book/table-of-contents/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Inform/Optimize/Operate maturity phases for cloud cost management</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>FinOps Foundation, FinOps Framework (accessed 2026-07)</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Token economics &amp; cost optimization</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.finops.org/framework/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Multi-dimensional partitioning for low-latency large-model inference at scale</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Pope et al., Efficiently Scaling Transformer Inference (2022)</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Latency &amp; model right-sizing</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2211.05102</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Named LLM-specific risk categories and mitigations</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>OWASP Foundation, OWASP Top 10 for Large Language Model Applications (2025)</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Prompt injection &amp; untrusted model I/O</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>https://owasp.org/www-project-top-10-for-large-language-model-applications/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Privacy risk-management structure: identify/govern/control/communicate/protect</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>NIST, NIST Privacy Framework: A Tool for Improving Privacy through Enterprise Risk Management, Version 1.0 (2020)</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Data privacy &amp; PII handling</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nist.gov/privacy-framework</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Self-critique/revision technique for scalable safety oversight</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Bai et al., Constitutional AI: Harmlessness from AI Feedback, Anthropic (2022)</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Guardrails &amp; output safety</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2212.08073</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Formalizes statistical fairness criteria and their trade-offs/impossibility results</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Barocas, Hardt &amp; Narayanan, Fairness and Machine Learning: Limitations and Opportunities (MIT Press, 2023)</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Harm mitigation &amp; safety behavior</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>https://fairmlbook.org/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Practice rules incl. leakage, training/serving skew, launching without ML</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Zinkevich, Rules of Machine Learning: Best Practices for ML Engineering, Google (accessed 2026-07)</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Problem framing &amp; solution fit</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>https://developers.google.com/machine-learning/guides/rules-of-ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Empirical linkage between deployment/release engineering maturity and organizational performance</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Forsgren, Humble &amp; Kim, Accelerate: The Science of Lean Software and DevOps (IT Revolution Press, 2018)</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Outcome measurement &amp; business value</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>https://itrevolution.com/product/accelerate/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Definitive agile estimation/planning practice reference</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Cohn, Agile Estimating and Planning (Prentice Hall, 2005)</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Planning under model uncertainty</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mountaingoatsoftware.com/books/agile-estimating-and-planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Deployment pipeline environment-parity and release-automation discipline</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Humble &amp; Farley, Continuous Delivery: Reliable Software Releases through Build Test and Deployment Automation (Addison-Wesley, 2010)</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Incremental delivery &amp; de-risking</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>https://continuousdelivery.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Ownership/accountability leadership doctrine; grounds delivery-accountability leveling</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Willink &amp; Babin, Extreme Ownership: How U.S. Navy SEALs Lead and Win (St. Martin's Press, 2015)</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Ownership &amp; delivery accountability</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>https://openlibrary.org/books/OL27197173M/Extreme_ownership</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Tech Lead / Solver / Architect / Right-Hand archetypes for senior IC technical leadership scope</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Larson, Staff Engineer: Leadership Beyond the Management Track (self-published, 2021)</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Technical communication &amp; writing</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>https://staffeng.com/book/</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Team boundaries; org-level team formation patterns</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Skelton &amp; Pais, Team Topologies (IT Revolution, 2019)</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Cross-functional collaboration</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Standardized dataset documentation: motivation, collection, provenance</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Gebru et al., Datasheets for Datasets, Communications of the ACM 64(12), 86-92 (2021)</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Documentation &amp; knowledge sharing</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/1803.09010</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Progression from tech lead credibility through senior engineering leadership</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Fournier, The Manager's Path (O'Reilly, 2017)</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Mentoring &amp; knowledge sharing</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oreilly.com/library/view/the-managers-path/9781491973882/</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr"/>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Kleppmann, Designing Data-Intensive Applications: The Big Ideas Behind Reliable, Scalable, and Maintainable Systems (O'Reilly, 2017) — https://dataintensive.net/</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr"/>
+      <c r="D41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr"/>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>SFIA Foundation, Skills Framework for the Information Age, version 9 (2024) — https://sfia-online.org/en/sfia-9</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr"/>
+      <c r="D42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr"/>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Larson, Staff Engineer: Leadership Beyond the Management Track (self-published, 2021) — https://staffeng.com/book/</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr"/>
+      <c r="D43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr"/>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Fielding, Architectural Styles and the Design of Network-based Software Architectures (PhD dissertation, University of California Irvine, 2000) — https://roy.gbiv.com/pubs/dissertation/top.htm</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr"/>
+      <c r="D44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr"/>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>McConnell, Code Complete: A Practical Handbook of Software Construction, 2nd Edition (Microsoft Press, 2004) — https://www.microsoftpressstore.com/store/code-complete-9780735619678</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr"/>
+      <c r="D45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr"/>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Winters, Manshreck &amp; Wright, Software Engineering at Google: Lessons Learned from Programming Over Time (O'Reilly, 2020) — https://abseil.io/resources/swe-book</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr"/>
+      <c r="D46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr"/>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Zeller, Why Programs Fail: A Guide to Systematic Debugging, 2nd Edition (Morgan Kaufmann, 2009) — https://www.oreilly.com/library/view/why-programs-fail/9780123745156/</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr"/>
+      <c r="D47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr"/>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Cohn, Succeeding with Agile: Software Development Using Scrum (Addison-Wesley, 2009)</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr"/>
+      <c r="D48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr"/>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>DORA (Google Cloud), Accelerate State of DevOps Report 2024 (2024) — https://dora.dev/research/2024/dora-report/</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr"/>
+      <c r="D49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr"/>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Brown et al., Language Models are Few-Shot Learners, NeurIPS 2020 — https://arxiv.org/abs/2005.14165</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr"/>
+      <c r="D50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr"/>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Bommasani et al., On the Opportunities and Risks of Foundation Models, Stanford CRFM (2021) — https://arxiv.org/abs/2108.07258</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr"/>
+      <c r="D51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr"/>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>King, Parse, Don't Validate (lexi-lambda.github.io, 2019) — https://lexi-lambda.github.io/blog/2019/11/05/parse-don-t-validate/</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr"/>
+      <c r="D52" s="4" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr"/>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Lewis et al., Retrieval-Augmented Generation for Knowledge-Intensive NLP Tasks, NeurIPS 2020 — https://arxiv.org/abs/2005.11401</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr"/>
+      <c r="D53" s="4" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr"/>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Johnson, Douze &amp; Jegou, Billion-Scale Similarity Search with GPUs, IEEE Transactions on Big Data (2019) — https://arxiv.org/abs/1702.08734</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr"/>
+      <c r="D54" s="4" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr"/>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Gao et al., Retrieval-Augmented Generation for Large Language Models: A Survey (2023) — https://arxiv.org/abs/2312.10997</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr"/>
+      <c r="D55" s="4" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr"/>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Yao et al., ReAct: Synergizing Reasoning and Acting in Language Models, ICLR 2023 — https://arxiv.org/abs/2210.03629</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr"/>
+      <c r="D56" s="4" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr"/>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Anthropic, Model Context Protocol Specification (2025-11-25) — https://modelcontextprotocol.io/specification/2025-11-25</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr"/>
+      <c r="D57" s="4" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr"/>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>NIST, Artificial Intelligence Risk Management Framework (AI RMF 1.0), NIST AI 100-1 (2023) — https://www.nist.gov/publications/artificial-intelligence-risk-management-framework-ai-rmf-10</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr"/>
+      <c r="D58" s="4" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr"/>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Helland, Idempotence Is Not a Medical Condition, ACM Queue 10(4) (2012) — https://queue.acm.org/detail.cfm?id=2187821</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr"/>
+      <c r="D59" s="4" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr"/>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Nygard, Release It!: Design and Deploy Production-Ready Software, 2nd Edition (Pragmatic Bookshelf, 2018) — https://pragprog.com/titles/mnee2/release-it-second-edition/</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr"/>
+      <c r="D60" s="4" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr"/>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Sambasivan et al., "Everyone wants to do the model work, not the data work": Data Cascades in High-Stakes AI, CHI 2021 — https://dl.acm.org/doi/10.1145/3411764.3445518</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr"/>
+      <c r="D61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr"/>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>Zheng et al., Judging LLM-as-a-Judge with MT-Bench and Chatbot Arena, NeurIPS 2023 — https://arxiv.org/abs/2306.05685</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr"/>
+      <c r="D62" s="4" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr"/>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Sculley et al., Hidden Technical Debt in Machine Learning Systems, NeurIPS 2015 — https://research.google/pubs/hidden-technical-debt-in-machine-learning-systems/</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr"/>
+      <c r="D63" s="4" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr"/>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Sridharan, Distributed Systems Observability: A Guide to Building Robust Systems (O'Reilly, 2018) — https://www.oreilly.com/library/view/distributed-systems-observability/9781492033431/</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr"/>
+      <c r="D64" s="4" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr"/>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Gama et al., A Survey on Concept Drift Adaptation, ACM Computing Surveys 46(4) (2014) — https://dl.acm.org/doi/10.1145/2523813</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr"/>
+      <c r="D65" s="4" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr"/>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>Beyer, Jones, Petoff &amp; Murphy (eds.), Site Reliability Engineering: How Google Runs Production Systems (O'Reilly/Google, 2016) — https://sre.google/sre-book/table-of-contents/</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr"/>
+      <c r="D66" s="4" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr"/>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>FinOps Foundation, FinOps Framework (accessed 2026-07) — https://www.finops.org/framework/</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr"/>
+      <c r="D67" s="4" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr"/>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Pope et al., Efficiently Scaling Transformer Inference (2022) — https://arxiv.org/abs/2211.05102</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr"/>
+      <c r="D68" s="4" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr"/>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>OWASP Foundation, OWASP Top 10 for Large Language Model Applications (2025) — https://owasp.org/www-project-top-10-for-large-language-model-applications/</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr"/>
+      <c r="D69" s="4" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr"/>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>NIST, NIST Privacy Framework: A Tool for Improving Privacy through Enterprise Risk Management, Version 1.0 (2020) — https://www.nist.gov/privacy-framework</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr"/>
+      <c r="D70" s="4" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr"/>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Bai et al., Constitutional AI: Harmlessness from AI Feedback, Anthropic (2022) — https://arxiv.org/abs/2212.08073</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr"/>
+      <c r="D71" s="4" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr"/>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Barocas, Hardt &amp; Narayanan, Fairness and Machine Learning: Limitations and Opportunities (MIT Press, 2023) — https://fairmlbook.org/</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr"/>
+      <c r="D72" s="4" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr"/>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>European Parliament and Council, Regulation (EU) 2024/1689 (Artificial Intelligence Act) (2024) — https://eur-lex.europa.eu/eli/reg/2024/1689/oj/eng</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr"/>
+      <c r="D73" s="4" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr"/>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>Zinkevich, Rules of Machine Learning: Best Practices for ML Engineering, Google (accessed 2026-07) — https://developers.google.com/machine-learning/guides/rules-of-ml</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr"/>
+      <c r="D74" s="4" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr"/>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Forsgren, Humble &amp; Kim, Accelerate: The Science of Lean Software and DevOps (IT Revolution Press, 2018) — https://itrevolution.com/product/accelerate/</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr"/>
+      <c r="D75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr"/>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Cohn, Agile Estimating and Planning (Prentice Hall, 2005) — https://www.mountaingoatsoftware.com/books/agile-estimating-and-planning</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr"/>
+      <c r="D76" s="4" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr"/>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Humble &amp; Farley, Continuous Delivery: Reliable Software Releases through Build Test and Deployment Automation (Addison-Wesley, 2010) — https://continuousdelivery.com/</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr"/>
+      <c r="D77" s="4" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr"/>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Willink &amp; Babin, Extreme Ownership: How U.S. Navy SEALs Lead and Win (St. Martin's Press, 2015) — https://openlibrary.org/books/OL27197173M/Extreme_ownership</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr"/>
+      <c r="D78" s="4" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr"/>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Skelton &amp; Pais, Team Topologies (IT Revolution, 2019)</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr"/>
+      <c r="D79" s="4" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr"/>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Gebru et al., Datasheets for Datasets, Communications of the ACM 64(12), 86-92 (2021) — https://arxiv.org/abs/1803.09010</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr"/>
+      <c r="D80" s="4" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr"/>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Fournier, The Manager's Path (O'Reilly, 2017) — https://www.oreilly.com/library/view/the-managers-path/9781491973882/</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr"/>
+      <c r="D81" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(render): blank-line separators in ladder cells
</commit_message>
<xml_diff>
--- a/roles/ai-engineer/ladder.xlsx
+++ b/roles/ai-engineer/ladder.xlsx
@@ -808,32 +808,44 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Implements designs specified by others; asks why, not just how. Evidenced by: Explains the system's architecture in their own words. Scope: task.</t>
+          <t>Depth: Implements designs specified by others; asks why, not just how.
+Evidenced by: Explains the system's architecture in their own words.
+Scope: task.</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs sound components; understands coupling, cohesion, interface design. Evidenced by: Designs a component and writes the short design note for it. Scope: component.</t>
+          <t>Depth: Designs sound components; understands coupling, cohesion, interface design.
+Evidenced by: Designs a component and writes the short design note for it.
+Scope: component.</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs systems for evolution: clean seams, versioned interfaces, replaceable parts. Evidenced by: Selects patterns by trade-off in design docs that name the alternatives and failure modes. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs systems for evolution: clean seams, versioned interfaces, replaceable parts.
+Evidenced by: Selects patterns by trade-off in design docs that name the alternatives and failure modes.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Mastery of architecture for complex systems; sets patterns and prevents drift. Evidenced by: Writes the reference architectures other teams instantiate. Scope: multiple teams.</t>
+          <t>Depth: Mastery of architecture for complex systems; sets patterns and prevents drift.
+Evidenced by: Writes the reference architectures other teams instantiate.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets multi-year architecture direction across the org. Evidenced by: Sets the architectural direction for AI systems across the org. Scope: organization.</t>
+          <t>Depth: Sets multi-year architecture direction across the org.
+Evidenced by: Sets the architectural direction for AI systems across the org.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>Depth: Authoritative and externally credible; defines architectural approach others follow. Evidenced by: Defines the company's long-horizon technical bets for AI systems. Scope: company.</t>
+          <t>Depth: Authoritative and externally credible; defines architectural approach others follow.
+Evidenced by: Defines the company's long-horizon technical bets for AI systems.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -870,32 +882,44 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands HTTP/REST and the deploy pipeline; makes guided changes. Evidenced by: Implements endpoints to an existing API contract, including error responses, and flags mismatches between spec and behavior. Scope: task.</t>
+          <t>Depth: Understands HTTP/REST and the deploy pipeline; makes guided changes.
+Evidenced by: Implements endpoints to an existing API contract, including error responses, and flags mismatches between spec and behavior.
+Scope: task.</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs clean APIs; understands rate limits, retries, timeouts, idempotency. Evidenced by: Designs the API surface for a component and documents it well enough that a consumer needs no walkthrough. Scope: component.</t>
+          <t>Depth: Designs clean APIs; understands rate limits, retries, timeouts, idempotency.
+Evidenced by: Designs the API surface for a component and documents it well enough that a consumer needs no walkthrough.
+Scope: component.</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs services for scale and cost; understands distributed failure modes. Evidenced by: Designs contracts that isolate consumers from model and provider changes and rejects designs that leak provider details to callers. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs services for scale and cost; understands distributed failure modes.
+Evidenced by: Designs contracts that isolate consumers from model and provider changes and rejects designs that leak provider details to callers.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in platform/service design (multi-tenancy, capacity, shared services). Evidenced by: Sets the API conventions multiple teams follow for model-backed services and retires inconsistent legacy surfaces with migration paths. Scope: multiple teams.</t>
+          <t>Depth: Expert in platform/service design (multi-tenancy, capacity, shared services).
+Evidenced by: Sets the API conventions multiple teams follow for model-backed services and retires inconsistent legacy surfaces with migration paths.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets interface standards used across the org. Evidenced by: Drives the org's interface strategy — which capabilities become shared platforms, and the deprecation policy that keeps the surface coherent. Scope: organization.</t>
+          <t>Depth: Sets interface standards used across the org.
+Evidenced by: Drives the org's interface strategy — which capabilities become shared platforms, and the deprecation policy that keeps the surface coherent.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines company-wide API approach; trusted with irreversible interface bets. Evidenced by: Shapes the company's external and partner-facing AI interfaces, balancing product commitments against provider volatility. Scope: company.</t>
+          <t>Depth: Defines company-wide API approach; trusted with irreversible interface bets.
+Evidenced by: Shapes the company's external and partner-facing AI interfaces, balancing product commitments against provider volatility.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -932,32 +956,44 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes working, readable code in the team's language; debugs own changes. Evidenced by: Implements the retry-with-backoff helper for a flaky provider call exactly to spec and finds the off-by-one in their own token-counting logic before it reaches review. Scope: task.</t>
+          <t>Depth: Writes working, readable code in the team's language; debugs own changes.
+Evidenced by: Implements the retry-with-backoff helper for a flaky provider call exactly to spec and finds the off-by-one in their own token-counting logic before it reaches review.
+Scope: task.</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Proficient in the primary language/ecosystem; handles errors, async and concurrency basics correctly. Evidenced by: Ships the async job that reprocesses failed embedding batches, handling partial-batch failures and concurrent writes to the vector store without a teammate having to point them out. Scope: component.</t>
+          <t>Depth: Proficient in the primary language/ecosystem; handles errors, async and concurrency basics correctly.
+Evidenced by: Ships the async job that reprocesses failed embedding batches, handling partial-batch failures and concurrent writes to the vector store without a teammate having to point them out.
+Scope: component.</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Code is a reference others learn from; debugs the hard problems (races, memory, nondeterminism). Evidenced by: Writes the concurrent request-batching code newer engineers copy verbatim, and is the one who finds the race condition in the streaming-response handler that only shows up under load. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Code is a reference others learn from; debugs the hard problems (races, memory, nondeterminism).
+Evidenced by: Writes the concurrent request-batching code newer engineers copy verbatim, and is the one who finds the race condition in the streaming-response handler that only shows up under load.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Mastery across multiple stacks/paradigms; solves problems others can't; sets implementation patterns. Evidenced by: Rewrites the team's Python retrieval service in Rust for a client with different concurrency guarantees, solving a memory-pressure bug in the vector index that stumped two other engineers. Scope: multiple teams.</t>
+          <t>Depth: Mastery across multiple stacks/paradigms; solves problems others can't; sets implementation patterns.
+Evidenced by: Rewrites the team's Python retrieval service in Rust for a client with different concurrency guarantees, solving a memory-pressure bug in the vector index that stumped two other engineers.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets implementation standards adopted across the org; anticipates where code breaks at scale. Evidenced by: Sets the org's async-error-handling convention after a postmortem shows three teams' AI services failed the same way under provider timeout spikes. Scope: organization.</t>
+          <t>Depth: Sets implementation standards adopted across the org; anticipates where code breaks at scale.
+Evidenced by: Sets the org's async-error-handling convention after a postmortem shows three teams' AI services failed the same way under provider timeout spikes.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Depth: Industry-level depth; authors foundational primitives and idioms others build on. Evidenced by: Writes the request-batching primitive now vendored into every AI service's client library company-wide, the reference implementation new hires study. Scope: company.</t>
+          <t>Depth: Industry-level depth; authors foundational primitives and idioms others build on.
+Evidenced by: Writes the request-batching primitive now vendored into every AI service's client library company-wide, the reference implementation new hires study.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -994,32 +1030,44 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes functional, readable code; uses version control correctly; responds well to review. Evidenced by: Submits small, reviewable changes that pass CI first try more often than not and responds to review feedback by fixing the pattern, not just the line. Scope: task.</t>
+          <t>Depth: Writes functional, readable code; uses version control correctly; responds well to review.
+Evidenced by: Submits small, reviewable changes that pass CI first try more often than not and responds to review feedback by fixing the pattern, not just the line.
+Scope: task.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes clean, documented, modular code; gives useful review feedback. Evidenced by: Reviews peers' changes with substantive comments and keeps the code they touch consistently readable. Scope: component.</t>
+          <t>Depth: Writes clean, documented, modular code; gives useful review feedback.
+Evidenced by: Reviews peers' changes with substantive comments and keeps the code they touch consistently readable.
+Scope: component.</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs for maintainability; leads refactors of problem areas; review feedback teaches. Evidenced by: Holds the quality bar in review for a whole domain, including AI-generated code, articulating why a change is risky rather than just that it is. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs for maintainability; leads refactors of problem areas; review feedback teaches.
+Evidenced by: Holds the quality bar in review for a whole domain, including AI-generated code, articulating why a change is risky rather than just that it is.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in code health at scale (shared libraries, deprecations, large migrations). Evidenced by: Codifies review and code-health standards multiple teams adopt and measurably reduces defect escape in the areas they steward. Scope: multiple teams.</t>
+          <t>Depth: Expert in code health at scale (shared libraries, deprecations, large migrations).
+Evidenced by: Codifies review and code-health standards multiple teams adopt and measurably reduces defect escape in the areas they steward.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes org-wide engineering standards for long-lived codebases. Evidenced by: Changes how the org reviews and maintains code — tooling, norms, and the standards for machine-authored changes. Scope: organization.</t>
+          <t>Depth: Shapes org-wide engineering standards for long-lived codebases.
+Evidenced by: Changes how the org reviews and maintains code — tooling, norms, and the standards for machine-authored changes.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines what good engineering looks like company-wide; externally recognized. Evidenced by: Sets the company's engineering quality bar, cited when quality trade-offs reach executive decisions. Scope: company.</t>
+          <t>Depth: Defines what good engineering looks like company-wide; externally recognized.
+Evidenced by: Sets the company's engineering quality bar, cited when quality trade-offs reach executive decisions.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1056,32 +1104,44 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Debugs issues in own code with support; uses basic tooling. Evidenced by: Reproduces a reported bug and bisects it to a candidate cause with guidance, reading logs and stack traces before asking for help. Scope: task.</t>
+          <t>Depth: Debugs issues in own code with support; uses basic tooling.
+Evidenced by: Reproduces a reported bug and bisects it to a candidate cause with guidance, reading logs and stack traces before asking for help.
+Scope: task.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Independently diagnoses defects in own area systematically. Evidenced by: Isolates faults across service boundaries unaided, distinguishing deterministic code bugs from model-behavior variance before escalating. Scope: component.</t>
+          <t>Depth: Independently diagnoses defects in own area systematically.
+Evidenced by: Isolates faults across service boundaries unaided, distinguishing deterministic code bugs from model-behavior variance before escalating.
+Scope: component.</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Leads diagnosis of hard, cross-cutting failures; root cause not symptoms. Evidenced by: Debugs the hardest failures in a capability, including intermittent model-dependent ones, and writes the reproduction others rerun. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Leads diagnosis of hard, cross-cutting failures; root cause not symptoms.
+Evidenced by: Debugs the hardest failures in a capability, including intermittent model-dependent ones, and writes the reproduction others rerun.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert at the rare/systemic failures; builds tooling that makes them visible. Evidenced by: Untangles cross-team failures where no single owner sees the whole path and leaves behind the instrumentation that makes the next one cheap. Scope: multiple teams.</t>
+          <t>Depth: Expert at the rare/systemic failures; builds tooling that makes them visible.
+Evidenced by: Untangles cross-team failures where no single owner sees the whole path and leaves behind the instrumentation that makes the next one cheap.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Depth: The person called for the worst failures; sets diagnostic practice org-wide. Evidenced by: Spots systemic failure classes from incident patterns across the org and drives the architectural fixes. Scope: organization.</t>
+          <t>Depth: The person called for the worst failures; sets diagnostic practice org-wide.
+Evidenced by: Spots systemic failure classes from incident patterns across the org and drives the architectural fixes.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Depth: Authority on diagnosis; advances the discipline. Evidenced by: Is the debugger of last resort for company-critical AI incidents and turns each into a durable prevention mechanism. Scope: company.</t>
+          <t>Depth: Authority on diagnosis; advances the discipline.
+Evidenced by: Is the debugger of last resort for company-critical AI incidents and turns each into a durable prevention mechanism.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1118,32 +1178,44 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes unit tests with guidance; tests own changes before merging. Evidenced by: Writes unit tests for the deterministic parts of a change and can say which behaviors are testable versus eval-able when asked. Scope: task.</t>
+          <t>Depth: Writes unit tests with guidance; tests own changes before merging.
+Evidenced by: Writes unit tests for the deterministic parts of a change and can say which behaviors are testable versus eval-able when asked.
+Scope: task.</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Applies the testing pyramid; everything shipped arrives tested; mocks dependencies sensibly. Evidenced by: Draws the test/eval boundary correctly for a component and keeps CI fast and free of flaky model-dependent assertions. Scope: component.</t>
+          <t>Depth: Applies the testing pyramid; everything shipped arrives tested; mocks dependencies sensibly.
+Evidenced by: Draws the test/eval boundary correctly for a component and keeps CI fast and free of flaky model-dependent assertions.
+Scope: component.</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs testable systems (contract, property-based, replay from prod); owns a test strategy. Evidenced by: Designs the verification strategy for a capability and rejects flaky model-in-the-loop tests in review with a stated rule. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs testable systems (contract, property-based, replay from prod); owns a test strategy.
+Evidenced by: Designs the verification strategy for a capability and rejects flaky model-in-the-loop tests in review with a stated rule.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in test strategy at scale (test data, environments, deployment safety). Evidenced by: Standardizes the test-vs-eval discipline across teams with shared fixtures, replay harnesses, and CI policy for what may block a merge. Scope: multiple teams.</t>
+          <t>Depth: Expert in test strategy at scale (test data, environments, deployment safety).
+Evidenced by: Standardizes the test-vs-eval discipline across teams with shared fixtures, replay harnesses, and CI policy for what may block a merge.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets testing/verification discipline across the org. Evidenced by: Owns the org's verification strategy for AI systems, funding the harnesses that make the right split cheap and killing the theater. Scope: organization.</t>
+          <t>Depth: Sets testing/verification discipline across the org.
+Evidenced by: Owns the org's verification strategy for AI systems, funding the harnesses that make the right split cheap and killing the theater.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes the company-wide quality culture; advances verification practice. Evidenced by: Sets company policy for what 'verified' means for AI products, traceable from CI to eval to production evidence. Scope: company.</t>
+          <t>Depth: Shapes the company-wide quality culture; advances verification practice.
+Evidenced by: Sets company policy for what 'verified' means for AI products, traceable from CI to eval to production evidence.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1180,32 +1252,44 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Uses AI coding tools with the output treated as a draft - reads every generated line, tests it, and can explain any part of the diff when asked. Evidenced by: Has the agent draft the schema-migration script, then reads and runs every line by hand and can walk a reviewer through why the down-migration is safe. Scope: task.</t>
+          <t>Depth: Uses AI coding tools with the output treated as a draft - reads every generated line, tests it, and can explain any part of the diff when asked.
+Evidenced by: Has the agent draft the schema-migration script, then reads and runs every line by hand and can walk a reviewer through why the down-migration is safe.
+Scope: task.</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Calibrates when generation helps and when it misleads for the work at hand; catches plausible-but-wrong generated code before review, and their AI-assisted changes pass review at the same rate as hand-written ones. Evidenced by: Accepts the agent's generated boilerplate for a new API route unchanged but rewrites its generated cache-invalidation logic by hand after spotting a stale-read bug; their AI-assisted PRs land clean at the same rate as their hand-written ones. Scope: component.</t>
+          <t>Depth: Calibrates when generation helps and when it misleads for the work at hand; catches plausible-but-wrong generated code before review, and their AI-assisted changes pass review at the same rate as hand-written ones.
+Evidenced by: Accepts the agent's generated boilerplate for a new API route unchanged but rewrites its generated cache-invalidation logic by hand after spotting a stale-read bug; their AI-assisted PRs land clean at the same rate as their hand-written ones.
+Scope: component.</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the norms for AI-assisted work in a domain - what may be delegated to agents, what verification it requires, how provenance is noted in review - and coaches others out of over-trust and under-use. Evidenced by: Writes the team's rule that agents may draft data-pipeline glue code unattended but never touch auth logic without a human diff review, and talks a skeptical teammate into trying agent-assisted refactors for mechanical renames instead of hand-editing forty files. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Sets the norms for AI-assisted work in a domain - what may be delegated to agents, what verification it requires, how provenance is noted in review - and coaches others out of over-trust and under-use.
+Evidenced by: Writes the team's rule that agents may draft data-pipeline glue code unattended but never touch auth logic without a human diff review, and talks a skeptical teammate into trying agent-assisted refactors for mechanical renames instead of hand-editing forty files.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines AI-assisted engineering practice across teams - where agents run in the delivery lifecycle, what gates their output - justified by throughput and defect data rather than vendor claims. Evidenced by: Decides, with six months of defect-escape data across three teams, which pipeline stages autonomous coding agents may run in unattended and which require a human gate before merge. Scope: multiple teams.</t>
+          <t>Depth: Defines AI-assisted engineering practice across teams - where agents run in the delivery lifecycle, what gates their output - justified by throughput and defect data rather than vendor claims.
+Evidenced by: Decides, with six months of defect-escape data across three teams, which pipeline stages autonomous coding agents may run in unattended and which require a human gate before merge.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Drives an organization's AI-augmented engineering strategy - tooling selection, workflow redesign, skill expectations - and adjusts policy from measured delivery outcomes. Evidenced by: Picks the org's standard coding-agent tooling after a bake-off, redesigns the PR template around provenance tags, and walks back a workflow change once the data shows it slowed incident response. Scope: organization.</t>
+          <t>Depth: Drives an organization's AI-augmented engineering strategy - tooling selection, workflow redesign, skill expectations - and adjusts policy from measured delivery outcomes.
+Evidenced by: Picks the org's standard coding-agent tooling after a bake-off, redesigns the PR template around provenance tags, and walks back a workflow change once the data shows it slowed incident response.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes how software engineering itself changes with AI at company and industry level; a credible public voice on what changes and what doesn't. Evidenced by: Writes the engineering blog post other companies cite when re-tooling their own build process around agentic coding. Scope: company.</t>
+          <t>Depth: Shapes how software engineering itself changes with AI at company and industry level; a credible public voice on what changes and what doesn't.
+Evidenced by: Writes the engineering blog post other companies cite when re-tooling their own build process around agentic coding.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1242,32 +1326,44 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands LLM basics (tokens, context windows, temperature, system prompts); calls model APIs correctly. Evidenced by: Makes targeted edits to existing prompts and verifies the effect against known cases before committing, following the team's prompt-versioning convention. Scope: task.</t>
+          <t>Depth: Understands LLM basics (tokens, context windows, temperature, system prompts); calls model APIs correctly.
+Evidenced by: Makes targeted edits to existing prompts and verifies the effect against known cases before committing, following the team's prompt-versioning convention.
+Scope: task.</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes effective prompts; uses structured outputs, function calling and streaming; understands model differences and pricing. Evidenced by: Writes production prompts from scratch and iterates against a saved sample set rather than one lucky output. Scope: component.</t>
+          <t>Depth: Writes effective prompts; uses structured outputs, function calling and streaming; understands model differences and pricing.
+Evidenced by: Writes production prompts from scratch and iterates against a saved sample set rather than one lucky output.
+Scope: component.</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert prompt/context design (few-shot, decomposition, chaining); knows when fine-tuning beats prompting (rarely); designs for model swappability. Evidenced by: Treats prompts as versioned, eval-gated artifacts and diagnoses failures to the responsible prompt section. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Expert prompt/context design (few-shot, decomposition, chaining); knows when fine-tuning beats prompting (rarely); designs for model swappability.
+Evidenced by: Treats prompts as versioned, eval-gated artifacts and diagnoses failures to the responsible prompt section.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Mastery of model behavior across providers and versions; designs upgrade-migration strategies; squeezes capability others can't. Evidenced by: Establishes prompt-engineering standards across teams and untangles the prompt failures others are stuck on. Scope: multiple teams.</t>
+          <t>Depth: Mastery of model behavior across providers and versions; designs upgrade-migration strategies; squeezes capability others can't.
+Evidenced by: Establishes prompt-engineering standards across teams and untangles the prompt failures others are stuck on.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Deep expertise; anticipates capability shifts (new modalities, reasoning models) and repositions ahead of them. Evidenced by: Drives org-wide prompt and context craft, deciding where prompting ends and fine-tuning or tool-building begins. Scope: organization.</t>
+          <t>Depth: Deep expertise; anticipates capability shifts (new modalities, reasoning models) and repositions ahead of them.
+Evidenced by: Drives org-wide prompt and context craft, deciding where prompting ends and fine-tuning or tool-building begins.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Depth: Authority on applied LLM engineering; may influence industry practice. Evidenced by: Represents the state of the art to the company, resetting practice when model generations obsolete current techniques. Scope: company.</t>
+          <t>Depth: Authority on applied LLM engineering; may influence industry practice.
+Evidenced by: Represents the state of the art to the company, resetting practice when model generations obsolete current techniques.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1304,32 +1400,44 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands LLM basics (tokens, context windows, temperature, system prompts); calls model APIs correctly. Evidenced by: Integrates a specified model through the team's client layer per existing patterns. Scope: task.</t>
+          <t>Depth: Understands LLM basics (tokens, context windows, temperature, system prompts); calls model APIs correctly.
+Evidenced by: Integrates a specified model through the team's client layer per existing patterns.
+Scope: task.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes effective prompts; uses structured outputs, function calling and streaming; understands model differences and pricing. Evidenced by: Runs a small structured comparison before picking a model for a feature and records the result. Scope: component.</t>
+          <t>Depth: Writes effective prompts; uses structured outputs, function calling and streaming; understands model differences and pricing.
+Evidenced by: Runs a small structured comparison before picking a model for a feature and records the result.
+Scope: component.</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert prompt/context design (few-shot, decomposition, chaining); knows when fine-tuning beats prompting (rarely); designs for model swappability. Evidenced by: Owns model choice for a capability, re-benchmarks when providers ship new models, and swaps models behind stable interfaces without consumer churn. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Expert prompt/context design (few-shot, decomposition, chaining); knows when fine-tuning beats prompting (rarely); designs for model swappability.
+Evidenced by: Owns model choice for a capability, re-benchmarks when providers ship new models, and swaps models behind stable interfaces without consumer churn.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Mastery of model behavior across providers and versions; designs upgrade-migration strategies; squeezes capability others can't. Evidenced by: Defines the model-selection playbook and abstraction layers multiple teams use, making provider swaps routine instead of rewrites. Scope: multiple teams.</t>
+          <t>Depth: Mastery of model behavior across providers and versions; designs upgrade-migration strategies; squeezes capability others can't.
+Evidenced by: Defines the model-selection playbook and abstraction layers multiple teams use, making provider swaps routine instead of rewrites.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Deep expertise; anticipates capability shifts (new modalities, reasoning models) and repositions ahead of them. Evidenced by: Sets the org's model portfolio strategy with cost and risk analysis leadership signs off on. Scope: organization.</t>
+          <t>Depth: Deep expertise; anticipates capability shifts (new modalities, reasoning models) and repositions ahead of them.
+Evidenced by: Sets the org's model portfolio strategy with cost and risk analysis leadership signs off on.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Depth: Authority on applied LLM engineering; may influence industry practice. Evidenced by: Owns the company's model-sourcing strategy and its biggest bets and negotiates the strategic provider commitments behind them. Scope: company.</t>
+          <t>Depth: Authority on applied LLM engineering; may influence industry practice.
+Evidenced by: Owns the company's model-sourcing strategy and its biggest bets and negotiates the strategic provider commitments behind them.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1366,32 +1474,44 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Uses the codebase's shared contract types and schema validators at boundaries rather than hand-casting external data, and can point to where a type is checked at runtime. Evidenced by: Validates model outputs against a given schema and handles rejects rather than trusting parses. Scope: task.</t>
+          <t>Depth: Uses the codebase's shared contract types and schema validators at boundaries rather than hand-casting external data, and can point to where a type is checked at runtime.
+Evidenced by: Validates model outputs against a given schema and handles rejects rather than trusting parses.
+Scope: task.</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Puts runtime validation at every I/O boundary they touch — requests, messages, configuration — deriving static types from the runtime schemas so compile-time and runtime cannot drift. Evidenced by: Designs output schemas and tool signatures the model reliably satisfies, measuring parse and validation failure rates. Scope: component.</t>
+          <t>Depth: Puts runtime validation at every I/O boundary they touch — requests, messages, configuration — deriving static types from the runtime schemas so compile-time and runtime cannot drift.
+Evidenced by: Designs output schemas and tool signatures the model reliably satisfies, measuring parse and validation failure rates.
+Scope: component.</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs end-to-end type integrity for a capability — schema-first contracts, generated clients, contract drift caught in continuous integration — and blocks unsound casts and unvalidated edges in review. Evidenced by: Owns the structured-I/O layer for a capability — schema evolution, repair strategies, when to constrain decoding versus post-validate. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs end-to-end type integrity for a capability — schema-first contracts, generated clients, contract drift caught in continuous integration — and blocks unsound casts and unvalidated edges in review.
+Evidenced by: Owns the structured-I/O layer for a capability — schema evolution, repair strategies, when to constrain decoding versus post-validate.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds the code-generation and contract-typing infrastructure multiple teams inherit, making boundary safety the default rather than a discipline, and resolves cross-team type drift at its source. Evidenced by: Sets cross-team standards for tool definitions and output contracts and audits integrations that skip them. Scope: multiple teams.</t>
+          <t>Depth: Builds the code-generation and contract-typing infrastructure multiple teams inherit, making boundary safety the default rather than a discipline, and resolves cross-team type drift at its source.
+Evidenced by: Sets cross-team standards for tool definitions and output contracts and audits integrations that skip them.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the organization's boundary-safety standard and the platform tooling that enforces it, with incident evidence showing the failure classes it removed. Evidenced by: Owns the org's model-I/O reliability strategy, driving shared validation infrastructure. Scope: organization.</t>
+          <t>Depth: Sets the organization's boundary-safety standard and the platform tooling that enforces it, with incident evidence showing the failure classes it removed.
+Evidenced by: Owns the org's model-I/O reliability strategy, driving shared validation infrastructure.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns contract-integrity strategy across products and external interfaces where a broken contract is a business event, and advances the state of practice publicly. Evidenced by: Defines company-wide norms for machine-actionable model output, including what external partners may depend on. Scope: company.</t>
+          <t>Depth: Owns contract-integrity strategy across products and external interfaces where a broken contract is a business event, and advances the state of practice publicly.
+Evidenced by: Defines company-wide norms for machine-actionable model output, including what external partners may depend on.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1428,32 +1548,44 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands embeddings, similarity search and why grounding reduces hallucination. Evidenced by: Runs and modifies an existing ingestion/retrieval pipeline and verifies retrieval hits by inspection. Scope: task.</t>
+          <t>Depth: Understands embeddings, similarity search and why grounding reduces hallucination.
+Evidenced by: Runs and modifies an existing ingestion/retrieval pipeline and verifies retrieval hits by inspection.
+Scope: task.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds standard RAG pipelines (chunking, embedding, retrieval, reranking); manages context budgets deliberately. Evidenced by: Builds a retrieval pipeline for a corpus end to end and measures retrieval quality separately from answer quality. Scope: component.</t>
+          <t>Depth: Builds standard RAG pipelines (chunking, embedding, retrieval, reranking); manages context budgets deliberately.
+Evidenced by: Builds a retrieval pipeline for a corpus end to end and measures retrieval quality separately from answer quality.
+Scope: component.</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs retrieval quality systems (hybrid search, reranking, freshness, citation, memory for multi-turn). Evidenced by: Diagnoses failures to the responsible stage with evidence and chooses hybrid, re-ranking, or structured-lookup strategies by measured trade-off. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs retrieval quality systems (hybrid search, reranking, freshness, citation, memory for multi-turn).
+Evidenced by: Diagnoses failures to the responsible stage with evidence and chooses hybrid, re-ranking, or structured-lookup strategies by measured trade-off.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in retrieval at scale (index strategy, multi-source federation, permission-aware retrieval). Evidenced by: Designs the retrieval architecture several teams share and consolidates duplicated pipelines into shared infrastructure. Scope: multiple teams.</t>
+          <t>Depth: Expert in retrieval at scale (index strategy, multi-source federation, permission-aware retrieval).
+Evidenced by: Designs the retrieval architecture several teams share and consolidates duplicated pipelines into shared infrastructure.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Deep expertise; anticipates how longer context and new architectures change retrieval economics. Evidenced by: Sets the org's knowledge-grounding strategy — what corpora exist, who owns them, entitlement-aware access, and quality accountability. Scope: organization.</t>
+          <t>Depth: Deep expertise; anticipates how longer context and new architectures change retrieval economics.
+Evidenced by: Sets the org's knowledge-grounding strategy — what corpora exist, who owns them, entitlement-aware access, and quality accountability.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>Depth: Mastery of the discipline; defines how AI systems access knowledge. Evidenced by: Decides company-level grounding bets — proprietary-data moats, retrieval vs. long-context vs. fine-tuning — and owns that thesis with executives. Scope: company.</t>
+          <t>Depth: Mastery of the discipline; defines how AI systems access knowledge.
+Evidenced by: Decides company-level grounding bets — proprietary-data moats, retrieval vs. long-context vs. fine-tuning — and owns that thesis with executives.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1490,32 +1622,44 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands embeddings, similarity search and why grounding reduces hallucination. Evidenced by: Generates and stores embeddings using the team's pipeline and explains what an embedding represents in plain language. Scope: task.</t>
+          <t>Depth: Understands embeddings, similarity search and why grounding reduces hallucination.
+Evidenced by: Generates and stores embeddings using the team's pipeline and explains what an embedding represents in plain language.
+Scope: task.</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds standard RAG pipelines (chunking, embedding, retrieval, reranking); manages context budgets deliberately. Evidenced by: Evaluates embedding models against the team's retrieval benchmarks and tunes similarity thresholds and index parameters with evidence. Scope: component.</t>
+          <t>Depth: Builds standard RAG pipelines (chunking, embedding, retrieval, reranking); manages context budgets deliberately.
+Evidenced by: Evaluates embedding models against the team's retrieval benchmarks and tunes similarity thresholds and index parameters with evidence.
+Scope: component.</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs retrieval quality systems (hybrid search, reranking, freshness, citation, memory for multi-turn). Evidenced by: Selects embedding models, dimensions, and index types by measured trade-off for a capability and designs re-embedding and migration plans when models change. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs retrieval quality systems (hybrid search, reranking, freshness, citation, memory for multi-turn).
+Evidenced by: Selects embedding models, dimensions, and index types by measured trade-off for a capability and designs re-embedding and migration plans when models change.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in retrieval at scale (index strategy, multi-source federation, permission-aware retrieval). Evidenced by: Standardizes embedding infrastructure across teams — shared models, versioning, migration tooling — ending per-team drift. Scope: multiple teams.</t>
+          <t>Depth: Expert in retrieval at scale (index strategy, multi-source federation, permission-aware retrieval).
+Evidenced by: Standardizes embedding infrastructure across teams — shared models, versioning, migration tooling — ending per-team drift.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Deep expertise; anticipates how longer context and new architectures change retrieval economics. Evidenced by: Drives the org's vector-infrastructure strategy, including build-vs-buy for vector stores and cost and scale planning. Scope: organization.</t>
+          <t>Depth: Deep expertise; anticipates how longer context and new architectures change retrieval economics.
+Evidenced by: Drives the org's vector-infrastructure strategy, including build-vs-buy for vector stores and cost and scale planning.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>Depth: Mastery of the discipline; defines how AI systems access knowledge. Evidenced by: Anticipates representation-layer shifts — multimodal embeddings, new architectures — and positions the company ahead of them. Scope: company.</t>
+          <t>Depth: Mastery of the discipline; defines how AI systems access knowledge.
+Evidenced by: Anticipates representation-layer shifts — multimodal embeddings, new architectures — and positions the company ahead of them.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1552,32 +1696,44 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands embeddings, similarity search and why grounding reduces hallucination. Evidenced by: Keeps requests within the context budget, truncating per team rules, and notices when overflow or truncation silently degrades output. Scope: task.</t>
+          <t>Depth: Understands embeddings, similarity search and why grounding reduces hallucination.
+Evidenced by: Keeps requests within the context budget, truncating per team rules, and notices when overflow or truncation silently degrades output.
+Scope: task.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds standard RAG pipelines (chunking, embedding, retrieval, reranking); manages context budgets deliberately. Evidenced by: Prioritizes what enters the window with explicit truncation rules and tests the effect of dropping each element. Scope: component.</t>
+          <t>Depth: Builds standard RAG pipelines (chunking, embedding, retrieval, reranking); manages context budgets deliberately.
+Evidenced by: Prioritizes what enters the window with explicit truncation rules and tests the effect of dropping each element.
+Scope: component.</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs retrieval quality systems (hybrid search, reranking, freshness, citation, memory for multi-turn). Evidenced by: Designs the context-assembly strategy for a capability and shows with evals where added context stops paying. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs retrieval quality systems (hybrid search, reranking, freshness, citation, memory for multi-turn).
+Evidenced by: Designs the context-assembly strategy for a capability and shows with evals where added context stops paying.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in retrieval at scale (index strategy, multi-source federation, permission-aware retrieval). Evidenced by: Defines context-management patterns multiple teams reuse and audits high-cost windows for waste. Scope: multiple teams.</t>
+          <t>Depth: Expert in retrieval at scale (index strategy, multi-source federation, permission-aware retrieval).
+Evidenced by: Defines context-management patterns multiple teams reuse and audits high-cost windows for waste.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Deep expertise; anticipates how longer context and new architectures change retrieval economics. Evidenced by: Drives org-level context and memory architecture, deciding what user and org state is durable memory versus per-request context. Scope: organization.</t>
+          <t>Depth: Deep expertise; anticipates how longer context and new architectures change retrieval economics.
+Evidenced by: Drives org-level context and memory architecture, deciding what user and org state is durable memory versus per-request context.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>Depth: Mastery of the discipline; defines how AI systems access knowledge. Evidenced by: Positions the company for context-regime shifts before they invalidate current designs. Scope: company.</t>
+          <t>Depth: Mastery of the discipline; defines how AI systems access knowledge.
+Evidenced by: Positions the company for context-regime shifts before they invalidate current designs.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1614,32 +1770,44 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands tool calling and the agent loop (plan, act, observe); knows why agents need constraints. Evidenced by: Traces an existing agent loop end to end, explaining why the agent took each step on a real transcript, and fixes defects in single steps. Scope: task.</t>
+          <t>Depth: Understands tool calling and the agent loop (plan, act, observe); knows why agents need constraints.
+Evidenced by: Traces an existing agent loop end to end, explaining why the agent took each step on a real transcript, and fixes defects in single steps.
+Scope: task.</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs good tool interfaces; builds single-agent workflows with sensible termination and confirmation points. Evidenced by: Builds single-agent workflows with a bounded tool set using the simplest pattern that works, with explicit termination conditions and step limits by default. Scope: component.</t>
+          <t>Depth: Designs good tool interfaces; builds single-agent workflows with sensible termination and confirmation points.
+Evidenced by: Builds single-agent workflows with a bounded tool set using the simplest pattern that works, with explicit termination conditions and step limits by default.
+Scope: component.</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs reliable multi-step agents (state, recovery, sandboxing, permissions, human-in-the-loop); knows when an agent is the wrong answer. Evidenced by: Chooses between workflow and autonomous-loop designs by failure-mode analysis and cuts autonomy when a simpler pipeline scores the same. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs reliable multi-step agents (state, recovery, sandboxing, permissions, human-in-the-loop); knows when an agent is the wrong answer.
+Evidenced by: Chooses between workflow and autonomous-loop designs by failure-mode analysis and cuts autonomy when a simpler pipeline scores the same.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in complex orchestration (multi-agent, long-running workflows, MCP-style standards) and safe constraint at scale. Evidenced by: Sets the agent-architecture patterns multiple teams follow and kills over-engineered designs with evidence. Scope: multiple teams.</t>
+          <t>Depth: Expert in complex orchestration (multi-agent, long-running workflows, MCP-style standards) and safe constraint at scale.
+Evidenced by: Sets the agent-architecture patterns multiple teams follow and kills over-engineered designs with evidence.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Deep expertise; anticipates how increasing model autonomy changes system design. Evidenced by: Owns the org's agentic-systems strategy, deciding where autonomy is worth its reliability cost and what the shared platform provides. Scope: organization.</t>
+          <t>Depth: Deep expertise; anticipates how increasing model autonomy changes system design.
+Evidenced by: Owns the org's agentic-systems strategy, deciding where autonomy is worth its reliability cost and what the shared platform provides.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>Depth: Authority on agentic systems; may influence emerging industry standards. Evidenced by: Sets company direction on agentic products — where agents act, where humans decide — informed by what current models can actually sustain. Scope: company.</t>
+          <t>Depth: Authority on agentic systems; may influence emerging industry standards.
+Evidenced by: Sets company direction on agentic products — where agents act, where humans decide — informed by what current models can actually sustain.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1676,32 +1844,44 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands tool calling and the agent loop (plan, act, observe); knows why agents need constraints. Evidenced by: Implements a tool to a given schema with validation and error strings a model can act on, and tests it standalone before wiring it to a model. Scope: task.</t>
+          <t>Depth: Understands tool calling and the agent loop (plan, act, observe); knows why agents need constraints.
+Evidenced by: Implements a tool to a given schema with validation and error strings a model can act on, and tests it standalone before wiring it to a model.
+Scope: task.</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs good tool interfaces; builds single-agent workflows with sensible termination and confirmation points. Evidenced by: Designs tool schemas a model uses correctly on the first try and iterates on them against transcripts of real misuse. Scope: component.</t>
+          <t>Depth: Designs good tool interfaces; builds single-agent workflows with sensible termination and confirmation points.
+Evidenced by: Designs tool schemas a model uses correctly on the first try and iterates on them against transcripts of real misuse.
+Scope: component.</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs reliable multi-step agents (state, recovery, sandboxing, permissions, human-in-the-loop); knows when an agent is the wrong answer. Evidenced by: Curates the tool surface of a capability — right granularity, idempotency and side-effect discipline, permission boundaries — pruning overlapping tools that confuse routing. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs reliable multi-step agents (state, recovery, sandboxing, permissions, human-in-the-loop); knows when an agent is the wrong answer.
+Evidenced by: Curates the tool surface of a capability — right granularity, idempotency and side-effect discipline, permission boundaries — pruning overlapping tools that confuse routing.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in complex orchestration (multi-agent, long-running workflows, MCP-style standards) and safe constraint at scale. Evidenced by: Defines tool-design standards and shared registries multiple teams consume, with review gates for high-risk tools, killing near-duplicate tools across agents. Scope: multiple teams.</t>
+          <t>Depth: Expert in complex orchestration (multi-agent, long-running workflows, MCP-style standards) and safe constraint at scale.
+Evidenced by: Defines tool-design standards and shared registries multiple teams consume, with review gates for high-risk tools, killing near-duplicate tools across agents.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Deep expertise; anticipates how increasing model autonomy changes system design. Evidenced by: Drives the org's tool and integration platform, deciding which internal systems get first-class tool interfaces. Scope: organization.</t>
+          <t>Depth: Deep expertise; anticipates how increasing model autonomy changes system design.
+Evidenced by: Drives the org's tool and integration platform, deciding which internal systems get first-class tool interfaces.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>Depth: Authority on agentic systems; may influence emerging industry standards. Evidenced by: Shapes the company's external tool ecosystem posture — what third parties may plug in, what the company exposes — as a durable interface bet. Scope: company.</t>
+          <t>Depth: Authority on agentic systems; may influence emerging industry standards.
+Evidenced by: Shapes the company's external tool ecosystem posture — what third parties may plug in, what the company exposes — as a durable interface bet.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1738,32 +1918,44 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands that models can be harmful, biased or confidently wrong; flags concerning behavior. Evidenced by: Implements the approval and confirmation steps a design specifies — never bypassing a human checkpoint without sign-off — and states which of their feature's actions are reversible. Scope: task.</t>
+          <t>Depth: Understands that models can be harmful, biased or confidently wrong; flags concerning behavior.
+Evidenced by: Implements the approval and confirmation steps a design specifies — never bypassing a human checkpoint without sign-off — and states which of their feature's actions are reversible.
+Scope: task.</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Implements guardrails (filtering, refusal handling, grounding checks); designs honest UX. Evidenced by: Designs approval gates by reversibility and blast radius, with dry-run modes, undo paths, and every escalation logged for audit. Scope: component.</t>
+          <t>Depth: Implements guardrails (filtering, refusal handling, grounding checks); designs honest UX.
+Evidenced by: Designs approval gates by reversibility and blast radius, with dry-run modes, undo paths, and every escalation logged for audit.
+Scope: component.</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs layered safety proportional to stakes; evaluates for bias/misuse before launch. Evidenced by: Calibrates autonomy per action class for a capability from observed override and failure data, and pushes back when a design grants an agent more authority than its error rate supports. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs layered safety proportional to stakes; evaluates for bias/misuse before launch.
+Evidenced by: Calibrates autonomy per action class for a capability from observed override and failure data, and pushes back when a design grants an agent more authority than its error rate supports.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in safety system design at scale; defines oversight and escalation frameworks. Evidenced by: Standardizes autonomy tiers and approval mechanisms across teams and reviews escalation designs for high-consequence actions. Scope: multiple teams.</t>
+          <t>Depth: Expert in safety system design at scale; defines oversight and escalation frameworks.
+Evidenced by: Standardizes autonomy tiers and approval mechanisms across teams and reviews escalation designs for high-consequence actions.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Deep expertise balancing capability and safety under real product pressure. Evidenced by: Owns the org's policy for delegated agent authority, aligned with legal and security, including the evidence bar for widening autonomy. Scope: organization.</t>
+          <t>Depth: Deep expertise balancing capability and safety under real product pressure.
+Evidenced by: Owns the org's policy for delegated agent authority, aligned with legal and security, including the evidence bar for widening autonomy.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Depth: Recognized authority; establishes responsible AI as a value; externally credible. Evidenced by: Decides how much authority the company delegates to AI systems in its products and operations and defends that line to regulators and customers. Scope: company.</t>
+          <t>Depth: Recognized authority; establishes responsible AI as a value; externally credible.
+Evidenced by: Decides how much authority the company delegates to AI systems in its products and operations and defends that line to regulators and customers.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1800,32 +1992,44 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Applies provided idempotency and retry patterns for simple cases under review. Evidenced by: Reproduces a failed agent run from its transcript and identifies the step where it went wrong — bad plan, bad tool result, lost state. Scope: task.</t>
+          <t>Depth: Applies provided idempotency and retry patterns for simple cases under review.
+Evidenced by: Reproduces a failed agent run from its transcript and identifies the step where it went wrong — bad plan, bad tool result, lost state.
+Scope: task.</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Implements standard reliability and retry handling independently. Evidenced by: Builds checkpointing, retries, loop limits, and budget caps into agent steps so a wandering run halts cheaply and an interrupted run resumes or fails cleanly. Scope: component.</t>
+          <t>Depth: Implements standard reliability and retry handling independently.
+Evidenced by: Builds checkpointing, retries, loop limits, and budget caps into agent steps so a wandering run halts cheaply and an interrupted run resumes or fails cleanly.
+Scope: component.</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs idempotent, reliable flows autonomously; resolves duplicate and partial-failure cases. Evidenced by: Designs the state and containment model for an agentic capability, quantifying compounded failure rates rather than trusting per-step accuracy, and proves recovery paths with fault injection. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs idempotent, reliable flows autonomously; resolves duplicate and partial-failure cases.
+Evidenced by: Designs the state and containment model for an agentic capability, quantifying compounded failure rates rather than trusting per-step accuracy, and proves recovery paths with fault injection.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines reliability patterns teams adopt; solves the hardest exactly-once and recovery problems. Evidenced by: Sets durable-execution and recovery patterns multiple teams adopt — resumable run state, saga-style compensation — with adoption they can show. Scope: multiple teams.</t>
+          <t>Depth: Defines reliability patterns teams adopt; solves the hardest exactly-once and recovery problems.
+Evidenced by: Sets durable-execution and recovery patterns multiple teams adopt — resumable run state, saga-style compensation — with adoption they can show.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets reliability and idempotency strategy across systems; anticipates evolving failure modes. Evidenced by: Drives the org's strategy for stateful, long-running AI execution, consolidating bespoke run-state code into platform, with reliability targets and failure drills. Scope: organization.</t>
+          <t>Depth: Sets reliability and idempotency strategy across systems; anticipates evolving failure modes.
+Evidenced by: Drives the org's strategy for stateful, long-running AI execution, consolidating bespoke run-state code into platform, with reliability targets and failure drills.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines best practice for reliability patterns industrywide; shapes widely adopted approaches. Evidenced by: Sets company reliability doctrine for autonomous systems, informing what the company will and won't promise customers. Scope: company.</t>
+          <t>Depth: Defines best practice for reliability patterns industrywide; shapes widely adopted approaches.
+Evidenced by: Sets company reliability doctrine for autonomous systems, informing what the company will and won't promise customers.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1862,32 +2066,44 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands tool calling and the agent loop (plan, act, observe); knows why agents need constraints. Evidenced by: Runs agents in the sandboxed environment provided and reports containment gaps they notice. Scope: task.</t>
+          <t>Depth: Understands tool calling and the agent loop (plan, act, observe); knows why agents need constraints.
+Evidenced by: Runs agents in the sandboxed environment provided and reports containment gaps they notice.
+Scope: task.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs good tool interfaces; builds single-agent workflows with sensible termination and confirmation points. Evidenced by: Scopes an agent's credentials and tool permissions to least privilege, and caps loops, spend, and side effects by construction. Scope: component.</t>
+          <t>Depth: Designs good tool interfaces; builds single-agent workflows with sensible termination and confirmation points.
+Evidenced by: Scopes an agent's credentials and tool permissions to least privilege, and caps loops, spend, and side effects by construction.
+Scope: component.</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs reliable multi-step agents (state, recovery, sandboxing, permissions, human-in-the-loop); knows when an agent is the wrong answer. Evidenced by: Designs containment for a capability's agents — sandboxing, budget kill-switches, reversible-by-default actions — and red-teams their own boundaries before launch. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs reliable multi-step agents (state, recovery, sandboxing, permissions, human-in-the-loop); knows when an agent is the wrong answer.
+Evidenced by: Designs containment for a capability's agents — sandboxing, budget kill-switches, reversible-by-default actions — and red-teams their own boundaries before launch.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in complex orchestration (multi-agent, long-running workflows, MCP-style standards) and safe constraint at scale. Evidenced by: Builds containment infrastructure several teams inherit rather than reimplement, and audits exceptions. Scope: multiple teams.</t>
+          <t>Depth: Expert in complex orchestration (multi-agent, long-running workflows, MCP-style standards) and safe constraint at scale.
+Evidenced by: Builds containment infrastructure several teams inherit rather than reimplement, and audits exceptions.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Deep expertise; anticipates how increasing model autonomy changes system design. Evidenced by: Sets the org's containment standards for autonomous systems and verifies them through game days. Scope: organization.</t>
+          <t>Depth: Deep expertise; anticipates how increasing model autonomy changes system design.
+Evidenced by: Sets the org's containment standards for autonomous systems and verifies them through game days.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>Depth: Authority on agentic systems; may influence emerging industry standards. Evidenced by: Owns the company's worst-case analysis for agentic products and the controls that bound it. Scope: company.</t>
+          <t>Depth: Authority on agentic systems; may influence emerging industry standards.
+Evidenced by: Owns the company's worst-case analysis for agentic products and the controls that bound it.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1924,32 +2140,44 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Labels data to clear guidelines and flags ambiguities under review. Evidenced by: Adds well-formed cases to an existing eval set, labeling edge cases consistently with the rubric and flagging ambiguous ones instead of guessing. Scope: task.</t>
+          <t>Depth: Labels data to clear guidelines and flags ambiguities under review.
+Evidenced by: Adds well-formed cases to an existing eval set, labeling edge cases consistently with the rubric and flagging ambiguous ones instead of guessing.
+Scope: task.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Curates and labels routine datasets independently, applying consistent guidelines. Evidenced by: Builds an eval set for a feature from production traces via error analysis, versioning golden data like code with documented inclusion criteria. Scope: component.</t>
+          <t>Depth: Curates and labels routine datasets independently, applying consistent guidelines.
+Evidenced by: Builds an eval set for a feature from production traces via error analysis, versioning golden data like code with documented inclusion criteria.
+Scope: component.</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs labeling schemes and resolves ambiguity and quality issues autonomously. Evidenced by: Owns the golden datasets of a capability, retiring stale cases and tracing every regression escape back to the missing case class. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs labeling schemes and resolves ambiguity and quality issues autonomously.
+Evidenced by: Owns the golden datasets of a capability, retiring stale cases and tracing every regression escape back to the missing case class.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines curation and annotation-quality standards others adopt. Evidenced by: Sets eval-data standards multiple teams follow and audits suites whose numbers look too good. Scope: multiple teams.</t>
+          <t>Depth: Defines curation and annotation-quality standards others adopt.
+Evidenced by: Sets eval-data standards multiple teams follow and audits suites whose numbers look too good.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets dataset strategy and anticipates shifts in labeling and curation practice. Evidenced by: Drives the org's evaluation-data strategy — shared corpora, labeling operations, data governance for eval assets. Scope: organization.</t>
+          <t>Depth: Sets dataset strategy and anticipates shifts in labeling and curation practice.
+Evidenced by: Drives the org's evaluation-data strategy — shared corpora, labeling operations, data governance for eval assets.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines industry best practice for dataset curation and is externally credible. Evidenced by: Defines how the company knows its AI works — the evidence doctrine cited in launch reviews and external claims. Scope: company.</t>
+          <t>Depth: Defines industry best practice for dataset curation and is externally credible.
+Evidenced by: Defines how the company knows its AI works — the evidence doctrine cited in launch reviews and external claims.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -1986,32 +2214,44 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands why 'it looked right in testing' is insufficient; runs existing evals and labels carefully. Evidenced by: Runs the eval harness and reads its reports correctly, distinguishing a real regression from noise with help and flagging results that look wrong instead of accepting them. Scope: task.</t>
+          <t>Depth: Understands why 'it looked right in testing' is insufficient; runs existing evals and labels carefully.
+Evidenced by: Runs the eval harness and reads its reports correctly, distinguishing a real regression from noise with help and flagging results that look wrong instead of accepting them.
+Scope: task.</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds basic eval sets from real usage; measures changes before shipping prompt/model updates. Evidenced by: Chooses graders that fit the behavior under test and spot-checks judge agreement against their own labels before trusting it. Scope: component.</t>
+          <t>Depth: Builds basic eval sets from real usage; measures changes before shipping prompt/model updates.
+Evidenced by: Chooses graders that fit the behavior under test and spot-checks judge agreement against their own labels before trusting it.
+Scope: component.</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs eval methodology (golden sets, LLM-as-judge with validation, human review, helpfulness/groundedness/safety metrics). Evidenced by: Designs the measurement itself for a capability — judges validated against human ratings with quantified agreement and bias, significance limits stated before declaring a win. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs eval methodology (golden sets, LLM-as-judge with validation, human review, helpfulness/groundedness/safety metrics).
+Evidenced by: Designs the measurement itself for a capability — judges validated against human ratings with quantified agreement and bias, significance limits stated before declaring a win.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in eval at scale (continuous eval, A/B testing AI features, drift detection). Evidenced by: Standardizes eval methodology across teams, calibrating judge models centrally so scores are comparable. Scope: multiple teams.</t>
+          <t>Depth: Expert in eval at scale (continuous eval, A/B testing AI features, drift detection).
+Evidenced by: Standardizes eval methodology across teams, calibrating judge models centrally so scores are comparable.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Deep expertise in measuring AI quality where ground truth is contested. Evidenced by: Owns the org's measurement strategy for AI quality, connecting offline evals to online outcomes and killing metrics that don't predict. Scope: organization.</t>
+          <t>Depth: Deep expertise in measuring AI quality where ground truth is contested.
+Evidenced by: Owns the org's measurement strategy for AI quality, connecting offline evals to online outcomes and killing metrics that don't predict.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>Depth: Mastery of the discipline; sets the bar for what 'proven to work' means. Evidenced by: Defines what 'good' means for the company's AI products in measurable terms executives, customers, and regulators accept. Scope: company.</t>
+          <t>Depth: Mastery of the discipline; sets the bar for what 'proven to work' means.
+Evidenced by: Defines what 'good' means for the company's AI products in measurable terms executives, customers, and regulators accept.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2048,32 +2288,44 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Adds tests to existing pipeline stages following defined configuration, reviewed before merge. Evidenced by: Runs the required evals before merging prompt or model changes and pastes results into the review, flagging regressions instead of explaining them away. Scope: task.</t>
+          <t>Depth: Adds tests to existing pipeline stages following defined configuration, reviewed before merge.
+Evidenced by: Runs the required evals before merging prompt or model changes and pastes results into the review, flagging regressions instead of explaining them away.
+Scope: task.</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Integrates and maintains automated test stages independently within standard pipelines. Evidenced by: Attaches eval deltas to every prompt, model, or retrieval change and blocks their own launches on regressions without being told. Scope: component.</t>
+          <t>Depth: Integrates and maintains automated test stages independently within standard pipelines.
+Evidenced by: Attaches eval deltas to every prompt, model, or retrieval change and blocks their own launches on regressions without being told.
+Scope: component.</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs fast, reliable test gating for complex pipelines balancing speed and confidence. Evidenced by: Defines the ship gate for a capability — which evals block release, what regression tolerance is, when human review is required — and holds the line under deadline pressure with the reasoning in writing. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs fast, reliable test gating for complex pipelines balancing speed and confidence.
+Evidenced by: Defines the ship gate for a capability — which evals block release, what regression tolerance is, when human review is required — and holds the line under deadline pressure with the reasoning in writing.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines continuous-testing patterns and gating strategy other teams adopt. Evidenced by: Installs measurement-gated release processes across teams — eval CI, canary analysis, staged rollouts teams actually use — and audits exceptions. Scope: multiple teams.</t>
+          <t>Depth: Defines continuous-testing patterns and gating strategy other teams adopt.
+Evidenced by: Installs measurement-gated release processes across teams — eval CI, canary analysis, staged rollouts teams actually use — and audits exceptions.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets continuous-testing strategy and anticipates how quality gates must evolve with delivery. Evidenced by: Owns the org's ship/no-ship framework for AI behavior changes and arbitrates escalations where speed and evidence conflict. Scope: organization.</t>
+          <t>Depth: Sets continuous-testing strategy and anticipates how quality gates must evolve with delivery.
+Evidenced by: Owns the org's ship/no-ship framework for AI behavior changes and arbitrates escalations where speed and evidence conflict.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines authoritative continuous-testing practice that shapes the discipline. Evidenced by: Sets company policy on the evidence required to ship AI behavior, balancing speed and risk explicitly. Scope: company.</t>
+          <t>Depth: Defines authoritative continuous-testing practice that shapes the discipline.
+Evidenced by: Sets company policy on the evidence required to ship AI behavior, balancing speed and risk explicitly.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2110,32 +2362,44 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands logs/metrics/traces; reads existing dashboards. Evidenced by: Uses existing traces to debug a failing request — walking prompt to retrieval to tool call to output — and adds a missing span when told what to capture. Scope: task.</t>
+          <t>Depth: Understands logs/metrics/traces; reads existing dashboards.
+Evidenced by: Uses existing traces to debug a failing request — walking prompt to retrieval to tool call to output — and adds a missing span when told what to capture.
+Scope: task.</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Instruments their services; builds dashboards; tunes alerts to limit noise. Evidenced by: Instruments a component end to end as structured spans with the metadata needed to reproduce any output later, with sampling and redaction applied correctly. Scope: component.</t>
+          <t>Depth: Instruments their services; builds dashboards; tunes alerts to limit noise.
+Evidenced by: Instruments a component end to end as structured spans with the metadata needed to reproduce any output later, with sampling and redaction applied correctly.
+Scope: component.</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs observability for complex systems (end-to-end traces, quality signals, cost attribution). Evidenced by: Designs the observability schema for a capability and builds the views that make failure clusters visible, answering 'why did this output happen' in minutes. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs observability for complex systems (end-to-end traces, quality signals, cost attribution).
+Evidenced by: Designs the observability schema for a capability and builds the views that make failure clusters visible, answering 'why did this output happen' in minutes.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in instrumentation trade-offs at scale, incl. privacy-safe logging. Evidenced by: Sets tracing conventions multiple teams emit, aligning attributes so cross-service AI requests join up in one lens. Scope: multiple teams.</t>
+          <t>Depth: Expert in instrumentation trade-offs at scale, incl. privacy-safe logging.
+Evidenced by: Sets tracing conventions multiple teams emit, aligning attributes so cross-service AI requests join up in one lens.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines org observability strategy. Evidenced by: Owns the org's AI observability platform strategy, including retention, privacy, and cost of trace data. Scope: organization.</t>
+          <t>Depth: Defines org observability strategy.
+Evidenced by: Owns the org's AI observability platform strategy, including retention, privacy, and cost of trace data.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes company-wide operational visibility; advances practice. Evidenced by: Ensures the company can answer 'why did the model do that?' for any production decision, as a matter of architecture. Scope: company.</t>
+          <t>Depth: Shapes company-wide operational visibility; advances practice.
+Evidenced by: Ensures the company can answer 'why did the model do that?' for any production decision, as a matter of architecture.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2172,32 +2436,44 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Watches configured monitors and reports alerts under guidance. Evidenced by: Watches the dashboards for their feature after deploys and escalates anomalies with the trace attached rather than assuming success. Scope: task.</t>
+          <t>Depth: Watches configured monitors and reports alerts under guidance.
+Evidenced by: Watches the dashboards for their feature after deploys and escalates anomalies with the trace attached rather than assuming success.
+Scope: task.</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets up standard performance and drift monitoring independently. Evidenced by: Builds behavioral monitors for a component with alert thresholds they can justify, promoting recurring failures into the eval set. Scope: component.</t>
+          <t>Depth: Sets up standard performance and drift monitoring independently.
+Evidenced by: Builds behavioral monitors for a component with alert thresholds they can justify, promoting recurring failures into the eval set.
+Scope: component.</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs monitoring that catches subtle drift and degradation autonomously and triages causes. Evidenced by: Detects silent degradation for a capability — baselines behavior, catches provider-side model changes and input-distribution drift — and has caught a real regression no user reported. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs monitoring that catches subtle drift and degradation autonomously and triages causes.
+Evidenced by: Detects silent degradation for a capability — baselines behavior, catches provider-side model changes and input-distribution drift — and has caught a real regression no user reported.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines monitoring and drift-detection patterns others adopt. Evidenced by: Standardizes behavioral monitoring and feedback-to-eval pipelines across teams, correlating cross-product regressions to a common upstream cause. Scope: multiple teams.</t>
+          <t>Depth: Defines monitoring and drift-detection patterns others adopt.
+Evidenced by: Standardizes behavioral monitoring and feedback-to-eval pipelines across teams, correlating cross-product regressions to a common upstream cause.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets monitoring strategy and anticipates advances in drift detection. Evidenced by: Owns the org's in-production AI quality picture, making drift review a routine practice with owners and SLAs. Scope: organization.</t>
+          <t>Depth: Sets monitoring strategy and anticipates advances in drift detection.
+Evidenced by: Owns the org's in-production AI quality picture, making drift review a routine practice with owners and SLAs.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines best practice for model monitoring and is externally credible. Evidenced by: Makes behavioral health a company-level operational metric, defining how the company absorbs provider upgrades without quality surprises. Scope: company.</t>
+          <t>Depth: Defines best practice for model monitoring and is externally credible.
+Evidenced by: Makes behavioral health a company-level operational metric, defining how the company absorbs provider upgrades without quality surprises.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2234,32 +2510,44 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands SLOs and common failure modes; keeps components healthy with guidance. Evidenced by: Implements the retry, timeout, and fallback behavior a design specifies and tests the failure path by forcing the failure, not just the happy path. Scope: task.</t>
+          <t>Depth: Understands SLOs and common failure modes; keeps components healthy with guidance.
+Evidenced by: Implements the retry, timeout, and fallback behavior a design specifies and tests the failure path by forcing the failure, not just the happy path.
+Scope: task.</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds retries, timeouts and fallbacks; understands blast radius. Evidenced by: Designs the degradation ladder for a component — retry budgets, circuit breaking on provider errors, cached or smaller-model fallbacks — and makes each rung observable. Scope: component.</t>
+          <t>Depth: Builds retries, timeouts and fallbacks; understands blast radius.
+Evidenced by: Designs the degradation ladder for a component — retry budgets, circuit breaking on provider errors, cached or smaller-model fallbacks — and makes each rung observable.
+Scope: component.</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs for graceful degradation; defines SLOs; accountable for a domain's reliability. Evidenced by: Owns availability design for a capability across providers — failover routing, brownout modes, load shedding — validated with game days rather than hope. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs for graceful degradation; defines SLOs; accountable for a domain's reliability.
+Evidenced by: Owns availability design for a capability across providers — failover routing, brownout modes, load shedding — validated with game days rather than hope.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in resilience and capacity planning at scale; drives down incidents systemically. Evidenced by: Builds the shared resilience layer multiple teams depend on and reviews launches for shared-fate provider risk. Scope: multiple teams.</t>
+          <t>Depth: Expert in resilience and capacity planning at scale; drives down incidents systemically.
+Evidenced by: Builds the shared resilience layer multiple teams depend on and reviews launches for shared-fate provider risk.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns org-level reliability; fixes risk in process and org design. Evidenced by: Owns org-level continuity for provider failure — multi-provider posture, capacity reservations, tested playbooks. Scope: organization.</t>
+          <t>Depth: Owns org-level reliability; fixes risk in process and org design.
+Evidenced by: Owns org-level continuity for provider failure — multi-provider posture, capacity reservations, tested playbooks.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the company's reliability philosophy. Evidenced by: Answers for company availability of AI products through provider incidents that make the news, setting the architecture doctrine behind the commitments. Scope: company.</t>
+          <t>Depth: Sets the company's reliability philosophy.
+Evidenced by: Answers for company availability of AI products through provider incidents that make the news, setting the architecture doctrine behind the commitments.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2296,32 +2584,44 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Responds to alerts with support; follows runbooks; escalates appropriately. Evidenced by: Follows the runbook during incidents, keeps the timeline updated, captures the traces responders need, and asks for help early. Scope: task.</t>
+          <t>Depth: Responds to alerts with support; follows runbooks; escalates appropriately.
+Evidenced by: Follows the runbook during incidents, keeps the timeline updated, captures the traces responders need, and asks for help early.
+Scope: task.</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Triages and resolves routine incidents; clear notes; takes on-call. Evidenced by: Debugs live model-system incidents independently — distinguishing provider outage from prompt regression from data problem — and writes the postmortem with concrete actions. Scope: component.</t>
+          <t>Depth: Triages and resolves routine incidents; clear notes; takes on-call.
+Evidenced by: Debugs live model-system incidents independently — distinguishing provider outage from prompt regression from data problem — and writes the postmortem with concrete actions.
+Scope: component.</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Leads response to complex failures; blameless postmortems; same failure never recurs. Evidenced by: Incident-commands for their capability, including quality and cost incidents that page no one by default, and drives postmortems to systemic fixes. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Leads response to complex failures; blameless postmortems; same failure never recurs.
+Evidenced by: Incident-commands for their capability, including quality and cost incidents that page no one by default, and drives postmortems to systemic fixes.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in incident-management design (rotations, severity, escalation). Evidenced by: Raises operational maturity across teams — severity definitions that include model-quality events, game days for AI failure classes, readiness reviews before launches. Scope: multiple teams.</t>
+          <t>Depth: Expert in incident-management design (rotations, severity, escalation).
+Evidenced by: Raises operational maturity across teams — severity definitions that include model-quality events, game days for AI failure classes, readiness reviews before launches.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Commands the highest-severity incidents; sets incident process org-wide. Evidenced by: Owns the org's incident-management standard for AI systems, reviewing the postmortems that cross team boundaries and closing systemic gaps. Scope: organization.</t>
+          <t>Depth: Commands the highest-severity incidents; sets incident process org-wide.
+Evidenced by: Owns the org's incident-management standard for AI systems, reviewing the postmortems that cross team boundaries and closing systemic gaps.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets the company's incident philosophy; calm authority in the worst moments. Evidenced by: Is the company's senior technical responder in its worst AI incidents and changes company practice from what they reveal. Scope: company.</t>
+          <t>Depth: Sets the company's incident philosophy; calm authority in the worst moments.
+Evidenced by: Is the company's senior technical responder in its worst AI incidents and changes company practice from what they reveal.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2358,32 +2658,44 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Gathers usage metrics and applies simple capacity estimates under guidance. Evidenced by: Monitors quota and rate-limit dashboards for their service and escalates approaching limits before they bite. Scope: task.</t>
+          <t>Depth: Gathers usage metrics and applies simple capacity estimates under guidance.
+Evidenced by: Monitors quota and rate-limit dashboards for their service and escalates approaching limits before they bite.
+Scope: task.</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Produces standard capacity forecasts and resource budgets independently. Evidenced by: Implements rate limiting, request queuing, and backoff for a component and tracks provider deprecation notices that affect it. Scope: component.</t>
+          <t>Depth: Produces standard capacity forecasts and resource budgets independently.
+Evidenced by: Implements rate limiting, request queuing, and backoff for a component and tracks provider deprecation notices that affect it.
+Scope: component.</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Plans capacity autonomously; models demand, headroom, and resource trade-offs. Evidenced by: Plans capacity for a capability — load forecasting, quota negotiation inputs, multi-region or multi-provider failover design — and runs model-version migrations without user-visible regression. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Plans capacity autonomously; models demand, headroom, and resource trade-offs.
+Evidenced by: Plans capacity for a capability — load forecasting, quota negotiation inputs, multi-region or multi-provider failover design — and runs model-version migrations without user-visible regression.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines capacity-planning approaches teams adopt; solves hard forecasting and efficiency problems. Evidenced by: Runs cross-team capacity and migration programs — org-wide model deprecation moves, shared quota pooling — that land on schedule. Scope: multiple teams.</t>
+          <t>Depth: Defines capacity-planning approaches teams adopt; solves hard forecasting and efficiency problems.
+Evidenced by: Runs cross-team capacity and migration programs — org-wide model deprecation moves, shared quota pooling — that land on schedule.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets capacity and resource-budgeting strategy across systems; anticipates long-term demand shifts. Evidenced by: Owns the org's provider risk management — concentration risk, contractual SLAs, burst capacity. Scope: organization.</t>
+          <t>Depth: Sets capacity and resource-budgeting strategy across systems; anticipates long-term demand shifts.
+Evidenced by: Owns the org's provider risk management — concentration risk, contractual SLAs, burst capacity.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes industry practice for capacity planning; pioneers influential approaches to resource budgeting. Evidenced by: Sets company posture on model-supply resilience as a business-continuity matter leadership understands. Scope: company.</t>
+          <t>Depth: Shapes industry practice for capacity planning; pioneers influential approaches to resource budgeting.
+Evidenced by: Sets company posture on model-supply resilience as a business-continuity matter leadership understands.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2420,32 +2732,44 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands cost/latency drivers of what they build. Evidenced by: States what their feature costs per request, attributing spend to prompt size, output length, and call count correctly, and checks the dashboard after changes ship. Scope: task.</t>
+          <t>Depth: Understands cost/latency drivers of what they build.
+Evidenced by: States what their feature costs per request, attributing spend to prompt size, output length, and call count correctly, and checks the dashboard after changes ship.
+Scope: task.</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Applies standard optimizations; stays within cost/latency budgets. Evidenced by: Cuts a component's cost with measured, quality-neutral levers — prompt trimming, caching, batching, output caps — and reports the before/after against any quality change. Scope: component.</t>
+          <t>Depth: Applies standard optimizations; stays within cost/latency budgets.
+Evidenced by: Cuts a component's cost with measured, quality-neutral levers — prompt trimming, caching, batching, output caps — and reports the before/after against any quality change.
+Scope: component.</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs cost-aware architectures; defines and tracks unit economics for a domain. Evidenced by: Owns the cost model of a capability — cost per request and per user action tracked against quality, budgets and anomaly alerts set, cost-quality trades explicit in design docs. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs cost-aware architectures; defines and tracks unit economics for a domain.
+Evidenced by: Owns the cost model of a capability — cost per request and per user action tracked against quality, budgets and anomaly alerts set, cost-quality trades explicit in design docs.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in economics at scale (fleet optimization, build-vs-buy). Evidenced by: Finds the cross-team cost structure — shared caches, duplicated calls, misrouted traffic — and drives the fixes worth the most, with cost governance teams adopt. Scope: multiple teams.</t>
+          <t>Depth: Expert in economics at scale (fleet optimization, build-vs-buy).
+Evidenced by: Finds the cross-team cost structure — shared caches, duplicated calls, misrouted traffic — and drives the fixes worth the most, with cost governance teams adopt.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns org-level spend strategy; cost decisions change margins. Evidenced by: Owns the org's inference-spend strategy — forecasting at product scale, informing provider negotiations, deciding where cost work beats feature work. Scope: organization.</t>
+          <t>Depth: Owns org-level spend strategy; cost decisions change margins.
+Evidenced by: Owns the org's inference-spend strategy — forecasting at product scale, informing provider negotiations, deciding where cost work beats feature work.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes the company economics of the products. Evidenced by: Keeps AI gross margins viable at company level, shaping pricing and architecture together. Scope: company.</t>
+          <t>Depth: Shapes the company economics of the products.
+Evidenced by: Keeps AI gross margins viable at company level, shaping pricing and architecture together.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2482,32 +2806,44 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Deploys models to a serving setup with given configs under review. Evidenced by: Measures end-to-end latency for their feature — including time-to-first-token — and identifies the slowest stage from traces. Scope: task.</t>
+          <t>Depth: Deploys models to a serving setup with given configs under review.
+Evidenced by: Measures end-to-end latency for their feature — including time-to-first-token — and identifies the slowest stage from traces.
+Scope: task.</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Serves models independently and applies standard latency and throughput tuning. Evidenced by: Applies standard latency levers independently — streaming, parallel calls, speculative work, caching — to hit a stated target, validated with p95, not averages. Scope: component.</t>
+          <t>Depth: Serves models independently and applies standard latency and throughput tuning.
+Evidenced by: Applies standard latency levers independently — streaming, parallel calls, speculative work, caching — to hit a stated target, validated with p95, not averages.
+Scope: component.</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Optimizes serving for hard latency, scale, and cost constraints autonomously. Evidenced by: Right-sizes models per task within a capability — proving with evals that the smaller, faster model holds the quality bar — and defines latency SLOs users actually feel. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Optimizes serving for hard latency, scale, and cost constraints autonomously.
+Evidenced by: Right-sizes models per task within a capability — proving with evals that the smaller, faster model holds the quality bar — and defines latency SLOs users actually feel.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines serving and inference-optimization patterns others adopt. Evidenced by: Builds or mandates the routing and caching infrastructure multiple teams use to meet shared latency standards, and audits over-provisioned model use. Scope: multiple teams.</t>
+          <t>Depth: Defines serving and inference-optimization patterns others adopt.
+Evidenced by: Builds or mandates the routing and caching infrastructure multiple teams use to meet shared latency standards, and audits over-provisioned model use.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets serving strategy and anticipates advances in inference efficiency. Evidenced by: Sets the org's latency/quality/cost frontier and the serving investments that move it. Scope: organization.</t>
+          <t>Depth: Sets serving strategy and anticipates advances in inference efficiency.
+Evidenced by: Sets the org's latency/quality/cost frontier and the serving investments that move it.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L29" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines best practice for model serving across the discipline and is externally recognized. Evidenced by: Makes speed a company-level product advantage, deciding where the company competes on latency and the architectural commitments behind it. Scope: company.</t>
+          <t>Depth: Defines best practice for model serving across the discipline and is externally recognized.
+Evidenced by: Makes speed a company-level product advantage, deciding where the company competes on latency and the architectural commitments behind it.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2544,32 +2880,44 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands core appsec; follows practices and flags concerns. Evidenced by: Treats model output and retrieved content as untrusted — never executes, renders, or queries with it unescaped — and can explain injection with a real example. Scope: task.</t>
+          <t>Depth: Understands core appsec; follows practices and flags concerns.
+Evidenced by: Treats model output and retrieved content as untrusted — never executes, renders, or queries with it unescaped — and can explain injection with a real example.
+Scope: task.</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Applies least privilege; validates/sanitizes inputs; knows common attacks. Evidenced by: Builds injection defenses into a component — privilege separation between instructions and data, output validation, allowlisted tool arguments — and writes adversarial cases into its tests. Scope: component.</t>
+          <t>Depth: Applies least privilege; validates/sanitizes inputs; knows common attacks.
+Evidenced by: Builds injection defenses into a component — privilege separation between instructions and data, output validation, allowlisted tool arguments — and writes adversarial cases into its tests.
+Scope: component.</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs defense in depth; thinks in abuse cases; owns a domain's posture. Evidenced by: Threat-models a capability's model I/O paths end to end, designs least-privilege mitigations accepted by security review, and red-teams their own features before attackers do. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs defense in depth; thinks in abuse cases; owns a domain's posture.
+Evidenced by: Threat-models a capability's model I/O paths end to end, designs least-privilege mitigations accepted by security review, and red-teams their own features before attackers do.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in securing systems at scale; leads red-teaming and remediation. Evidenced by: Sets secure-by-default patterns for model I/O that multiple teams inherit from shared libraries and runs adversarial reviews of high-exposure launches. Scope: multiple teams.</t>
+          <t>Depth: Expert in securing systems at scale; leads red-teaming and remediation.
+Evidenced by: Sets secure-by-default patterns for model I/O that multiple teams inherit from shared libraries and runs adversarial reviews of high-exposure launches.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines security strategy for the org's surface area. Evidenced by: Owns the org's LLM security program with the security org — threat models, red-team cadence, incident learnings folded back into platform defaults. Scope: organization.</t>
+          <t>Depth: Defines security strategy for the org's surface area.
+Evidenced by: Owns the org's LLM security program with the security org — threat models, red-team cadence, incident learnings folded back into platform defaults.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Depth: Company-level accountability; authority on the field. Evidenced by: Is accountable for the company's AI attack surface — deciding what the company will and won't expose to untrusted input — and represents the posture to customers, auditors, and researchers. Scope: company.</t>
+          <t>Depth: Company-level accountability; authority on the field.
+Evidenced by: Is accountable for the company's AI attack surface — deciding what the company will and won't expose to untrusted input — and represents the posture to customers, auditors, and researchers.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2606,32 +2954,44 @@
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Knows data handling has privacy implications; follows rules. Evidenced by: Follows the team's rules for what may enter prompts, logs, and eval data, and asks before sending a new data category to a model provider. Scope: task.</t>
+          <t>Depth: Knows data handling has privacy implications; follows rules.
+Evidenced by: Follows the team's rules for what may enter prompts, logs, and eval data, and asks before sending a new data category to a model provider.
+Scope: task.</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Applies PII handling, redaction, residency and retention correctly. Evidenced by: Implements redaction and minimization in a component's pipelines and verifies with tests that sensitive fields don't leak into telemetry. Scope: component.</t>
+          <t>Depth: Applies PII handling, redaction, residency and retention correctly.
+Evidenced by: Implements redaction and minimization in a component's pipelines and verifies with tests that sensitive fields don't leak into telemetry.
+Scope: component.</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs for compliance (consent, audit trails, regional rules); owns readiness for a domain. Evidenced by: Owns the data-flow map of a capability end to end — what user data reaches which provider under what retention terms — and catches new leak paths in design review. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs for compliance (consent, audit trails, regional rules); owns readiness for a domain.
+Evidenced by: Owns the data-flow map of a capability end to end — what user data reaches which provider under what retention terms — and catches new leak paths in design review.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert at translating regulation into controls; represents engineering in audits. Evidenced by: Standardizes privacy engineering for AI across teams — shared redaction tooling, review checklists, provider data-processing requirements — and audits the highest-sensitivity data flows. Scope: multiple teams.</t>
+          <t>Depth: Expert at translating regulation into controls; represents engineering in audits.
+Evidenced by: Standardizes privacy engineering for AI across teams — shared redaction tooling, review checklists, provider data-processing requirements — and audits the highest-sensitivity data flows.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets org compliance strategy; anticipates regulation. Evidenced by: Owns the org's data posture toward model providers, partnering with legal on agreements, audits, and the hard cases like eval data versus deletion requests. Scope: organization.</t>
+          <t>Depth: Sets org compliance strategy; anticipates regulation.
+Evidenced by: Owns the org's data posture toward model providers, partnering with legal on agreements, audits, and the hard cases like eval data versus deletion requests.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>Depth: Authoritative on the landscape; trusted interface to regulators. Evidenced by: Answers for the company's AI data-handling promises — what is committed to customers about their data, and the architecture that keeps it true. Scope: company.</t>
+          <t>Depth: Authoritative on the landscape; trusted interface to regulators.
+Evidenced by: Answers for the company's AI data-handling promises — what is committed to customers about their data, and the architecture that keeps it true.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2668,32 +3028,44 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands that models can be harmful, biased or confidently wrong; flags concerning behavior. Evidenced by: Wires existing guardrails into a feature, verifies rejects follow the designed path, and escalates outputs that feel harmful rather than shipping past them. Scope: task.</t>
+          <t>Depth: Understands that models can be harmful, biased or confidently wrong; flags concerning behavior.
+Evidenced by: Wires existing guardrails into a feature, verifies rejects follow the designed path, and escalates outputs that feel harmful rather than shipping past them.
+Scope: task.</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Implements guardrails (filtering, refusal handling, grounding checks); designs honest UX. Evidenced by: Implements layered guardrails for a component and measures their false-positive and false-negative rates instead of assuming they work. Scope: component.</t>
+          <t>Depth: Implements guardrails (filtering, refusal handling, grounding checks); designs honest UX.
+Evidenced by: Implements layered guardrails for a component and measures their false-positive and false-negative rates instead of assuming they work.
+Scope: component.</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs layered safety proportional to stakes; evaluates for bias/misuse before launch. Evidenced by: Designs the control stack for a capability from a written risk analysis, testing guardrails adversarially before launch and owning the harm/annoyance trade explicitly. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs layered safety proportional to stakes; evaluates for bias/misuse before launch.
+Evidenced by: Designs the control stack for a capability from a written risk analysis, testing guardrails adversarially before launch and owning the harm/annoyance trade explicitly.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert in safety system design at scale; defines oversight and escalation frameworks. Evidenced by: Standardizes guardrail patterns and shared safety infrastructure across teams, with authority to block a ship on control gaps. Scope: multiple teams.</t>
+          <t>Depth: Expert in safety system design at scale; defines oversight and escalation frameworks.
+Evidenced by: Standardizes guardrail patterns and shared safety infrastructure across teams, with authority to block a ship on control gaps.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Deep expertise balancing capability and safety under real product pressure. Evidenced by: Owns the org's output-safety standards and red-teaming program, reporting residual risk honestly to leadership. Scope: organization.</t>
+          <t>Depth: Deep expertise balancing capability and safety under real product pressure.
+Evidenced by: Owns the org's output-safety standards and red-teaming program, reporting residual risk honestly to leadership.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Depth: Recognized authority; establishes responsible AI as a value; externally credible. Evidenced by: Defines the company's safety bar for AI products — what its AI refuses, allows, and how that is defended publicly — including saying no to launches. Scope: company.</t>
+          <t>Depth: Recognized authority; establishes responsible AI as a value; externally credible.
+Evidenced by: Defines the company's safety bar for AI products — what its AI refuses, allows, and how that is defended publicly — including saying no to launches.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2730,32 +3102,44 @@
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Runs prescribed bias and error checks under review. Evidenced by: Recognizes and reports harmful or biased outputs found during development instead of shrugging them off as model quirks. Scope: task.</t>
+          <t>Depth: Runs prescribed bias and error checks under review.
+Evidenced by: Recognizes and reports harmful or biased outputs found during development instead of shrugging them off as model quirks.
+Scope: task.</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Performs standard fairness and error analysis independently for routine models. Evidenced by: Tests a component against the team's harm checklist and adds mitigations that measurably reduce hits. Scope: component.</t>
+          <t>Depth: Performs standard fairness and error analysis independently for routine models.
+Evidenced by: Tests a component against the team's harm checklist and adds mitigations that measurably reduce hits.
+Scope: component.</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Diagnoses subtle bias and failure modes in ambiguous cases and proposes remedies autonomously. Evidenced by: Defines the harm profile for a capability, ships mitigations with eval coverage per harm class, and makes a written ship/hold recommendation leadership can act on. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Diagnoses subtle bias and failure modes in ambiguous cases and proposes remedies autonomously.
+Evidenced by: Defines the harm profile for a capability, ships mitigations with eval coverage per harm class, and makes a written ship/hold recommendation leadership can act on.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines fairness and error-analysis frameworks others adopt. Evidenced by: Sets harm-analysis practice across teams and reviews launches with meaningful harm potential, arbitrating safety-vs-utility disputes with data. Scope: multiple teams.</t>
+          <t>Depth: Defines fairness and error-analysis frameworks others adopt.
+Evidenced by: Sets harm-analysis practice across teams and reviews launches with meaningful harm potential, arbitrating safety-vs-utility disputes with data.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets fairness strategy and anticipates evolving ethical and regulatory expectations. Evidenced by: Operationalizes the org's responsible-AI commitments into engineering requirements teams can actually implement. Scope: organization.</t>
+          <t>Depth: Sets fairness strategy and anticipates evolving ethical and regulatory expectations.
+Evidenced by: Operationalizes the org's responsible-AI commitments into engineering requirements teams can actually implement.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes industry practice for fairness and error analysis and is externally recognized. Evidenced by: Shapes the company's public safety posture and is accountable for it holding under scrutiny. Scope: company.</t>
+          <t>Depth: Shapes industry practice for fairness and error analysis and is externally recognized.
+Evidenced by: Shapes the company's public safety posture and is accountable for it holding under scrutiny.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2792,32 +3176,44 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Completes the risk checklist for their change accurately - identifying who is affected if the model is wrong - and escalates anything the checklist doesn't cover. Evidenced by: Fills out the launch checklist noting that a wrong classification would misroute a customer's support ticket to the wrong queue, and flags to their lead that the checklist has no question covering non-English input. Scope: task.</t>
+          <t>Depth: Completes the risk checklist for their change accurately - identifying who is affected if the model is wrong - and escalates anything the checklist doesn't cover.
+Evidenced by: Fills out the launch checklist noting that a wrong classification would misroute a customer's support ticket to the wrong queue, and flags to their lead that the checklist has no question covering non-English input.
+Scope: task.</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Assesses a feature's failure impact before build (misuse, error harm, disparate performance across user groups) and documents mitigations and residual risk unprompted. Evidenced by: Documents, before building a resume-screening feature, that the model underperforms on non-standard formats and adds a low-confidence-score fallback to human review without being asked. Scope: component.</t>
+          <t>Depth: Assesses a feature's failure impact before build (misuse, error harm, disparate performance across user groups) and documents mitigations and residual risk unprompted.
+Evidenced by: Documents, before building a resume-screening feature, that the model underperforms on non-standard formats and adds a low-confidence-score fallback to human review without being asked.
+Scope: component.</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Classifies a domain against the applicable risk framework, keeps its evidence pack (evals, controls, incidents) audit-ready, converts findings into engineering requirements with owners, and flags when a product change alters the risk class. Evidenced by: Classifies the support-triage capability as limited-risk under the applicable framework, keeps its eval and incident log current for the quarterly audit, and flags to legal when a new use case would push it toward high-risk. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Classifies a domain against the applicable risk framework, keeps its evidence pack (evals, controls, incidents) audit-ready, converts findings into engineering requirements with owners, and flags when a product change alters the risk class.
+Evidenced by: Classifies the support-triage capability as limited-risk under the applicable framework, keeps its eval and incident log current for the quarterly audit, and flags to legal when a new use case would push it toward high-risk.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Operates a cross-team AI risk-review process - fast enough that teams use it honestly, rigorous enough to catch real issues - and builds governance tooling that makes compliance a byproduct of normal engineering. Evidenced by: Runs the weekly cross-team risk-review that every AI launch across four teams goes through, and ships the CI check that blocks a PR missing a risk classification before a human has to catch it. Scope: multiple teams.</t>
+          <t>Depth: Operates a cross-team AI risk-review process - fast enough that teams use it honestly, rigorous enough to catch real issues - and builds governance tooling that makes compliance a byproduct of normal engineering.
+Evidenced by: Runs the weekly cross-team risk-review that every AI launch across four teams goes through, and ships the CI check that blocks a PR missing a risk classification before a human has to catch it.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns an organization's AI governance program jointly with legal and risk functions, translating regulation into engineering requirements without freezing delivery. Evidenced by: Co-owns the org's AI governance program with legal, turning a new regulation's high-risk-system obligations into a pre-launch checklist that ships features on schedule instead of stalling in review. Scope: organization.</t>
+          <t>Depth: Owns an organization's AI governance program jointly with legal and risk functions, translating regulation into engineering requirements without freezing delivery.
+Evidenced by: Co-owns the org's AI governance program with legal, turning a new regulation's high-risk-system obligations into a pre-launch checklist that ships features on schedule instead of stalling in review.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L34" s="4" t="inlineStr">
         <is>
-          <t>Depth: Positions a company ahead of AI regulation; accountable to executives, boards, and regulators for where the risk lines are drawn. Evidenced by: Briefs the board on where the company draws its AI risk lines before a regulator asks, and represents the company's position in an industry working group shaping upcoming AI-regulation guidance. Scope: company.</t>
+          <t>Depth: Positions a company ahead of AI regulation; accountable to executives, boards, and regulators for where the risk lines are drawn.
+Evidenced by: Briefs the board on where the company draws its AI risk lines before a regulator asks, and represents the company's position in an industry working group shaping upcoming AI-regulation guidance.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2854,32 +3250,44 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Translates a clearly scoped problem into a defined ML task under guidance. Evidenced by: States what user problem their task serves and raises it when a lookup table or heuristic would do what the ticket asks of a model. Scope: task.</t>
+          <t>Depth: Translates a clearly scoped problem into a defined ML task under guidance.
+Evidenced by: States what user problem their task serves and raises it when a lookup table or heuristic would do what the ticket asks of a model.
+Scope: task.</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Frames routine problems as appropriate ML solutions independently. Evidenced by: Prototypes the simplest adequate approach first — rules, search, classical ML, or a model — and recommends the model only when it beats the baseline, with the comparison documented. Scope: component.</t>
+          <t>Depth: Frames routine problems as appropriate ML solutions independently.
+Evidenced by: Prototypes the simplest adequate approach first — rules, search, classical ML, or a model — and recommends the model only when it beats the baseline, with the comparison documented.
+Scope: component.</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Frames ambiguous business problems into sound ML or non-ML approaches autonomously. Evidenced by: Kills LLM-shaped solutions to non-LLM problems in design review with evidence, reframing vague 'add AI' asks into testable user outcomes product partners agree to. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Frames ambiguous business problems into sound ML or non-ML approaches autonomously.
+Evidenced by: Kills LLM-shaped solutions to non-LLM problems in design review with evidence, reframing vague 'add AI' asks into testable user outcomes product partners agree to.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines solution-design patterns others adopt and reframes intractable problems. Evidenced by: Installs solution-fit review in how multiple teams take on AI work, redirecting AI-for-its-own-sake proposals and unwinding the most expensive misfit projects. Scope: multiple teams.</t>
+          <t>Depth: Defines solution-design patterns others adopt and reframes intractable problems.
+Evidenced by: Installs solution-fit review in how multiple teams take on AI work, redirecting AI-for-its-own-sake proposals and unwinding the most expensive misfit projects.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets ML solution strategy and anticipates where applicable techniques are heading. Evidenced by: Shapes which problems the org points AI at, pairing with product leadership on where models genuinely change the offering and cancelling bets the evidence turns against. Scope: organization.</t>
+          <t>Depth: Sets ML solution strategy and anticipates where applicable techniques are heading.
+Evidenced by: Shapes which problems the org points AI at, pairing with product leadership on where models genuinely change the offering and cancelling bets the evidence turns against.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines best practice for ML problem framing across the discipline and is externally recognized. Evidenced by: Advises company leadership on what AI makes newly possible versus fashionable — and is right often enough to be believed. Scope: company.</t>
+          <t>Depth: Defines best practice for ML problem framing across the discipline and is externally recognized.
+Evidenced by: Advises company leadership on what AI makes newly possible versus fashionable — and is right often enough to be believed.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2916,32 +3324,44 @@
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Understands the capability they're building and who uses it. Evidenced by: States how their feature's success will be measured beyond 'it works' and checks the metric after launch rather than moving on. Scope: task.</t>
+          <t>Depth: Understands the capability they're building and who uses it.
+Evidenced by: States how their feature's success will be measured beyond 'it works' and checks the metric after launch rather than moving on.
+Scope: task.</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Frames own work in user/business outcomes, not just tasks. Evidenced by: Defines success metrics with product partners before building and reports post-launch results honestly, including misses. Scope: component.</t>
+          <t>Depth: Frames own work in user/business outcomes, not just tasks.
+Evidenced by: Defines success metrics with product partners before building and reports post-launch results honestly, including misses.
+Scope: component.</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Treats their area as a product; uses metrics to decide what to build for a domain. Evidenced by: Connects a capability's engineering metrics to business outcomes — cost per outcome, retention, task completion — and recommends sunsetting features whose value evidence never arrives. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Treats their area as a product; uses metrics to decide what to build for a domain.
+Evidenced by: Connects a capability's engineering metrics to business outcomes — cost per outcome, retention, task completion — and recommends sunsetting features whose value evidence never arrives.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert at aligning technical bets with product strategy across teams. Evidenced by: Builds the value-measurement discipline multiple teams use for AI investments, surfacing which bets are and aren't paying off. Scope: multiple teams.</t>
+          <t>Depth: Expert at aligning technical bets with product strategy across teams.
+Evidenced by: Builds the value-measurement discipline multiple teams use for AI investments, surfacing which bets are and aren't paying off.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets product direction for an org's technical surface. Evidenced by: Owns the org's account of AI value delivered, credible to finance and product alike, and reallocates engineering toward what the evidence supports. Scope: organization.</t>
+          <t>Depth: Sets product direction for an org's technical surface.
+Evidenced by: Owns the org's account of AI value delivered, credible to finance and product alike, and reallocates engineering toward what the evidence supports.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes how the company creates value through technical products. Evidenced by: Shapes how the company invests in AI based on demonstrated value, with numbers that survive diligence at board level. Scope: company.</t>
+          <t>Depth: Shapes how the company creates value through technical products.
+Evidenced by: Shapes how the company invests in AI based on demonstrated value, with numbers that survive diligence at board level.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -2978,32 +3398,44 @@
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Learns to estimate; surfaces blockers; plans own tasks with guidance. Evidenced by: Breaks their work into small verifiable increments and flags early — with evidence — when the model can't do what the task assumed, instead of grinding silently. Scope: task.</t>
+          <t>Depth: Learns to estimate; surfaces blockers; plans own tasks with guidance.
+Evidenced by: Breaks their work into small verifiable increments and flags early — with evidence — when the model can't do what the task assumed, instead of grinding silently.
+Scope: task.</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Estimates scoped work realistically; plans own 1-3 week projects. Evidenced by: Plans feature work as a de-risking sequence — timeboxed feasibility spike, eval baseline, then build — giving estimates as ranges with stated confidence. Scope: component.</t>
+          <t>Depth: Estimates scoped work realistically; plans own 1-3 week projects.
+Evidenced by: Plans feature work as a de-risking sequence — timeboxed feasibility spike, eval baseline, then build — giving estimates as ranges with stated confidence.
+Scope: component.</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Plans quarter-scale, multi-workstream efforts including dependencies. Evidenced by: Structures a capability's roadmap around its riskiest unknowns — feasibility gates before commitments, kill criteria stated before the spike starts and honored when triggered. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Plans quarter-scale, multi-workstream efforts including dependencies.
+Evidenced by: Structures a capability's roadmap around its riskiest unknowns — feasibility gates before commitments, kill criteria stated before the spike starts and honored when triggered.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert at planning large programs; anticipates risk early. Evidenced by: Teaches teams to plan AI work honestly — separating engineering certainty from model uncertainty in commitments leaders can rely on — and de-risks the org's biggest AI commitments personally. Scope: multiple teams.</t>
+          <t>Depth: Expert at planning large programs; anticipates risk early.
+Evidenced by: Teaches teams to plan AI work honestly — separating engineering certainty from model uncertainty in commitments leaders can rely on — and de-risks the org's biggest AI commitments personally.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Plans org-level programs across quarters/years. Evidenced by: Shapes the org's portfolio of AI bets, balancing near-certain delivery against high-variance exploration and keeping leadership expectations calibrated to what evals actually show. Scope: organization.</t>
+          <t>Depth: Plans org-level programs across quarters/years.
+Evidenced by: Shapes the org's portfolio of AI bets, balancing near-certain delivery against high-variance exploration and keeping leadership expectations calibrated to what evals actually show.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes how the company plans major technical change. Evidenced by: Times company bets against the model-capability curve — what to build now versus wait for — and is accountable for the calls. Scope: company.</t>
+          <t>Depth: Shapes how the company plans major technical change.
+Evidenced by: Times company bets against the model-capability curve — what to build now versus wait for — and is accountable for the calls.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -3040,32 +3472,44 @@
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Follows the release process exactly — flags, staged rollout steps, verification checklists — verifies their change in production, and rolls back with guidance. Evidenced by: Ships work in small reviewable increments behind flags as directed and rolls back their own change cleanly when asked. Scope: task.</t>
+          <t>Depth: Follows the release process exactly — flags, staged rollout steps, verification checklists — verifies their change in production, and rolls back with guidance.
+Evidenced by: Ships work in small reviewable increments behind flags as directed and rolls back their own change cleanly when asked.
+Scope: task.</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Ships behind flags with a rollback plan by default, monitors rollouts and reverts on their own judgment when signals degrade, and writes changes that tolerate both versions running during rollout. Evidenced by: Designs a component's rollout as canary -&gt; percentage -&gt; full, watching evals and telemetry at each stage and rolling back on their own signal. Scope: component.</t>
+          <t>Depth: Ships behind flags with a rollback plan by default, monitors rollouts and reverts on their own judgment when signals degrade, and writes changes that tolerate both versions running during rollout.
+Evidenced by: Designs a component's rollout as canary -&gt; percentage -&gt; full, watching evals and telemetry at each stage and rolling back on their own signal.
+Scope: component.</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Designs the rollout for risky changes — canary criteria, migration sequencing, flag lifecycle, kill switches — and reviews others' rollout plans for blast radius; the person teams ask how to ship something safely. Evidenced by: Owns progressive-delivery strategy for a capability — shadow modes for new models, reversible-by-design changes, automated rollback triggers — and their launches are uneventful. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Designs the rollout for risky changes — canary criteria, migration sequencing, flag lifecycle, kill switches — and reviews others' rollout plans for blast radius; the person teams ask how to ship something safely.
+Evidenced by: Owns progressive-delivery strategy for a capability — shadow modes for new models, reversible-by-design changes, automated rollback triggers — and their launches are uneventful.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds progressive-delivery machinery multiple teams release through (flag platforms, automated canary analysis, automated rollback), retiring deploy patterns that cause repeat incidents and measurably raising deploy frequency. Evidenced by: Builds the progressive-delivery machinery multiple teams use for AI changes — flag conventions, automated rollback on eval regression. Scope: multiple teams.</t>
+          <t>Depth: Builds progressive-delivery machinery multiple teams release through (flag platforms, automated canary analysis, automated rollback), retiring deploy patterns that cause repeat incidents and measurably raising deploy frequency.
+Evidenced by: Builds the progressive-delivery machinery multiple teams use for AI changes — flag conventions, automated rollback on eval regression.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns release policy for an organization and its delivery metrics — rollout standards, freeze rules, environment strategy — dismantling ceremony that adds no safety. Evidenced by: Sets the org's release-engineering direction for AI products and its risk appetite per surface. Scope: organization.</t>
+          <t>Depth: Owns release policy for an organization and its delivery metrics — rollout standards, freeze rules, environment strategy — dismantling ceremony that adds no safety.
+Evidenced by: Sets the org's release-engineering direction for AI products and its risk appetite per surface.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets how an entire company's software reaches customers — the risk posture products ship under — and defends it to executives, auditors, and regulators. Evidenced by: Makes safe iteration speed a company capability competitors can't easily copy. Scope: company.</t>
+          <t>Depth: Sets how an entire company's software reaches customers — the risk posture products ship under — and defends it to executives, auditors, and regulators.
+Evidenced by: Makes safe iteration speed a company capability competitors can't easily copy.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -3102,32 +3546,44 @@
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Takes ownership of assigned tasks; honest about progress and blockers. Evidenced by: Tells their lead two days early that the eval-harness ticket will slip because the golden dataset isn't ready, instead of going quiet until standup. Scope: task.</t>
+          <t>Depth: Takes ownership of assigned tasks; honest about progress and blockers.
+Evidenced by: Tells their lead two days early that the eval-harness ticket will slip because the golden dataset isn't ready, instead of going quiet until standup.
+Scope: task.</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns components end-to-end; delivers committed work reliably. Evidenced by: Delivers the retrieval-reranking component on the date they committed to, having flagged and absorbed a provider API change mid-sprint without missing the deadline. Scope: component.</t>
+          <t>Depth: Owns components end-to-end; delivers committed work reliably.
+Evidenced by: Delivers the retrieval-reranking component on the date they committed to, having flagged and absorbed a provider API change mid-sprint without missing the deadline.
+Scope: component.</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns a domain; lands multi-week efforts without surprises; pushes back on unrealistic scope with reasons. Evidenced by: Owns the chatbot capability through a six-week model migration with no surprise regressions, and talks product out of a two-week scope add with a written cost estimate. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Owns a domain; lands multi-week efforts without surprises; pushes back on unrealistic scope with reasons.
+Evidenced by: Owns the chatbot capability through a six-week model migration with no surprise regressions, and talks product out of a two-week scope add with a written cost estimate.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns cross-team initiatives; unblocks teams; kills failing approaches early. Evidenced by: Runs the cross-team migration off the deprecated embedding model, unblocking two teams stuck on the same provider quota issue and cutting a doomed fine-tuning effort before it burns another sprint. Scope: multiple teams.</t>
+          <t>Depth: Owns cross-team initiatives; unblocks teams; kills failing approaches early.
+Evidenced by: Runs the cross-team migration off the deprecated embedding model, unblocking two teams stuck on the same provider quota issue and cutting a doomed fine-tuning effort before it burns another sprint.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>Depth: Owns an org-level portfolio of bets; sets direction others follow. Evidenced by: Owns the org's portfolio of AI reliability bets for the year, and three other teams plan their roadmaps around the sequencing they set. Scope: organization.</t>
+          <t>Depth: Owns an org-level portfolio of bets; sets direction others follow.
+Evidenced by: Owns the org's portfolio of AI reliability bets for the year, and three other teams plan their roadmaps around the sequencing they set.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>Depth: The go-to when something company-critical must land. Evidenced by: Is who leadership calls in when the flagship AI feature's launch is at risk two weeks out, and lands it. Scope: company.</t>
+          <t>Depth: The go-to when something company-critical must land.
+Evidenced by: Is who leadership calls in when the flagship AI feature's launch is at risk two weeks out, and lands it.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -3164,32 +3620,44 @@
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Communicates status clearly; documentation is accurate. Evidenced by: Writes clear task updates, commit messages, and questions with enough context that responders don't have to ask for it, summarizing eval results without overstating them. Scope: task.</t>
+          <t>Depth: Communicates status clearly; documentation is accurate.
+Evidenced by: Writes clear task updates, commit messages, and questions with enough context that responders don't have to ask for it, summarizing eval results without overstating them.
+Scope: task.</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes clear design notes, runbooks and PRs; explains trade-offs without overselling. Evidenced by: Writes design notes and runbooks peers act on without follow-up questions, and explains model behavior and its limits to non-experts without jargon or overclaiming. Scope: component.</t>
+          <t>Depth: Writes clear design notes, runbooks and PRs; explains trade-offs without overselling.
+Evidenced by: Writes design notes and runbooks peers act on without follow-up questions, and explains model behavior and its limits to non-experts without jargon or overclaiming.
+Scope: component.</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Writes design docs that drive decisions; translates technical risk for non-technical stakeholders. Evidenced by: Writes the docs that settle decisions and translates eval results and AI trade-offs so accurately that product decisions built on their word hold up. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Writes design docs that drive decisions; translates technical risk for non-technical stakeholders.
+Evidenced by: Writes the docs that settle decisions and translates eval results and AI trade-offs so accurately that product decisions built on their word hold up.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert at making complex capability/risk legible to executives without dumbing it down; RFCs align orgs. Evidenced by: Aligns multiple teams through writing — RFCs, strategies, decision records cited months later as the reference — and presents AI capability and risk to leadership without dumbing it down. Scope: multiple teams.</t>
+          <t>Depth: Expert at making complex capability/risk legible to executives without dumbing it down; RFCs align orgs.
+Evidenced by: Aligns multiple teams through writing — RFCs, strategies, decision records cited months later as the reference — and presents AI capability and risk to leadership without dumbing it down.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
-          <t>Depth: Strategy memos leadership acts on; org-wide and external reach. Evidenced by: Communicates org-level technical direction upward and outward, translating between executive and engineering registers without loss, including bad news early. Scope: organization.</t>
+          <t>Depth: Strategy memos leadership acts on; org-wide and external reach.
+Evidenced by: Communicates org-level technical direction upward and outward, translating between executive and engineering registers without loss, including bad news early.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L40" s="4" t="inlineStr">
         <is>
-          <t>Depth: A clarifying voice at company scale; externally recognized. Evidenced by: Is the company's technical voice on AI internally and externally — talks, publications, customer and regulator conversations that move the company's position. Scope: company.</t>
+          <t>Depth: A clarifying voice at company scale; externally recognized.
+Evidenced by: Is the company's technical voice on AI internally and externally — talks, publications, customer and regulator conversations that move the company's position.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -3226,32 +3694,44 @@
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Responsive to feedback; pairs willingly; asks for help appropriately. Evidenced by: Works effectively with designer and PM counterparts on task details, surfacing AI-specific constraints — latency, failure modes — early, and incorporates feedback without churn. Scope: task.</t>
+          <t>Depth: Responsive to feedback; pairs willingly; asks for help appropriately.
+Evidenced by: Works effectively with designer and PM counterparts on task details, surfacing AI-specific constraints — latency, failure modes — early, and incorporates feedback without churn.
+Scope: task.</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Collaborates smoothly with adjacent functions; handles disagreement constructively. Evidenced by: Partners with product and design on what the model can and can't support, involving them before the prompt is final and prototyping to resolve disagreements with evidence. Scope: component.</t>
+          <t>Depth: Collaborates smoothly with adjacent functions; handles disagreement constructively.
+Evidenced by: Partners with product and design on what the model can and can't support, involving them before the prompt is final and prototyping to resolve disagreements with evidence.
+Scope: component.</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds strong cross-team relationships; resolves friction directly. Evidenced by: Runs the cross-functional process for a capability — brings legal, security, and support in before launch, turns product intent into evaluable requirements — and resolves conflicts between functions without escalation. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Builds strong cross-team relationships; resolves friction directly.
+Evidenced by: Runs the cross-functional process for a capability — brings legal, security, and support in before launch, turns product intent into evaluable requirements — and resolves conflicts between functions without escalation.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Expert at aligning teams with competing priorities; mediates disputes between senior people. Evidenced by: Fixes broken cross-team interfaces — ownership gaps, handoff friction — building the review forums, interface agreements, and shared vocabularies several teams use. Scope: multiple teams.</t>
+          <t>Depth: Expert at aligning teams with competing priorities; mediates disputes between senior people.
+Evidenced by: Fixes broken cross-team interfaces — ownership gaps, handoff friction — building the review forums, interface agreements, and shared vocabularies several teams use.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Creates the forums and processes through which collaboration happens. Evidenced by: Builds the org's operating model between AI engineering and other functions — data, platform, trust, product — so work flows without heroics. Scope: organization.</t>
+          <t>Depth: Creates the forums and processes through which collaboration happens.
+Evidenced by: Builds the org's operating model between AI engineering and other functions — data, platform, trust, product — so work flows without heroics.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L41" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds coalitions at company scale and externally. Evidenced by: Brokers company-level alignment on AI initiatives across executive functions with durable results. Scope: company.</t>
+          <t>Depth: Builds coalitions at company scale and externally.
+Evidenced by: Brokers company-level alignment on AI initiatives across executive functions with durable results.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -3288,32 +3768,44 @@
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shares what they learn; keeps their docs accurate. Evidenced by: Keeps the docs for what they build current — setup, known limits, gotchas — and files gaps they find in others'. Scope: task.</t>
+          <t>Depth: Shares what they learn; keeps their docs accurate.
+Evidenced by: Keeps the docs for what they build current — setup, known limits, gotchas — and files gaps they find in others'.
+Scope: task.</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Documents their area well; proactively shares techniques with the team. Evidenced by: Documents a feature's behavior contract — intended use, eval results, failure modes, escalation paths — findable by the next engineer without asking. Scope: component.</t>
+          <t>Depth: Documents their area well; proactively shares techniques with the team.
+Evidenced by: Documents a feature's behavior contract — intended use, eval results, failure modes, escalation paths — findable by the next engineer without asking.
+Scope: component.</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Creates documentation and forums that raise a whole domain's understanding. Evidenced by: Maintains the canonical documentation for a capability — architecture, prompt rationale, eval history, runbooks — and prunes stale docs as ruthlessly as stale code. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Creates documentation and forums that raise a whole domain's understanding.
+Evidenced by: Maintains the canonical documentation for a capability — architecture, prompt rationale, eval history, runbooks — and prunes stale docs as ruthlessly as stale code.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Builds knowledge-sharing systems adopted across teams. Evidenced by: Drives documentation standards for AI systems across teams — behavior cards, decision records — and reviews for compliance. Scope: multiple teams.</t>
+          <t>Depth: Builds knowledge-sharing systems adopted across teams.
+Evidenced by: Drives documentation standards for AI systems across teams — behavior cards, decision records — and reviews for compliance.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Defines how the org captures and spreads knowledge. Evidenced by: Builds the org's AI knowledge base as infrastructure, making internal expertise discoverable. Scope: organization.</t>
+          <t>Depth: Defines how the org captures and spreads knowledge.
+Evidenced by: Builds the org's AI knowledge base as infrastructure, making internal expertise discoverable.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes industry-facing knowledge practice. Evidenced by: Externalizes company knowledge deliberately — publications, standards participation — where it compounds the company's position. Scope: company.</t>
+          <t>Depth: Shapes industry-facing knowledge practice.
+Evidenced by: Externalizes company knowledge deliberately — publications, standards participation — where it compounds the company's position.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -3350,32 +3842,44 @@
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Receptive to mentoring; shares what they learn. Evidenced by: Asks for help effectively and pays it forward, documenting what they learned where the next person will find it. Scope: task.</t>
+          <t>Depth: Receptive to mentoring; shares what they learn.
+Evidenced by: Asks for help effectively and pays it forward, documenting what they learned where the next person will find it.
+Scope: task.</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Helps onboard teammates; informally mentors juniors. Evidenced by: Onboards new teammates onto the AI stack and pairs generously, turning their own review comments and repeated questions into reusable explanations. Scope: component.</t>
+          <t>Depth: Helps onboard teammates; informally mentors juniors.
+Evidenced by: Onboards new teammates onto the AI stack and pairs generously, turning their own review comments and repeated questions into reusable explanations.
+Scope: component.</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Coaches engineers with growth-oriented feedback; measurably improves a team's skill. Evidenced by: Mentors engineers deliberately — stretch tasks matched to gaps, feedback that names behavior and impact — and levels a team up on AI-specific craft it didn't have before; mentees ship independently sooner. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Coaches engineers with growth-oriented feedback; measurably improves a team's skill.
+Evidenced by: Mentors engineers deliberately — stretch tasks matched to gaps, feedback that names behavior and impact — and levels a team up on AI-specific craft it didn't have before; mentees ship independently sooner.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Develops future leads across teams; shapes hiring and onboarding. Evidenced by: Grows senior engineers across teams, sponsoring others into leading work they would have led, and builds the guilds and curricula that scale beyond one-on-ones. Scope: multiple teams.</t>
+          <t>Depth: Develops future leads across teams; shapes hiring and onboarding.
+Evidenced by: Grows senior engineers across teams, sponsoring others into leading work they would have led, and builds the guilds and curricula that scale beyond one-on-ones.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Develops senior engineers and leaders; builds culture deliberately. Evidenced by: Builds the org's AI-engineering bench — hiring bar, growth paths, promotion evidence, succession for critical systems. Scope: organization.</t>
+          <t>Depth: Develops senior engineers and leaders; builds culture deliberately.
+Evidenced by: Builds the org's AI-engineering bench — hiring bar, growth paths, promotion evidence, succession for critical systems.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Depth: Develops the next generation of top talent; legacy outlasts tenure. Evidenced by: Develops the company's next generation of principal-level technical leaders, largely through others, and shapes how the company is known to candidates. Scope: company.</t>
+          <t>Depth: Develops the next generation of top talent; legacy outlasts tenure.
+Evidenced by: Develops the company's next generation of principal-level technical leaders, largely through others, and shapes how the company is known to candidates.
+Scope: company.</t>
         </is>
       </c>
     </row>
@@ -3412,32 +3916,44 @@
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Contributes informed opinions in technical discussions. Evidenced by: Volunteers for unglamorous work that unblocks others and raises risks early instead of waiting to be asked. Scope: task.</t>
+          <t>Depth: Contributes informed opinions in technical discussions.
+Evidenced by: Volunteers for unglamorous work that unblocks others and raises risks early instead of waiting to be asked.
+Scope: task.</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Influences component-level decisions through credibility. Evidenced by: Leads small technical efforts end to end — a migration, an integration — coordinating the people involved without formal authority or escalation. Scope: component.</t>
+          <t>Depth: Influences component-level decisions through credibility.
+Evidenced by: Leads small technical efforts end to end — a migration, an integration — coordinating the people involved without formal authority or escalation.
+Scope: component.</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Sets technical direction for a domain; others align to their calls. Evidenced by: Sets technical direction for a capability — making and documenting the contentious calls, taking responsibility when wrong — and is the engineer others seek out when an AI decision is stuck. Scope: capability / domain (terminal level).</t>
+          <t>Depth: Sets technical direction for a domain; others align to their calls.
+Evidenced by: Sets technical direction for a capability — making and documenting the contentious calls, taking responsibility when wrong — and is the engineer others seek out when an AI decision is stuck.
+Scope: capability / domain (terminal level).</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Shapes how multiple teams approach problems; trusted tiebreaker. Evidenced by: Creates alignment across teams that don't report to them, landing multi-team initiatives — platform migrations, model transitions — through writing, relationships, and demonstrated judgment. Scope: multiple teams.</t>
+          <t>Depth: Shapes how multiple teams approach problems; trusted tiebreaker.
+Evidenced by: Creates alignment across teams that don't report to them, landing multi-team initiatives — platform migrations, model transitions — through writing, relationships, and demonstrated judgment.
+Scope: multiple teams.</t>
         </is>
       </c>
       <c r="K44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Influences org-wide technical strategy. Evidenced by: Drives the org's technical strategy for AI, choosing the few bets that matter and getting leadership and teams genuinely behind them. Scope: organization.</t>
+          <t>Depth: Influences org-wide technical strategy.
+Evidenced by: Drives the org's technical strategy for AI, choosing the few bets that matter and getting leadership and teams genuinely behind them.
+Scope: organization.</t>
         </is>
       </c>
       <c r="L44" s="4" t="inlineStr">
         <is>
-          <t>Depth: Influences company strategic direction through insight. Evidenced by: Sets the company's long-term technical direction for AI, accountable for the bets years before they resolve. Scope: company.</t>
+          <t>Depth: Influences company strategic direction through insight.
+Evidenced by: Sets the company's long-term technical direction for AI, accountable for the bets years before they resolve.
+Scope: company.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(render): drop redundant scope clause from cells
</commit_message>
<xml_diff>
--- a/roles/ai-engineer/ladder.xlsx
+++ b/roles/ai-engineer/ladder.xlsx
@@ -809,43 +809,37 @@
       <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Depth: Implements designs specified by others; asks why, not just how.
-Evidenced by: Explains the system's architecture in their own words.
-Scope: task.</t>
+Evidenced by: Explains the system's architecture in their own words.</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs sound components; understands coupling, cohesion, interface design.
-Evidenced by: Designs a component and writes the short design note for it.
-Scope: component.</t>
+Evidenced by: Designs a component and writes the short design note for it.</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs systems for evolution: clean seams, versioned interfaces, replaceable parts.
-Evidenced by: Selects patterns by trade-off in design docs that name the alternatives and failure modes.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Selects patterns by trade-off in design docs that name the alternatives and failure modes.</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
           <t>Depth: Mastery of architecture for complex systems; sets patterns and prevents drift.
-Evidenced by: Writes the reference architectures other teams instantiate.
-Scope: multiple teams.</t>
+Evidenced by: Writes the reference architectures other teams instantiate.</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets multi-year architecture direction across the org.
-Evidenced by: Sets the architectural direction for AI systems across the org.
-Scope: organization.</t>
+Evidenced by: Sets the architectural direction for AI systems across the org.</t>
         </is>
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
           <t>Depth: Authoritative and externally credible; defines architectural approach others follow.
-Evidenced by: Defines the company's long-horizon technical bets for AI systems.
-Scope: company.</t>
+Evidenced by: Defines the company's long-horizon technical bets for AI systems.</t>
         </is>
       </c>
     </row>
@@ -883,43 +877,37 @@
       <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands HTTP/REST and the deploy pipeline; makes guided changes.
-Evidenced by: Implements endpoints to an existing API contract, including error responses, and flags mismatches between spec and behavior.
-Scope: task.</t>
+Evidenced by: Implements endpoints to an existing API contract, including error responses, and flags mismatches between spec and behavior.</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs clean APIs; understands rate limits, retries, timeouts, idempotency.
-Evidenced by: Designs the API surface for a component and documents it well enough that a consumer needs no walkthrough.
-Scope: component.</t>
+Evidenced by: Designs the API surface for a component and documents it well enough that a consumer needs no walkthrough.</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs services for scale and cost; understands distributed failure modes.
-Evidenced by: Designs contracts that isolate consumers from model and provider changes and rejects designs that leak provider details to callers.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Designs contracts that isolate consumers from model and provider changes and rejects designs that leak provider details to callers.</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in platform/service design (multi-tenancy, capacity, shared services).
-Evidenced by: Sets the API conventions multiple teams follow for model-backed services and retires inconsistent legacy surfaces with migration paths.
-Scope: multiple teams.</t>
+Evidenced by: Sets the API conventions multiple teams follow for model-backed services and retires inconsistent legacy surfaces with migration paths.</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets interface standards used across the org.
-Evidenced by: Drives the org's interface strategy — which capabilities become shared platforms, and the deprecation policy that keeps the surface coherent.
-Scope: organization.</t>
+Evidenced by: Drives the org's interface strategy — which capabilities become shared platforms, and the deprecation policy that keeps the surface coherent.</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines company-wide API approach; trusted with irreversible interface bets.
-Evidenced by: Shapes the company's external and partner-facing AI interfaces, balancing product commitments against provider volatility.
-Scope: company.</t>
+Evidenced by: Shapes the company's external and partner-facing AI interfaces, balancing product commitments against provider volatility.</t>
         </is>
       </c>
     </row>
@@ -957,43 +945,37 @@
       <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Depth: Writes working, readable code in the team's language; debugs own changes.
-Evidenced by: Implements the retry-with-backoff helper for a flaky provider call exactly to spec and finds the off-by-one in their own token-counting logic before it reaches review.
-Scope: task.</t>
+Evidenced by: Implements the retry-with-backoff helper for a flaky provider call exactly to spec and finds the off-by-one in their own token-counting logic before it reaches review.</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Depth: Proficient in the primary language/ecosystem; handles errors, async and concurrency basics correctly.
-Evidenced by: Ships the async job that reprocesses failed embedding batches, handling partial-batch failures and concurrent writes to the vector store without a teammate having to point them out.
-Scope: component.</t>
+Evidenced by: Ships the async job that reprocesses failed embedding batches, handling partial-batch failures and concurrent writes to the vector store without a teammate having to point them out.</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Depth: Code is a reference others learn from; debugs the hard problems (races, memory, nondeterminism).
-Evidenced by: Writes the concurrent request-batching code newer engineers copy verbatim, and is the one who finds the race condition in the streaming-response handler that only shows up under load.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Writes the concurrent request-batching code newer engineers copy verbatim, and is the one who finds the race condition in the streaming-response handler that only shows up under load.</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Depth: Mastery across multiple stacks/paradigms; solves problems others can't; sets implementation patterns.
-Evidenced by: Rewrites the team's Python retrieval service in Rust for a client with different concurrency guarantees, solving a memory-pressure bug in the vector index that stumped two other engineers.
-Scope: multiple teams.</t>
+Evidenced by: Rewrites the team's Python retrieval service in Rust for a client with different concurrency guarantees, solving a memory-pressure bug in the vector index that stumped two other engineers.</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets implementation standards adopted across the org; anticipates where code breaks at scale.
-Evidenced by: Sets the org's async-error-handling convention after a postmortem shows three teams' AI services failed the same way under provider timeout spikes.
-Scope: organization.</t>
+Evidenced by: Sets the org's async-error-handling convention after a postmortem shows three teams' AI services failed the same way under provider timeout spikes.</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Depth: Industry-level depth; authors foundational primitives and idioms others build on.
-Evidenced by: Writes the request-batching primitive now vendored into every AI service's client library company-wide, the reference implementation new hires study.
-Scope: company.</t>
+Evidenced by: Writes the request-batching primitive now vendored into every AI service's client library company-wide, the reference implementation new hires study.</t>
         </is>
       </c>
     </row>
@@ -1031,43 +1013,37 @@
       <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Depth: Writes functional, readable code; uses version control correctly; responds well to review.
-Evidenced by: Submits small, reviewable changes that pass CI first try more often than not and responds to review feedback by fixing the pattern, not just the line.
-Scope: task.</t>
+Evidenced by: Submits small, reviewable changes that pass CI first try more often than not and responds to review feedback by fixing the pattern, not just the line.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Depth: Writes clean, documented, modular code; gives useful review feedback.
-Evidenced by: Reviews peers' changes with substantive comments and keeps the code they touch consistently readable.
-Scope: component.</t>
+Evidenced by: Reviews peers' changes with substantive comments and keeps the code they touch consistently readable.</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs for maintainability; leads refactors of problem areas; review feedback teaches.
-Evidenced by: Holds the quality bar in review for a whole domain, including AI-generated code, articulating why a change is risky rather than just that it is.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Holds the quality bar in review for a whole domain, including AI-generated code, articulating why a change is risky rather than just that it is.</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in code health at scale (shared libraries, deprecations, large migrations).
-Evidenced by: Codifies review and code-health standards multiple teams adopt and measurably reduces defect escape in the areas they steward.
-Scope: multiple teams.</t>
+Evidenced by: Codifies review and code-health standards multiple teams adopt and measurably reduces defect escape in the areas they steward.</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Depth: Shapes org-wide engineering standards for long-lived codebases.
-Evidenced by: Changes how the org reviews and maintains code — tooling, norms, and the standards for machine-authored changes.
-Scope: organization.</t>
+Evidenced by: Changes how the org reviews and maintains code — tooling, norms, and the standards for machine-authored changes.</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines what good engineering looks like company-wide; externally recognized.
-Evidenced by: Sets the company's engineering quality bar, cited when quality trade-offs reach executive decisions.
-Scope: company.</t>
+Evidenced by: Sets the company's engineering quality bar, cited when quality trade-offs reach executive decisions.</t>
         </is>
       </c>
     </row>
@@ -1105,43 +1081,37 @@
       <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Depth: Debugs issues in own code with support; uses basic tooling.
-Evidenced by: Reproduces a reported bug and bisects it to a candidate cause with guidance, reading logs and stack traces before asking for help.
-Scope: task.</t>
+Evidenced by: Reproduces a reported bug and bisects it to a candidate cause with guidance, reading logs and stack traces before asking for help.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
           <t>Depth: Independently diagnoses defects in own area systematically.
-Evidenced by: Isolates faults across service boundaries unaided, distinguishing deterministic code bugs from model-behavior variance before escalating.
-Scope: component.</t>
+Evidenced by: Isolates faults across service boundaries unaided, distinguishing deterministic code bugs from model-behavior variance before escalating.</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Depth: Leads diagnosis of hard, cross-cutting failures; root cause not symptoms.
-Evidenced by: Debugs the hardest failures in a capability, including intermittent model-dependent ones, and writes the reproduction others rerun.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Debugs the hardest failures in a capability, including intermittent model-dependent ones, and writes the reproduction others rerun.</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert at the rare/systemic failures; builds tooling that makes them visible.
-Evidenced by: Untangles cross-team failures where no single owner sees the whole path and leaves behind the instrumentation that makes the next one cheap.
-Scope: multiple teams.</t>
+Evidenced by: Untangles cross-team failures where no single owner sees the whole path and leaves behind the instrumentation that makes the next one cheap.</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Depth: The person called for the worst failures; sets diagnostic practice org-wide.
-Evidenced by: Spots systemic failure classes from incident patterns across the org and drives the architectural fixes.
-Scope: organization.</t>
+Evidenced by: Spots systemic failure classes from incident patterns across the org and drives the architectural fixes.</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
           <t>Depth: Authority on diagnosis; advances the discipline.
-Evidenced by: Is the debugger of last resort for company-critical AI incidents and turns each into a durable prevention mechanism.
-Scope: company.</t>
+Evidenced by: Is the debugger of last resort for company-critical AI incidents and turns each into a durable prevention mechanism.</t>
         </is>
       </c>
     </row>
@@ -1179,43 +1149,37 @@
       <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Depth: Writes unit tests with guidance; tests own changes before merging.
-Evidenced by: Writes unit tests for the deterministic parts of a change and can say which behaviors are testable versus eval-able when asked.
-Scope: task.</t>
+Evidenced by: Writes unit tests for the deterministic parts of a change and can say which behaviors are testable versus eval-able when asked.</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Depth: Applies the testing pyramid; everything shipped arrives tested; mocks dependencies sensibly.
-Evidenced by: Draws the test/eval boundary correctly for a component and keeps CI fast and free of flaky model-dependent assertions.
-Scope: component.</t>
+Evidenced by: Draws the test/eval boundary correctly for a component and keeps CI fast and free of flaky model-dependent assertions.</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs testable systems (contract, property-based, replay from prod); owns a test strategy.
-Evidenced by: Designs the verification strategy for a capability and rejects flaky model-in-the-loop tests in review with a stated rule.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Designs the verification strategy for a capability and rejects flaky model-in-the-loop tests in review with a stated rule.</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in test strategy at scale (test data, environments, deployment safety).
-Evidenced by: Standardizes the test-vs-eval discipline across teams with shared fixtures, replay harnesses, and CI policy for what may block a merge.
-Scope: multiple teams.</t>
+Evidenced by: Standardizes the test-vs-eval discipline across teams with shared fixtures, replay harnesses, and CI policy for what may block a merge.</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets testing/verification discipline across the org.
-Evidenced by: Owns the org's verification strategy for AI systems, funding the harnesses that make the right split cheap and killing the theater.
-Scope: organization.</t>
+Evidenced by: Owns the org's verification strategy for AI systems, funding the harnesses that make the right split cheap and killing the theater.</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Depth: Shapes the company-wide quality culture; advances verification practice.
-Evidenced by: Sets company policy for what 'verified' means for AI products, traceable from CI to eval to production evidence.
-Scope: company.</t>
+Evidenced by: Sets company policy for what 'verified' means for AI products, traceable from CI to eval to production evidence.</t>
         </is>
       </c>
     </row>
@@ -1253,43 +1217,37 @@
       <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Depth: Uses AI coding tools with the output treated as a draft - reads every generated line, tests it, and can explain any part of the diff when asked.
-Evidenced by: Has the agent draft the schema-migration script, then reads and runs every line by hand and can walk a reviewer through why the down-migration is safe.
-Scope: task.</t>
+Evidenced by: Has the agent draft the schema-migration script, then reads and runs every line by hand and can walk a reviewer through why the down-migration is safe.</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
           <t>Depth: Calibrates when generation helps and when it misleads for the work at hand; catches plausible-but-wrong generated code before review, and their AI-assisted changes pass review at the same rate as hand-written ones.
-Evidenced by: Accepts the agent's generated boilerplate for a new API route unchanged but rewrites its generated cache-invalidation logic by hand after spotting a stale-read bug; their AI-assisted PRs land clean at the same rate as their hand-written ones.
-Scope: component.</t>
+Evidenced by: Accepts the agent's generated boilerplate for a new API route unchanged but rewrites its generated cache-invalidation logic by hand after spotting a stale-read bug; their AI-assisted PRs land clean at the same rate as their hand-written ones.</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets the norms for AI-assisted work in a domain - what may be delegated to agents, what verification it requires, how provenance is noted in review - and coaches others out of over-trust and under-use.
-Evidenced by: Writes the team's rule that agents may draft data-pipeline glue code unattended but never touch auth logic without a human diff review, and talks a skeptical teammate into trying agent-assisted refactors for mechanical renames instead of hand-editing forty files.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Writes the team's rule that agents may draft data-pipeline glue code unattended but never touch auth logic without a human diff review, and talks a skeptical teammate into trying agent-assisted refactors for mechanical renames instead of hand-editing forty files.</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines AI-assisted engineering practice across teams - where agents run in the delivery lifecycle, what gates their output - justified by throughput and defect data rather than vendor claims.
-Evidenced by: Decides, with six months of defect-escape data across three teams, which pipeline stages autonomous coding agents may run in unattended and which require a human gate before merge.
-Scope: multiple teams.</t>
+Evidenced by: Decides, with six months of defect-escape data across three teams, which pipeline stages autonomous coding agents may run in unattended and which require a human gate before merge.</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
           <t>Depth: Drives an organization's AI-augmented engineering strategy - tooling selection, workflow redesign, skill expectations - and adjusts policy from measured delivery outcomes.
-Evidenced by: Picks the org's standard coding-agent tooling after a bake-off, redesigns the PR template around provenance tags, and walks back a workflow change once the data shows it slowed incident response.
-Scope: organization.</t>
+Evidenced by: Picks the org's standard coding-agent tooling after a bake-off, redesigns the PR template around provenance tags, and walks back a workflow change once the data shows it slowed incident response.</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
           <t>Depth: Shapes how software engineering itself changes with AI at company and industry level; a credible public voice on what changes and what doesn't.
-Evidenced by: Writes the engineering blog post other companies cite when re-tooling their own build process around agentic coding.
-Scope: company.</t>
+Evidenced by: Writes the engineering blog post other companies cite when re-tooling their own build process around agentic coding.</t>
         </is>
       </c>
     </row>
@@ -1327,43 +1285,37 @@
       <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands LLM basics (tokens, context windows, temperature, system prompts); calls model APIs correctly.
-Evidenced by: Makes targeted edits to existing prompts and verifies the effect against known cases before committing, following the team's prompt-versioning convention.
-Scope: task.</t>
+Evidenced by: Makes targeted edits to existing prompts and verifies the effect against known cases before committing, following the team's prompt-versioning convention.</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Depth: Writes effective prompts; uses structured outputs, function calling and streaming; understands model differences and pricing.
-Evidenced by: Writes production prompts from scratch and iterates against a saved sample set rather than one lucky output.
-Scope: component.</t>
+Evidenced by: Writes production prompts from scratch and iterates against a saved sample set rather than one lucky output.</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert prompt/context design (few-shot, decomposition, chaining); knows when fine-tuning beats prompting (rarely); designs for model swappability.
-Evidenced by: Treats prompts as versioned, eval-gated artifacts and diagnoses failures to the responsible prompt section.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Treats prompts as versioned, eval-gated artifacts and diagnoses failures to the responsible prompt section.</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
           <t>Depth: Mastery of model behavior across providers and versions; designs upgrade-migration strategies; squeezes capability others can't.
-Evidenced by: Establishes prompt-engineering standards across teams and untangles the prompt failures others are stuck on.
-Scope: multiple teams.</t>
+Evidenced by: Establishes prompt-engineering standards across teams and untangles the prompt failures others are stuck on.</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
           <t>Depth: Deep expertise; anticipates capability shifts (new modalities, reasoning models) and repositions ahead of them.
-Evidenced by: Drives org-wide prompt and context craft, deciding where prompting ends and fine-tuning or tool-building begins.
-Scope: organization.</t>
+Evidenced by: Drives org-wide prompt and context craft, deciding where prompting ends and fine-tuning or tool-building begins.</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
           <t>Depth: Authority on applied LLM engineering; may influence industry practice.
-Evidenced by: Represents the state of the art to the company, resetting practice when model generations obsolete current techniques.
-Scope: company.</t>
+Evidenced by: Represents the state of the art to the company, resetting practice when model generations obsolete current techniques.</t>
         </is>
       </c>
     </row>
@@ -1401,43 +1353,37 @@
       <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands LLM basics (tokens, context windows, temperature, system prompts); calls model APIs correctly.
-Evidenced by: Integrates a specified model through the team's client layer per existing patterns.
-Scope: task.</t>
+Evidenced by: Integrates a specified model through the team's client layer per existing patterns.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
           <t>Depth: Writes effective prompts; uses structured outputs, function calling and streaming; understands model differences and pricing.
-Evidenced by: Runs a small structured comparison before picking a model for a feature and records the result.
-Scope: component.</t>
+Evidenced by: Runs a small structured comparison before picking a model for a feature and records the result.</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert prompt/context design (few-shot, decomposition, chaining); knows when fine-tuning beats prompting (rarely); designs for model swappability.
-Evidenced by: Owns model choice for a capability, re-benchmarks when providers ship new models, and swaps models behind stable interfaces without consumer churn.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Owns model choice for a capability, re-benchmarks when providers ship new models, and swaps models behind stable interfaces without consumer churn.</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
           <t>Depth: Mastery of model behavior across providers and versions; designs upgrade-migration strategies; squeezes capability others can't.
-Evidenced by: Defines the model-selection playbook and abstraction layers multiple teams use, making provider swaps routine instead of rewrites.
-Scope: multiple teams.</t>
+Evidenced by: Defines the model-selection playbook and abstraction layers multiple teams use, making provider swaps routine instead of rewrites.</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
           <t>Depth: Deep expertise; anticipates capability shifts (new modalities, reasoning models) and repositions ahead of them.
-Evidenced by: Sets the org's model portfolio strategy with cost and risk analysis leadership signs off on.
-Scope: organization.</t>
+Evidenced by: Sets the org's model portfolio strategy with cost and risk analysis leadership signs off on.</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
           <t>Depth: Authority on applied LLM engineering; may influence industry practice.
-Evidenced by: Owns the company's model-sourcing strategy and its biggest bets and negotiates the strategic provider commitments behind them.
-Scope: company.</t>
+Evidenced by: Owns the company's model-sourcing strategy and its biggest bets and negotiates the strategic provider commitments behind them.</t>
         </is>
       </c>
     </row>
@@ -1475,43 +1421,37 @@
       <c r="G11" s="4" t="inlineStr">
         <is>
           <t>Depth: Uses the codebase's shared contract types and schema validators at boundaries rather than hand-casting external data, and can point to where a type is checked at runtime.
-Evidenced by: Validates model outputs against a given schema and handles rejects rather than trusting parses.
-Scope: task.</t>
+Evidenced by: Validates model outputs against a given schema and handles rejects rather than trusting parses.</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
           <t>Depth: Puts runtime validation at every I/O boundary they touch — requests, messages, configuration — deriving static types from the runtime schemas so compile-time and runtime cannot drift.
-Evidenced by: Designs output schemas and tool signatures the model reliably satisfies, measuring parse and validation failure rates.
-Scope: component.</t>
+Evidenced by: Designs output schemas and tool signatures the model reliably satisfies, measuring parse and validation failure rates.</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs end-to-end type integrity for a capability — schema-first contracts, generated clients, contract drift caught in continuous integration — and blocks unsound casts and unvalidated edges in review.
-Evidenced by: Owns the structured-I/O layer for a capability — schema evolution, repair strategies, when to constrain decoding versus post-validate.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Owns the structured-I/O layer for a capability — schema evolution, repair strategies, when to constrain decoding versus post-validate.</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
           <t>Depth: Builds the code-generation and contract-typing infrastructure multiple teams inherit, making boundary safety the default rather than a discipline, and resolves cross-team type drift at its source.
-Evidenced by: Sets cross-team standards for tool definitions and output contracts and audits integrations that skip them.
-Scope: multiple teams.</t>
+Evidenced by: Sets cross-team standards for tool definitions and output contracts and audits integrations that skip them.</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets the organization's boundary-safety standard and the platform tooling that enforces it, with incident evidence showing the failure classes it removed.
-Evidenced by: Owns the org's model-I/O reliability strategy, driving shared validation infrastructure.
-Scope: organization.</t>
+Evidenced by: Owns the org's model-I/O reliability strategy, driving shared validation infrastructure.</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
           <t>Depth: Owns contract-integrity strategy across products and external interfaces where a broken contract is a business event, and advances the state of practice publicly.
-Evidenced by: Defines company-wide norms for machine-actionable model output, including what external partners may depend on.
-Scope: company.</t>
+Evidenced by: Defines company-wide norms for machine-actionable model output, including what external partners may depend on.</t>
         </is>
       </c>
     </row>
@@ -1549,43 +1489,37 @@
       <c r="G12" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands embeddings, similarity search and why grounding reduces hallucination.
-Evidenced by: Runs and modifies an existing ingestion/retrieval pipeline and verifies retrieval hits by inspection.
-Scope: task.</t>
+Evidenced by: Runs and modifies an existing ingestion/retrieval pipeline and verifies retrieval hits by inspection.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
           <t>Depth: Builds standard RAG pipelines (chunking, embedding, retrieval, reranking); manages context budgets deliberately.
-Evidenced by: Builds a retrieval pipeline for a corpus end to end and measures retrieval quality separately from answer quality.
-Scope: component.</t>
+Evidenced by: Builds a retrieval pipeline for a corpus end to end and measures retrieval quality separately from answer quality.</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs retrieval quality systems (hybrid search, reranking, freshness, citation, memory for multi-turn).
-Evidenced by: Diagnoses failures to the responsible stage with evidence and chooses hybrid, re-ranking, or structured-lookup strategies by measured trade-off.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Diagnoses failures to the responsible stage with evidence and chooses hybrid, re-ranking, or structured-lookup strategies by measured trade-off.</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in retrieval at scale (index strategy, multi-source federation, permission-aware retrieval).
-Evidenced by: Designs the retrieval architecture several teams share and consolidates duplicated pipelines into shared infrastructure.
-Scope: multiple teams.</t>
+Evidenced by: Designs the retrieval architecture several teams share and consolidates duplicated pipelines into shared infrastructure.</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
           <t>Depth: Deep expertise; anticipates how longer context and new architectures change retrieval economics.
-Evidenced by: Sets the org's knowledge-grounding strategy — what corpora exist, who owns them, entitlement-aware access, and quality accountability.
-Scope: organization.</t>
+Evidenced by: Sets the org's knowledge-grounding strategy — what corpora exist, who owns them, entitlement-aware access, and quality accountability.</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
           <t>Depth: Mastery of the discipline; defines how AI systems access knowledge.
-Evidenced by: Decides company-level grounding bets — proprietary-data moats, retrieval vs. long-context vs. fine-tuning — and owns that thesis with executives.
-Scope: company.</t>
+Evidenced by: Decides company-level grounding bets — proprietary-data moats, retrieval vs. long-context vs. fine-tuning — and owns that thesis with executives.</t>
         </is>
       </c>
     </row>
@@ -1623,43 +1557,37 @@
       <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands embeddings, similarity search and why grounding reduces hallucination.
-Evidenced by: Generates and stores embeddings using the team's pipeline and explains what an embedding represents in plain language.
-Scope: task.</t>
+Evidenced by: Generates and stores embeddings using the team's pipeline and explains what an embedding represents in plain language.</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Depth: Builds standard RAG pipelines (chunking, embedding, retrieval, reranking); manages context budgets deliberately.
-Evidenced by: Evaluates embedding models against the team's retrieval benchmarks and tunes similarity thresholds and index parameters with evidence.
-Scope: component.</t>
+Evidenced by: Evaluates embedding models against the team's retrieval benchmarks and tunes similarity thresholds and index parameters with evidence.</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs retrieval quality systems (hybrid search, reranking, freshness, citation, memory for multi-turn).
-Evidenced by: Selects embedding models, dimensions, and index types by measured trade-off for a capability and designs re-embedding and migration plans when models change.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Selects embedding models, dimensions, and index types by measured trade-off for a capability and designs re-embedding and migration plans when models change.</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in retrieval at scale (index strategy, multi-source federation, permission-aware retrieval).
-Evidenced by: Standardizes embedding infrastructure across teams — shared models, versioning, migration tooling — ending per-team drift.
-Scope: multiple teams.</t>
+Evidenced by: Standardizes embedding infrastructure across teams — shared models, versioning, migration tooling — ending per-team drift.</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
           <t>Depth: Deep expertise; anticipates how longer context and new architectures change retrieval economics.
-Evidenced by: Drives the org's vector-infrastructure strategy, including build-vs-buy for vector stores and cost and scale planning.
-Scope: organization.</t>
+Evidenced by: Drives the org's vector-infrastructure strategy, including build-vs-buy for vector stores and cost and scale planning.</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
           <t>Depth: Mastery of the discipline; defines how AI systems access knowledge.
-Evidenced by: Anticipates representation-layer shifts — multimodal embeddings, new architectures — and positions the company ahead of them.
-Scope: company.</t>
+Evidenced by: Anticipates representation-layer shifts — multimodal embeddings, new architectures — and positions the company ahead of them.</t>
         </is>
       </c>
     </row>
@@ -1697,43 +1625,37 @@
       <c r="G14" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands embeddings, similarity search and why grounding reduces hallucination.
-Evidenced by: Keeps requests within the context budget, truncating per team rules, and notices when overflow or truncation silently degrades output.
-Scope: task.</t>
+Evidenced by: Keeps requests within the context budget, truncating per team rules, and notices when overflow or truncation silently degrades output.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
           <t>Depth: Builds standard RAG pipelines (chunking, embedding, retrieval, reranking); manages context budgets deliberately.
-Evidenced by: Prioritizes what enters the window with explicit truncation rules and tests the effect of dropping each element.
-Scope: component.</t>
+Evidenced by: Prioritizes what enters the window with explicit truncation rules and tests the effect of dropping each element.</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs retrieval quality systems (hybrid search, reranking, freshness, citation, memory for multi-turn).
-Evidenced by: Designs the context-assembly strategy for a capability and shows with evals where added context stops paying.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Designs the context-assembly strategy for a capability and shows with evals where added context stops paying.</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in retrieval at scale (index strategy, multi-source federation, permission-aware retrieval).
-Evidenced by: Defines context-management patterns multiple teams reuse and audits high-cost windows for waste.
-Scope: multiple teams.</t>
+Evidenced by: Defines context-management patterns multiple teams reuse and audits high-cost windows for waste.</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
           <t>Depth: Deep expertise; anticipates how longer context and new architectures change retrieval economics.
-Evidenced by: Drives org-level context and memory architecture, deciding what user and org state is durable memory versus per-request context.
-Scope: organization.</t>
+Evidenced by: Drives org-level context and memory architecture, deciding what user and org state is durable memory versus per-request context.</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
           <t>Depth: Mastery of the discipline; defines how AI systems access knowledge.
-Evidenced by: Positions the company for context-regime shifts before they invalidate current designs.
-Scope: company.</t>
+Evidenced by: Positions the company for context-regime shifts before they invalidate current designs.</t>
         </is>
       </c>
     </row>
@@ -1771,43 +1693,37 @@
       <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands tool calling and the agent loop (plan, act, observe); knows why agents need constraints.
-Evidenced by: Traces an existing agent loop end to end, explaining why the agent took each step on a real transcript, and fixes defects in single steps.
-Scope: task.</t>
+Evidenced by: Traces an existing agent loop end to end, explaining why the agent took each step on a real transcript, and fixes defects in single steps.</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs good tool interfaces; builds single-agent workflows with sensible termination and confirmation points.
-Evidenced by: Builds single-agent workflows with a bounded tool set using the simplest pattern that works, with explicit termination conditions and step limits by default.
-Scope: component.</t>
+Evidenced by: Builds single-agent workflows with a bounded tool set using the simplest pattern that works, with explicit termination conditions and step limits by default.</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs reliable multi-step agents (state, recovery, sandboxing, permissions, human-in-the-loop); knows when an agent is the wrong answer.
-Evidenced by: Chooses between workflow and autonomous-loop designs by failure-mode analysis and cuts autonomy when a simpler pipeline scores the same.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Chooses between workflow and autonomous-loop designs by failure-mode analysis and cuts autonomy when a simpler pipeline scores the same.</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in complex orchestration (multi-agent, long-running workflows, MCP-style standards) and safe constraint at scale.
-Evidenced by: Sets the agent-architecture patterns multiple teams follow and kills over-engineered designs with evidence.
-Scope: multiple teams.</t>
+Evidenced by: Sets the agent-architecture patterns multiple teams follow and kills over-engineered designs with evidence.</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
           <t>Depth: Deep expertise; anticipates how increasing model autonomy changes system design.
-Evidenced by: Owns the org's agentic-systems strategy, deciding where autonomy is worth its reliability cost and what the shared platform provides.
-Scope: organization.</t>
+Evidenced by: Owns the org's agentic-systems strategy, deciding where autonomy is worth its reliability cost and what the shared platform provides.</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
           <t>Depth: Authority on agentic systems; may influence emerging industry standards.
-Evidenced by: Sets company direction on agentic products — where agents act, where humans decide — informed by what current models can actually sustain.
-Scope: company.</t>
+Evidenced by: Sets company direction on agentic products — where agents act, where humans decide — informed by what current models can actually sustain.</t>
         </is>
       </c>
     </row>
@@ -1845,43 +1761,37 @@
       <c r="G16" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands tool calling and the agent loop (plan, act, observe); knows why agents need constraints.
-Evidenced by: Implements a tool to a given schema with validation and error strings a model can act on, and tests it standalone before wiring it to a model.
-Scope: task.</t>
+Evidenced by: Implements a tool to a given schema with validation and error strings a model can act on, and tests it standalone before wiring it to a model.</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs good tool interfaces; builds single-agent workflows with sensible termination and confirmation points.
-Evidenced by: Designs tool schemas a model uses correctly on the first try and iterates on them against transcripts of real misuse.
-Scope: component.</t>
+Evidenced by: Designs tool schemas a model uses correctly on the first try and iterates on them against transcripts of real misuse.</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs reliable multi-step agents (state, recovery, sandboxing, permissions, human-in-the-loop); knows when an agent is the wrong answer.
-Evidenced by: Curates the tool surface of a capability — right granularity, idempotency and side-effect discipline, permission boundaries — pruning overlapping tools that confuse routing.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Curates the tool surface of a capability — right granularity, idempotency and side-effect discipline, permission boundaries — pruning overlapping tools that confuse routing.</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in complex orchestration (multi-agent, long-running workflows, MCP-style standards) and safe constraint at scale.
-Evidenced by: Defines tool-design standards and shared registries multiple teams consume, with review gates for high-risk tools, killing near-duplicate tools across agents.
-Scope: multiple teams.</t>
+Evidenced by: Defines tool-design standards and shared registries multiple teams consume, with review gates for high-risk tools, killing near-duplicate tools across agents.</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
           <t>Depth: Deep expertise; anticipates how increasing model autonomy changes system design.
-Evidenced by: Drives the org's tool and integration platform, deciding which internal systems get first-class tool interfaces.
-Scope: organization.</t>
+Evidenced by: Drives the org's tool and integration platform, deciding which internal systems get first-class tool interfaces.</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
           <t>Depth: Authority on agentic systems; may influence emerging industry standards.
-Evidenced by: Shapes the company's external tool ecosystem posture — what third parties may plug in, what the company exposes — as a durable interface bet.
-Scope: company.</t>
+Evidenced by: Shapes the company's external tool ecosystem posture — what third parties may plug in, what the company exposes — as a durable interface bet.</t>
         </is>
       </c>
     </row>
@@ -1919,43 +1829,37 @@
       <c r="G17" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands that models can be harmful, biased or confidently wrong; flags concerning behavior.
-Evidenced by: Implements the approval and confirmation steps a design specifies — never bypassing a human checkpoint without sign-off — and states which of their feature's actions are reversible.
-Scope: task.</t>
+Evidenced by: Implements the approval and confirmation steps a design specifies — never bypassing a human checkpoint without sign-off — and states which of their feature's actions are reversible.</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Depth: Implements guardrails (filtering, refusal handling, grounding checks); designs honest UX.
-Evidenced by: Designs approval gates by reversibility and blast radius, with dry-run modes, undo paths, and every escalation logged for audit.
-Scope: component.</t>
+Evidenced by: Designs approval gates by reversibility and blast radius, with dry-run modes, undo paths, and every escalation logged for audit.</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs layered safety proportional to stakes; evaluates for bias/misuse before launch.
-Evidenced by: Calibrates autonomy per action class for a capability from observed override and failure data, and pushes back when a design grants an agent more authority than its error rate supports.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Calibrates autonomy per action class for a capability from observed override and failure data, and pushes back when a design grants an agent more authority than its error rate supports.</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in safety system design at scale; defines oversight and escalation frameworks.
-Evidenced by: Standardizes autonomy tiers and approval mechanisms across teams and reviews escalation designs for high-consequence actions.
-Scope: multiple teams.</t>
+Evidenced by: Standardizes autonomy tiers and approval mechanisms across teams and reviews escalation designs for high-consequence actions.</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
           <t>Depth: Deep expertise balancing capability and safety under real product pressure.
-Evidenced by: Owns the org's policy for delegated agent authority, aligned with legal and security, including the evidence bar for widening autonomy.
-Scope: organization.</t>
+Evidenced by: Owns the org's policy for delegated agent authority, aligned with legal and security, including the evidence bar for widening autonomy.</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
           <t>Depth: Recognized authority; establishes responsible AI as a value; externally credible.
-Evidenced by: Decides how much authority the company delegates to AI systems in its products and operations and defends that line to regulators and customers.
-Scope: company.</t>
+Evidenced by: Decides how much authority the company delegates to AI systems in its products and operations and defends that line to regulators and customers.</t>
         </is>
       </c>
     </row>
@@ -1993,43 +1897,37 @@
       <c r="G18" s="4" t="inlineStr">
         <is>
           <t>Depth: Applies provided idempotency and retry patterns for simple cases under review.
-Evidenced by: Reproduces a failed agent run from its transcript and identifies the step where it went wrong — bad plan, bad tool result, lost state.
-Scope: task.</t>
+Evidenced by: Reproduces a failed agent run from its transcript and identifies the step where it went wrong — bad plan, bad tool result, lost state.</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Depth: Implements standard reliability and retry handling independently.
-Evidenced by: Builds checkpointing, retries, loop limits, and budget caps into agent steps so a wandering run halts cheaply and an interrupted run resumes or fails cleanly.
-Scope: component.</t>
+Evidenced by: Builds checkpointing, retries, loop limits, and budget caps into agent steps so a wandering run halts cheaply and an interrupted run resumes or fails cleanly.</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs idempotent, reliable flows autonomously; resolves duplicate and partial-failure cases.
-Evidenced by: Designs the state and containment model for an agentic capability, quantifying compounded failure rates rather than trusting per-step accuracy, and proves recovery paths with fault injection.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Designs the state and containment model for an agentic capability, quantifying compounded failure rates rather than trusting per-step accuracy, and proves recovery paths with fault injection.</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines reliability patterns teams adopt; solves the hardest exactly-once and recovery problems.
-Evidenced by: Sets durable-execution and recovery patterns multiple teams adopt — resumable run state, saga-style compensation — with adoption they can show.
-Scope: multiple teams.</t>
+Evidenced by: Sets durable-execution and recovery patterns multiple teams adopt — resumable run state, saga-style compensation — with adoption they can show.</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets reliability and idempotency strategy across systems; anticipates evolving failure modes.
-Evidenced by: Drives the org's strategy for stateful, long-running AI execution, consolidating bespoke run-state code into platform, with reliability targets and failure drills.
-Scope: organization.</t>
+Evidenced by: Drives the org's strategy for stateful, long-running AI execution, consolidating bespoke run-state code into platform, with reliability targets and failure drills.</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines best practice for reliability patterns industrywide; shapes widely adopted approaches.
-Evidenced by: Sets company reliability doctrine for autonomous systems, informing what the company will and won't promise customers.
-Scope: company.</t>
+Evidenced by: Sets company reliability doctrine for autonomous systems, informing what the company will and won't promise customers.</t>
         </is>
       </c>
     </row>
@@ -2067,43 +1965,37 @@
       <c r="G19" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands tool calling and the agent loop (plan, act, observe); knows why agents need constraints.
-Evidenced by: Runs agents in the sandboxed environment provided and reports containment gaps they notice.
-Scope: task.</t>
+Evidenced by: Runs agents in the sandboxed environment provided and reports containment gaps they notice.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs good tool interfaces; builds single-agent workflows with sensible termination and confirmation points.
-Evidenced by: Scopes an agent's credentials and tool permissions to least privilege, and caps loops, spend, and side effects by construction.
-Scope: component.</t>
+Evidenced by: Scopes an agent's credentials and tool permissions to least privilege, and caps loops, spend, and side effects by construction.</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs reliable multi-step agents (state, recovery, sandboxing, permissions, human-in-the-loop); knows when an agent is the wrong answer.
-Evidenced by: Designs containment for a capability's agents — sandboxing, budget kill-switches, reversible-by-default actions — and red-teams their own boundaries before launch.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Designs containment for a capability's agents — sandboxing, budget kill-switches, reversible-by-default actions — and red-teams their own boundaries before launch.</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in complex orchestration (multi-agent, long-running workflows, MCP-style standards) and safe constraint at scale.
-Evidenced by: Builds containment infrastructure several teams inherit rather than reimplement, and audits exceptions.
-Scope: multiple teams.</t>
+Evidenced by: Builds containment infrastructure several teams inherit rather than reimplement, and audits exceptions.</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
           <t>Depth: Deep expertise; anticipates how increasing model autonomy changes system design.
-Evidenced by: Sets the org's containment standards for autonomous systems and verifies them through game days.
-Scope: organization.</t>
+Evidenced by: Sets the org's containment standards for autonomous systems and verifies them through game days.</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
           <t>Depth: Authority on agentic systems; may influence emerging industry standards.
-Evidenced by: Owns the company's worst-case analysis for agentic products and the controls that bound it.
-Scope: company.</t>
+Evidenced by: Owns the company's worst-case analysis for agentic products and the controls that bound it.</t>
         </is>
       </c>
     </row>
@@ -2141,43 +2033,37 @@
       <c r="G20" s="4" t="inlineStr">
         <is>
           <t>Depth: Labels data to clear guidelines and flags ambiguities under review.
-Evidenced by: Adds well-formed cases to an existing eval set, labeling edge cases consistently with the rubric and flagging ambiguous ones instead of guessing.
-Scope: task.</t>
+Evidenced by: Adds well-formed cases to an existing eval set, labeling edge cases consistently with the rubric and flagging ambiguous ones instead of guessing.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
           <t>Depth: Curates and labels routine datasets independently, applying consistent guidelines.
-Evidenced by: Builds an eval set for a feature from production traces via error analysis, versioning golden data like code with documented inclusion criteria.
-Scope: component.</t>
+Evidenced by: Builds an eval set for a feature from production traces via error analysis, versioning golden data like code with documented inclusion criteria.</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs labeling schemes and resolves ambiguity and quality issues autonomously.
-Evidenced by: Owns the golden datasets of a capability, retiring stale cases and tracing every regression escape back to the missing case class.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Owns the golden datasets of a capability, retiring stale cases and tracing every regression escape back to the missing case class.</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines curation and annotation-quality standards others adopt.
-Evidenced by: Sets eval-data standards multiple teams follow and audits suites whose numbers look too good.
-Scope: multiple teams.</t>
+Evidenced by: Sets eval-data standards multiple teams follow and audits suites whose numbers look too good.</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets dataset strategy and anticipates shifts in labeling and curation practice.
-Evidenced by: Drives the org's evaluation-data strategy — shared corpora, labeling operations, data governance for eval assets.
-Scope: organization.</t>
+Evidenced by: Drives the org's evaluation-data strategy — shared corpora, labeling operations, data governance for eval assets.</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines industry best practice for dataset curation and is externally credible.
-Evidenced by: Defines how the company knows its AI works — the evidence doctrine cited in launch reviews and external claims.
-Scope: company.</t>
+Evidenced by: Defines how the company knows its AI works — the evidence doctrine cited in launch reviews and external claims.</t>
         </is>
       </c>
     </row>
@@ -2215,43 +2101,37 @@
       <c r="G21" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands why 'it looked right in testing' is insufficient; runs existing evals and labels carefully.
-Evidenced by: Runs the eval harness and reads its reports correctly, distinguishing a real regression from noise with help and flagging results that look wrong instead of accepting them.
-Scope: task.</t>
+Evidenced by: Runs the eval harness and reads its reports correctly, distinguishing a real regression from noise with help and flagging results that look wrong instead of accepting them.</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
           <t>Depth: Builds basic eval sets from real usage; measures changes before shipping prompt/model updates.
-Evidenced by: Chooses graders that fit the behavior under test and spot-checks judge agreement against their own labels before trusting it.
-Scope: component.</t>
+Evidenced by: Chooses graders that fit the behavior under test and spot-checks judge agreement against their own labels before trusting it.</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs eval methodology (golden sets, LLM-as-judge with validation, human review, helpfulness/groundedness/safety metrics).
-Evidenced by: Designs the measurement itself for a capability — judges validated against human ratings with quantified agreement and bias, significance limits stated before declaring a win.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Designs the measurement itself for a capability — judges validated against human ratings with quantified agreement and bias, significance limits stated before declaring a win.</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in eval at scale (continuous eval, A/B testing AI features, drift detection).
-Evidenced by: Standardizes eval methodology across teams, calibrating judge models centrally so scores are comparable.
-Scope: multiple teams.</t>
+Evidenced by: Standardizes eval methodology across teams, calibrating judge models centrally so scores are comparable.</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
           <t>Depth: Deep expertise in measuring AI quality where ground truth is contested.
-Evidenced by: Owns the org's measurement strategy for AI quality, connecting offline evals to online outcomes and killing metrics that don't predict.
-Scope: organization.</t>
+Evidenced by: Owns the org's measurement strategy for AI quality, connecting offline evals to online outcomes and killing metrics that don't predict.</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
           <t>Depth: Mastery of the discipline; sets the bar for what 'proven to work' means.
-Evidenced by: Defines what 'good' means for the company's AI products in measurable terms executives, customers, and regulators accept.
-Scope: company.</t>
+Evidenced by: Defines what 'good' means for the company's AI products in measurable terms executives, customers, and regulators accept.</t>
         </is>
       </c>
     </row>
@@ -2289,43 +2169,37 @@
       <c r="G22" s="4" t="inlineStr">
         <is>
           <t>Depth: Adds tests to existing pipeline stages following defined configuration, reviewed before merge.
-Evidenced by: Runs the required evals before merging prompt or model changes and pastes results into the review, flagging regressions instead of explaining them away.
-Scope: task.</t>
+Evidenced by: Runs the required evals before merging prompt or model changes and pastes results into the review, flagging regressions instead of explaining them away.</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
           <t>Depth: Integrates and maintains automated test stages independently within standard pipelines.
-Evidenced by: Attaches eval deltas to every prompt, model, or retrieval change and blocks their own launches on regressions without being told.
-Scope: component.</t>
+Evidenced by: Attaches eval deltas to every prompt, model, or retrieval change and blocks their own launches on regressions without being told.</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs fast, reliable test gating for complex pipelines balancing speed and confidence.
-Evidenced by: Defines the ship gate for a capability — which evals block release, what regression tolerance is, when human review is required — and holds the line under deadline pressure with the reasoning in writing.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Defines the ship gate for a capability — which evals block release, what regression tolerance is, when human review is required — and holds the line under deadline pressure with the reasoning in writing.</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines continuous-testing patterns and gating strategy other teams adopt.
-Evidenced by: Installs measurement-gated release processes across teams — eval CI, canary analysis, staged rollouts teams actually use — and audits exceptions.
-Scope: multiple teams.</t>
+Evidenced by: Installs measurement-gated release processes across teams — eval CI, canary analysis, staged rollouts teams actually use — and audits exceptions.</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets continuous-testing strategy and anticipates how quality gates must evolve with delivery.
-Evidenced by: Owns the org's ship/no-ship framework for AI behavior changes and arbitrates escalations where speed and evidence conflict.
-Scope: organization.</t>
+Evidenced by: Owns the org's ship/no-ship framework for AI behavior changes and arbitrates escalations where speed and evidence conflict.</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines authoritative continuous-testing practice that shapes the discipline.
-Evidenced by: Sets company policy on the evidence required to ship AI behavior, balancing speed and risk explicitly.
-Scope: company.</t>
+Evidenced by: Sets company policy on the evidence required to ship AI behavior, balancing speed and risk explicitly.</t>
         </is>
       </c>
     </row>
@@ -2363,43 +2237,37 @@
       <c r="G23" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands logs/metrics/traces; reads existing dashboards.
-Evidenced by: Uses existing traces to debug a failing request — walking prompt to retrieval to tool call to output — and adds a missing span when told what to capture.
-Scope: task.</t>
+Evidenced by: Uses existing traces to debug a failing request — walking prompt to retrieval to tool call to output — and adds a missing span when told what to capture.</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
           <t>Depth: Instruments their services; builds dashboards; tunes alerts to limit noise.
-Evidenced by: Instruments a component end to end as structured spans with the metadata needed to reproduce any output later, with sampling and redaction applied correctly.
-Scope: component.</t>
+Evidenced by: Instruments a component end to end as structured spans with the metadata needed to reproduce any output later, with sampling and redaction applied correctly.</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs observability for complex systems (end-to-end traces, quality signals, cost attribution).
-Evidenced by: Designs the observability schema for a capability and builds the views that make failure clusters visible, answering 'why did this output happen' in minutes.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Designs the observability schema for a capability and builds the views that make failure clusters visible, answering 'why did this output happen' in minutes.</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in instrumentation trade-offs at scale, incl. privacy-safe logging.
-Evidenced by: Sets tracing conventions multiple teams emit, aligning attributes so cross-service AI requests join up in one lens.
-Scope: multiple teams.</t>
+Evidenced by: Sets tracing conventions multiple teams emit, aligning attributes so cross-service AI requests join up in one lens.</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines org observability strategy.
-Evidenced by: Owns the org's AI observability platform strategy, including retention, privacy, and cost of trace data.
-Scope: organization.</t>
+Evidenced by: Owns the org's AI observability platform strategy, including retention, privacy, and cost of trace data.</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
           <t>Depth: Shapes company-wide operational visibility; advances practice.
-Evidenced by: Ensures the company can answer 'why did the model do that?' for any production decision, as a matter of architecture.
-Scope: company.</t>
+Evidenced by: Ensures the company can answer 'why did the model do that?' for any production decision, as a matter of architecture.</t>
         </is>
       </c>
     </row>
@@ -2437,43 +2305,37 @@
       <c r="G24" s="4" t="inlineStr">
         <is>
           <t>Depth: Watches configured monitors and reports alerts under guidance.
-Evidenced by: Watches the dashboards for their feature after deploys and escalates anomalies with the trace attached rather than assuming success.
-Scope: task.</t>
+Evidenced by: Watches the dashboards for their feature after deploys and escalates anomalies with the trace attached rather than assuming success.</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets up standard performance and drift monitoring independently.
-Evidenced by: Builds behavioral monitors for a component with alert thresholds they can justify, promoting recurring failures into the eval set.
-Scope: component.</t>
+Evidenced by: Builds behavioral monitors for a component with alert thresholds they can justify, promoting recurring failures into the eval set.</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs monitoring that catches subtle drift and degradation autonomously and triages causes.
-Evidenced by: Detects silent degradation for a capability — baselines behavior, catches provider-side model changes and input-distribution drift — and has caught a real regression no user reported.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Detects silent degradation for a capability — baselines behavior, catches provider-side model changes and input-distribution drift — and has caught a real regression no user reported.</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines monitoring and drift-detection patterns others adopt.
-Evidenced by: Standardizes behavioral monitoring and feedback-to-eval pipelines across teams, correlating cross-product regressions to a common upstream cause.
-Scope: multiple teams.</t>
+Evidenced by: Standardizes behavioral monitoring and feedback-to-eval pipelines across teams, correlating cross-product regressions to a common upstream cause.</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets monitoring strategy and anticipates advances in drift detection.
-Evidenced by: Owns the org's in-production AI quality picture, making drift review a routine practice with owners and SLAs.
-Scope: organization.</t>
+Evidenced by: Owns the org's in-production AI quality picture, making drift review a routine practice with owners and SLAs.</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines best practice for model monitoring and is externally credible.
-Evidenced by: Makes behavioral health a company-level operational metric, defining how the company absorbs provider upgrades without quality surprises.
-Scope: company.</t>
+Evidenced by: Makes behavioral health a company-level operational metric, defining how the company absorbs provider upgrades without quality surprises.</t>
         </is>
       </c>
     </row>
@@ -2511,43 +2373,37 @@
       <c r="G25" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands SLOs and common failure modes; keeps components healthy with guidance.
-Evidenced by: Implements the retry, timeout, and fallback behavior a design specifies and tests the failure path by forcing the failure, not just the happy path.
-Scope: task.</t>
+Evidenced by: Implements the retry, timeout, and fallback behavior a design specifies and tests the failure path by forcing the failure, not just the happy path.</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
           <t>Depth: Builds retries, timeouts and fallbacks; understands blast radius.
-Evidenced by: Designs the degradation ladder for a component — retry budgets, circuit breaking on provider errors, cached or smaller-model fallbacks — and makes each rung observable.
-Scope: component.</t>
+Evidenced by: Designs the degradation ladder for a component — retry budgets, circuit breaking on provider errors, cached or smaller-model fallbacks — and makes each rung observable.</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs for graceful degradation; defines SLOs; accountable for a domain's reliability.
-Evidenced by: Owns availability design for a capability across providers — failover routing, brownout modes, load shedding — validated with game days rather than hope.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Owns availability design for a capability across providers — failover routing, brownout modes, load shedding — validated with game days rather than hope.</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in resilience and capacity planning at scale; drives down incidents systemically.
-Evidenced by: Builds the shared resilience layer multiple teams depend on and reviews launches for shared-fate provider risk.
-Scope: multiple teams.</t>
+Evidenced by: Builds the shared resilience layer multiple teams depend on and reviews launches for shared-fate provider risk.</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
           <t>Depth: Owns org-level reliability; fixes risk in process and org design.
-Evidenced by: Owns org-level continuity for provider failure — multi-provider posture, capacity reservations, tested playbooks.
-Scope: organization.</t>
+Evidenced by: Owns org-level continuity for provider failure — multi-provider posture, capacity reservations, tested playbooks.</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets the company's reliability philosophy.
-Evidenced by: Answers for company availability of AI products through provider incidents that make the news, setting the architecture doctrine behind the commitments.
-Scope: company.</t>
+Evidenced by: Answers for company availability of AI products through provider incidents that make the news, setting the architecture doctrine behind the commitments.</t>
         </is>
       </c>
     </row>
@@ -2585,43 +2441,37 @@
       <c r="G26" s="4" t="inlineStr">
         <is>
           <t>Depth: Responds to alerts with support; follows runbooks; escalates appropriately.
-Evidenced by: Follows the runbook during incidents, keeps the timeline updated, captures the traces responders need, and asks for help early.
-Scope: task.</t>
+Evidenced by: Follows the runbook during incidents, keeps the timeline updated, captures the traces responders need, and asks for help early.</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
           <t>Depth: Triages and resolves routine incidents; clear notes; takes on-call.
-Evidenced by: Debugs live model-system incidents independently — distinguishing provider outage from prompt regression from data problem — and writes the postmortem with concrete actions.
-Scope: component.</t>
+Evidenced by: Debugs live model-system incidents independently — distinguishing provider outage from prompt regression from data problem — and writes the postmortem with concrete actions.</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
           <t>Depth: Leads response to complex failures; blameless postmortems; same failure never recurs.
-Evidenced by: Incident-commands for their capability, including quality and cost incidents that page no one by default, and drives postmortems to systemic fixes.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Incident-commands for their capability, including quality and cost incidents that page no one by default, and drives postmortems to systemic fixes.</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in incident-management design (rotations, severity, escalation).
-Evidenced by: Raises operational maturity across teams — severity definitions that include model-quality events, game days for AI failure classes, readiness reviews before launches.
-Scope: multiple teams.</t>
+Evidenced by: Raises operational maturity across teams — severity definitions that include model-quality events, game days for AI failure classes, readiness reviews before launches.</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
           <t>Depth: Commands the highest-severity incidents; sets incident process org-wide.
-Evidenced by: Owns the org's incident-management standard for AI systems, reviewing the postmortems that cross team boundaries and closing systemic gaps.
-Scope: organization.</t>
+Evidenced by: Owns the org's incident-management standard for AI systems, reviewing the postmortems that cross team boundaries and closing systemic gaps.</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets the company's incident philosophy; calm authority in the worst moments.
-Evidenced by: Is the company's senior technical responder in its worst AI incidents and changes company practice from what they reveal.
-Scope: company.</t>
+Evidenced by: Is the company's senior technical responder in its worst AI incidents and changes company practice from what they reveal.</t>
         </is>
       </c>
     </row>
@@ -2659,43 +2509,37 @@
       <c r="G27" s="4" t="inlineStr">
         <is>
           <t>Depth: Gathers usage metrics and applies simple capacity estimates under guidance.
-Evidenced by: Monitors quota and rate-limit dashboards for their service and escalates approaching limits before they bite.
-Scope: task.</t>
+Evidenced by: Monitors quota and rate-limit dashboards for their service and escalates approaching limits before they bite.</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
           <t>Depth: Produces standard capacity forecasts and resource budgets independently.
-Evidenced by: Implements rate limiting, request queuing, and backoff for a component and tracks provider deprecation notices that affect it.
-Scope: component.</t>
+Evidenced by: Implements rate limiting, request queuing, and backoff for a component and tracks provider deprecation notices that affect it.</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
           <t>Depth: Plans capacity autonomously; models demand, headroom, and resource trade-offs.
-Evidenced by: Plans capacity for a capability — load forecasting, quota negotiation inputs, multi-region or multi-provider failover design — and runs model-version migrations without user-visible regression.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Plans capacity for a capability — load forecasting, quota negotiation inputs, multi-region or multi-provider failover design — and runs model-version migrations without user-visible regression.</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines capacity-planning approaches teams adopt; solves hard forecasting and efficiency problems.
-Evidenced by: Runs cross-team capacity and migration programs — org-wide model deprecation moves, shared quota pooling — that land on schedule.
-Scope: multiple teams.</t>
+Evidenced by: Runs cross-team capacity and migration programs — org-wide model deprecation moves, shared quota pooling — that land on schedule.</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets capacity and resource-budgeting strategy across systems; anticipates long-term demand shifts.
-Evidenced by: Owns the org's provider risk management — concentration risk, contractual SLAs, burst capacity.
-Scope: organization.</t>
+Evidenced by: Owns the org's provider risk management — concentration risk, contractual SLAs, burst capacity.</t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr">
         <is>
           <t>Depth: Shapes industry practice for capacity planning; pioneers influential approaches to resource budgeting.
-Evidenced by: Sets company posture on model-supply resilience as a business-continuity matter leadership understands.
-Scope: company.</t>
+Evidenced by: Sets company posture on model-supply resilience as a business-continuity matter leadership understands.</t>
         </is>
       </c>
     </row>
@@ -2733,43 +2577,37 @@
       <c r="G28" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands cost/latency drivers of what they build.
-Evidenced by: States what their feature costs per request, attributing spend to prompt size, output length, and call count correctly, and checks the dashboard after changes ship.
-Scope: task.</t>
+Evidenced by: States what their feature costs per request, attributing spend to prompt size, output length, and call count correctly, and checks the dashboard after changes ship.</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
           <t>Depth: Applies standard optimizations; stays within cost/latency budgets.
-Evidenced by: Cuts a component's cost with measured, quality-neutral levers — prompt trimming, caching, batching, output caps — and reports the before/after against any quality change.
-Scope: component.</t>
+Evidenced by: Cuts a component's cost with measured, quality-neutral levers — prompt trimming, caching, batching, output caps — and reports the before/after against any quality change.</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs cost-aware architectures; defines and tracks unit economics for a domain.
-Evidenced by: Owns the cost model of a capability — cost per request and per user action tracked against quality, budgets and anomaly alerts set, cost-quality trades explicit in design docs.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Owns the cost model of a capability — cost per request and per user action tracked against quality, budgets and anomaly alerts set, cost-quality trades explicit in design docs.</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in economics at scale (fleet optimization, build-vs-buy).
-Evidenced by: Finds the cross-team cost structure — shared caches, duplicated calls, misrouted traffic — and drives the fixes worth the most, with cost governance teams adopt.
-Scope: multiple teams.</t>
+Evidenced by: Finds the cross-team cost structure — shared caches, duplicated calls, misrouted traffic — and drives the fixes worth the most, with cost governance teams adopt.</t>
         </is>
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
           <t>Depth: Owns org-level spend strategy; cost decisions change margins.
-Evidenced by: Owns the org's inference-spend strategy — forecasting at product scale, informing provider negotiations, deciding where cost work beats feature work.
-Scope: organization.</t>
+Evidenced by: Owns the org's inference-spend strategy — forecasting at product scale, informing provider negotiations, deciding where cost work beats feature work.</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
           <t>Depth: Shapes the company economics of the products.
-Evidenced by: Keeps AI gross margins viable at company level, shaping pricing and architecture together.
-Scope: company.</t>
+Evidenced by: Keeps AI gross margins viable at company level, shaping pricing and architecture together.</t>
         </is>
       </c>
     </row>
@@ -2807,43 +2645,37 @@
       <c r="G29" s="4" t="inlineStr">
         <is>
           <t>Depth: Deploys models to a serving setup with given configs under review.
-Evidenced by: Measures end-to-end latency for their feature — including time-to-first-token — and identifies the slowest stage from traces.
-Scope: task.</t>
+Evidenced by: Measures end-to-end latency for their feature — including time-to-first-token — and identifies the slowest stage from traces.</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
           <t>Depth: Serves models independently and applies standard latency and throughput tuning.
-Evidenced by: Applies standard latency levers independently — streaming, parallel calls, speculative work, caching — to hit a stated target, validated with p95, not averages.
-Scope: component.</t>
+Evidenced by: Applies standard latency levers independently — streaming, parallel calls, speculative work, caching — to hit a stated target, validated with p95, not averages.</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
           <t>Depth: Optimizes serving for hard latency, scale, and cost constraints autonomously.
-Evidenced by: Right-sizes models per task within a capability — proving with evals that the smaller, faster model holds the quality bar — and defines latency SLOs users actually feel.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Right-sizes models per task within a capability — proving with evals that the smaller, faster model holds the quality bar — and defines latency SLOs users actually feel.</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines serving and inference-optimization patterns others adopt.
-Evidenced by: Builds or mandates the routing and caching infrastructure multiple teams use to meet shared latency standards, and audits over-provisioned model use.
-Scope: multiple teams.</t>
+Evidenced by: Builds or mandates the routing and caching infrastructure multiple teams use to meet shared latency standards, and audits over-provisioned model use.</t>
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets serving strategy and anticipates advances in inference efficiency.
-Evidenced by: Sets the org's latency/quality/cost frontier and the serving investments that move it.
-Scope: organization.</t>
+Evidenced by: Sets the org's latency/quality/cost frontier and the serving investments that move it.</t>
         </is>
       </c>
       <c r="L29" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines best practice for model serving across the discipline and is externally recognized.
-Evidenced by: Makes speed a company-level product advantage, deciding where the company competes on latency and the architectural commitments behind it.
-Scope: company.</t>
+Evidenced by: Makes speed a company-level product advantage, deciding where the company competes on latency and the architectural commitments behind it.</t>
         </is>
       </c>
     </row>
@@ -2881,43 +2713,37 @@
       <c r="G30" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands core appsec; follows practices and flags concerns.
-Evidenced by: Treats model output and retrieved content as untrusted — never executes, renders, or queries with it unescaped — and can explain injection with a real example.
-Scope: task.</t>
+Evidenced by: Treats model output and retrieved content as untrusted — never executes, renders, or queries with it unescaped — and can explain injection with a real example.</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
           <t>Depth: Applies least privilege; validates/sanitizes inputs; knows common attacks.
-Evidenced by: Builds injection defenses into a component — privilege separation between instructions and data, output validation, allowlisted tool arguments — and writes adversarial cases into its tests.
-Scope: component.</t>
+Evidenced by: Builds injection defenses into a component — privilege separation between instructions and data, output validation, allowlisted tool arguments — and writes adversarial cases into its tests.</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs defense in depth; thinks in abuse cases; owns a domain's posture.
-Evidenced by: Threat-models a capability's model I/O paths end to end, designs least-privilege mitigations accepted by security review, and red-teams their own features before attackers do.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Threat-models a capability's model I/O paths end to end, designs least-privilege mitigations accepted by security review, and red-teams their own features before attackers do.</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in securing systems at scale; leads red-teaming and remediation.
-Evidenced by: Sets secure-by-default patterns for model I/O that multiple teams inherit from shared libraries and runs adversarial reviews of high-exposure launches.
-Scope: multiple teams.</t>
+Evidenced by: Sets secure-by-default patterns for model I/O that multiple teams inherit from shared libraries and runs adversarial reviews of high-exposure launches.</t>
         </is>
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines security strategy for the org's surface area.
-Evidenced by: Owns the org's LLM security program with the security org — threat models, red-team cadence, incident learnings folded back into platform defaults.
-Scope: organization.</t>
+Evidenced by: Owns the org's LLM security program with the security org — threat models, red-team cadence, incident learnings folded back into platform defaults.</t>
         </is>
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
           <t>Depth: Company-level accountability; authority on the field.
-Evidenced by: Is accountable for the company's AI attack surface — deciding what the company will and won't expose to untrusted input — and represents the posture to customers, auditors, and researchers.
-Scope: company.</t>
+Evidenced by: Is accountable for the company's AI attack surface — deciding what the company will and won't expose to untrusted input — and represents the posture to customers, auditors, and researchers.</t>
         </is>
       </c>
     </row>
@@ -2955,43 +2781,37 @@
       <c r="G31" s="4" t="inlineStr">
         <is>
           <t>Depth: Knows data handling has privacy implications; follows rules.
-Evidenced by: Follows the team's rules for what may enter prompts, logs, and eval data, and asks before sending a new data category to a model provider.
-Scope: task.</t>
+Evidenced by: Follows the team's rules for what may enter prompts, logs, and eval data, and asks before sending a new data category to a model provider.</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
           <t>Depth: Applies PII handling, redaction, residency and retention correctly.
-Evidenced by: Implements redaction and minimization in a component's pipelines and verifies with tests that sensitive fields don't leak into telemetry.
-Scope: component.</t>
+Evidenced by: Implements redaction and minimization in a component's pipelines and verifies with tests that sensitive fields don't leak into telemetry.</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs for compliance (consent, audit trails, regional rules); owns readiness for a domain.
-Evidenced by: Owns the data-flow map of a capability end to end — what user data reaches which provider under what retention terms — and catches new leak paths in design review.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Owns the data-flow map of a capability end to end — what user data reaches which provider under what retention terms — and catches new leak paths in design review.</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert at translating regulation into controls; represents engineering in audits.
-Evidenced by: Standardizes privacy engineering for AI across teams — shared redaction tooling, review checklists, provider data-processing requirements — and audits the highest-sensitivity data flows.
-Scope: multiple teams.</t>
+Evidenced by: Standardizes privacy engineering for AI across teams — shared redaction tooling, review checklists, provider data-processing requirements — and audits the highest-sensitivity data flows.</t>
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets org compliance strategy; anticipates regulation.
-Evidenced by: Owns the org's data posture toward model providers, partnering with legal on agreements, audits, and the hard cases like eval data versus deletion requests.
-Scope: organization.</t>
+Evidenced by: Owns the org's data posture toward model providers, partnering with legal on agreements, audits, and the hard cases like eval data versus deletion requests.</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
           <t>Depth: Authoritative on the landscape; trusted interface to regulators.
-Evidenced by: Answers for the company's AI data-handling promises — what is committed to customers about their data, and the architecture that keeps it true.
-Scope: company.</t>
+Evidenced by: Answers for the company's AI data-handling promises — what is committed to customers about their data, and the architecture that keeps it true.</t>
         </is>
       </c>
     </row>
@@ -3029,43 +2849,37 @@
       <c r="G32" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands that models can be harmful, biased or confidently wrong; flags concerning behavior.
-Evidenced by: Wires existing guardrails into a feature, verifies rejects follow the designed path, and escalates outputs that feel harmful rather than shipping past them.
-Scope: task.</t>
+Evidenced by: Wires existing guardrails into a feature, verifies rejects follow the designed path, and escalates outputs that feel harmful rather than shipping past them.</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
           <t>Depth: Implements guardrails (filtering, refusal handling, grounding checks); designs honest UX.
-Evidenced by: Implements layered guardrails for a component and measures their false-positive and false-negative rates instead of assuming they work.
-Scope: component.</t>
+Evidenced by: Implements layered guardrails for a component and measures their false-positive and false-negative rates instead of assuming they work.</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs layered safety proportional to stakes; evaluates for bias/misuse before launch.
-Evidenced by: Designs the control stack for a capability from a written risk analysis, testing guardrails adversarially before launch and owning the harm/annoyance trade explicitly.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Designs the control stack for a capability from a written risk analysis, testing guardrails adversarially before launch and owning the harm/annoyance trade explicitly.</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert in safety system design at scale; defines oversight and escalation frameworks.
-Evidenced by: Standardizes guardrail patterns and shared safety infrastructure across teams, with authority to block a ship on control gaps.
-Scope: multiple teams.</t>
+Evidenced by: Standardizes guardrail patterns and shared safety infrastructure across teams, with authority to block a ship on control gaps.</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
           <t>Depth: Deep expertise balancing capability and safety under real product pressure.
-Evidenced by: Owns the org's output-safety standards and red-teaming program, reporting residual risk honestly to leadership.
-Scope: organization.</t>
+Evidenced by: Owns the org's output-safety standards and red-teaming program, reporting residual risk honestly to leadership.</t>
         </is>
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
           <t>Depth: Recognized authority; establishes responsible AI as a value; externally credible.
-Evidenced by: Defines the company's safety bar for AI products — what its AI refuses, allows, and how that is defended publicly — including saying no to launches.
-Scope: company.</t>
+Evidenced by: Defines the company's safety bar for AI products — what its AI refuses, allows, and how that is defended publicly — including saying no to launches.</t>
         </is>
       </c>
     </row>
@@ -3103,43 +2917,37 @@
       <c r="G33" s="4" t="inlineStr">
         <is>
           <t>Depth: Runs prescribed bias and error checks under review.
-Evidenced by: Recognizes and reports harmful or biased outputs found during development instead of shrugging them off as model quirks.
-Scope: task.</t>
+Evidenced by: Recognizes and reports harmful or biased outputs found during development instead of shrugging them off as model quirks.</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
           <t>Depth: Performs standard fairness and error analysis independently for routine models.
-Evidenced by: Tests a component against the team's harm checklist and adds mitigations that measurably reduce hits.
-Scope: component.</t>
+Evidenced by: Tests a component against the team's harm checklist and adds mitigations that measurably reduce hits.</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
           <t>Depth: Diagnoses subtle bias and failure modes in ambiguous cases and proposes remedies autonomously.
-Evidenced by: Defines the harm profile for a capability, ships mitigations with eval coverage per harm class, and makes a written ship/hold recommendation leadership can act on.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Defines the harm profile for a capability, ships mitigations with eval coverage per harm class, and makes a written ship/hold recommendation leadership can act on.</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines fairness and error-analysis frameworks others adopt.
-Evidenced by: Sets harm-analysis practice across teams and reviews launches with meaningful harm potential, arbitrating safety-vs-utility disputes with data.
-Scope: multiple teams.</t>
+Evidenced by: Sets harm-analysis practice across teams and reviews launches with meaningful harm potential, arbitrating safety-vs-utility disputes with data.</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets fairness strategy and anticipates evolving ethical and regulatory expectations.
-Evidenced by: Operationalizes the org's responsible-AI commitments into engineering requirements teams can actually implement.
-Scope: organization.</t>
+Evidenced by: Operationalizes the org's responsible-AI commitments into engineering requirements teams can actually implement.</t>
         </is>
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
           <t>Depth: Shapes industry practice for fairness and error analysis and is externally recognized.
-Evidenced by: Shapes the company's public safety posture and is accountable for it holding under scrutiny.
-Scope: company.</t>
+Evidenced by: Shapes the company's public safety posture and is accountable for it holding under scrutiny.</t>
         </is>
       </c>
     </row>
@@ -3177,43 +2985,37 @@
       <c r="G34" s="4" t="inlineStr">
         <is>
           <t>Depth: Completes the risk checklist for their change accurately - identifying who is affected if the model is wrong - and escalates anything the checklist doesn't cover.
-Evidenced by: Fills out the launch checklist noting that a wrong classification would misroute a customer's support ticket to the wrong queue, and flags to their lead that the checklist has no question covering non-English input.
-Scope: task.</t>
+Evidenced by: Fills out the launch checklist noting that a wrong classification would misroute a customer's support ticket to the wrong queue, and flags to their lead that the checklist has no question covering non-English input.</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
           <t>Depth: Assesses a feature's failure impact before build (misuse, error harm, disparate performance across user groups) and documents mitigations and residual risk unprompted.
-Evidenced by: Documents, before building a resume-screening feature, that the model underperforms on non-standard formats and adds a low-confidence-score fallback to human review without being asked.
-Scope: component.</t>
+Evidenced by: Documents, before building a resume-screening feature, that the model underperforms on non-standard formats and adds a low-confidence-score fallback to human review without being asked.</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
           <t>Depth: Classifies a domain against the applicable risk framework, keeps its evidence pack (evals, controls, incidents) audit-ready, converts findings into engineering requirements with owners, and flags when a product change alters the risk class.
-Evidenced by: Classifies the support-triage capability as limited-risk under the applicable framework, keeps its eval and incident log current for the quarterly audit, and flags to legal when a new use case would push it toward high-risk.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Classifies the support-triage capability as limited-risk under the applicable framework, keeps its eval and incident log current for the quarterly audit, and flags to legal when a new use case would push it toward high-risk.</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
           <t>Depth: Operates a cross-team AI risk-review process - fast enough that teams use it honestly, rigorous enough to catch real issues - and builds governance tooling that makes compliance a byproduct of normal engineering.
-Evidenced by: Runs the weekly cross-team risk-review that every AI launch across four teams goes through, and ships the CI check that blocks a PR missing a risk classification before a human has to catch it.
-Scope: multiple teams.</t>
+Evidenced by: Runs the weekly cross-team risk-review that every AI launch across four teams goes through, and ships the CI check that blocks a PR missing a risk classification before a human has to catch it.</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
           <t>Depth: Owns an organization's AI governance program jointly with legal and risk functions, translating regulation into engineering requirements without freezing delivery.
-Evidenced by: Co-owns the org's AI governance program with legal, turning a new regulation's high-risk-system obligations into a pre-launch checklist that ships features on schedule instead of stalling in review.
-Scope: organization.</t>
+Evidenced by: Co-owns the org's AI governance program with legal, turning a new regulation's high-risk-system obligations into a pre-launch checklist that ships features on schedule instead of stalling in review.</t>
         </is>
       </c>
       <c r="L34" s="4" t="inlineStr">
         <is>
           <t>Depth: Positions a company ahead of AI regulation; accountable to executives, boards, and regulators for where the risk lines are drawn.
-Evidenced by: Briefs the board on where the company draws its AI risk lines before a regulator asks, and represents the company's position in an industry working group shaping upcoming AI-regulation guidance.
-Scope: company.</t>
+Evidenced by: Briefs the board on where the company draws its AI risk lines before a regulator asks, and represents the company's position in an industry working group shaping upcoming AI-regulation guidance.</t>
         </is>
       </c>
     </row>
@@ -3251,43 +3053,37 @@
       <c r="G35" s="4" t="inlineStr">
         <is>
           <t>Depth: Translates a clearly scoped problem into a defined ML task under guidance.
-Evidenced by: States what user problem their task serves and raises it when a lookup table or heuristic would do what the ticket asks of a model.
-Scope: task.</t>
+Evidenced by: States what user problem their task serves and raises it when a lookup table or heuristic would do what the ticket asks of a model.</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
           <t>Depth: Frames routine problems as appropriate ML solutions independently.
-Evidenced by: Prototypes the simplest adequate approach first — rules, search, classical ML, or a model — and recommends the model only when it beats the baseline, with the comparison documented.
-Scope: component.</t>
+Evidenced by: Prototypes the simplest adequate approach first — rules, search, classical ML, or a model — and recommends the model only when it beats the baseline, with the comparison documented.</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
           <t>Depth: Frames ambiguous business problems into sound ML or non-ML approaches autonomously.
-Evidenced by: Kills LLM-shaped solutions to non-LLM problems in design review with evidence, reframing vague 'add AI' asks into testable user outcomes product partners agree to.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Kills LLM-shaped solutions to non-LLM problems in design review with evidence, reframing vague 'add AI' asks into testable user outcomes product partners agree to.</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines solution-design patterns others adopt and reframes intractable problems.
-Evidenced by: Installs solution-fit review in how multiple teams take on AI work, redirecting AI-for-its-own-sake proposals and unwinding the most expensive misfit projects.
-Scope: multiple teams.</t>
+Evidenced by: Installs solution-fit review in how multiple teams take on AI work, redirecting AI-for-its-own-sake proposals and unwinding the most expensive misfit projects.</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets ML solution strategy and anticipates where applicable techniques are heading.
-Evidenced by: Shapes which problems the org points AI at, pairing with product leadership on where models genuinely change the offering and cancelling bets the evidence turns against.
-Scope: organization.</t>
+Evidenced by: Shapes which problems the org points AI at, pairing with product leadership on where models genuinely change the offering and cancelling bets the evidence turns against.</t>
         </is>
       </c>
       <c r="L35" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines best practice for ML problem framing across the discipline and is externally recognized.
-Evidenced by: Advises company leadership on what AI makes newly possible versus fashionable — and is right often enough to be believed.
-Scope: company.</t>
+Evidenced by: Advises company leadership on what AI makes newly possible versus fashionable — and is right often enough to be believed.</t>
         </is>
       </c>
     </row>
@@ -3325,43 +3121,37 @@
       <c r="G36" s="4" t="inlineStr">
         <is>
           <t>Depth: Understands the capability they're building and who uses it.
-Evidenced by: States how their feature's success will be measured beyond 'it works' and checks the metric after launch rather than moving on.
-Scope: task.</t>
+Evidenced by: States how their feature's success will be measured beyond 'it works' and checks the metric after launch rather than moving on.</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
           <t>Depth: Frames own work in user/business outcomes, not just tasks.
-Evidenced by: Defines success metrics with product partners before building and reports post-launch results honestly, including misses.
-Scope: component.</t>
+Evidenced by: Defines success metrics with product partners before building and reports post-launch results honestly, including misses.</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
           <t>Depth: Treats their area as a product; uses metrics to decide what to build for a domain.
-Evidenced by: Connects a capability's engineering metrics to business outcomes — cost per outcome, retention, task completion — and recommends sunsetting features whose value evidence never arrives.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Connects a capability's engineering metrics to business outcomes — cost per outcome, retention, task completion — and recommends sunsetting features whose value evidence never arrives.</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert at aligning technical bets with product strategy across teams.
-Evidenced by: Builds the value-measurement discipline multiple teams use for AI investments, surfacing which bets are and aren't paying off.
-Scope: multiple teams.</t>
+Evidenced by: Builds the value-measurement discipline multiple teams use for AI investments, surfacing which bets are and aren't paying off.</t>
         </is>
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets product direction for an org's technical surface.
-Evidenced by: Owns the org's account of AI value delivered, credible to finance and product alike, and reallocates engineering toward what the evidence supports.
-Scope: organization.</t>
+Evidenced by: Owns the org's account of AI value delivered, credible to finance and product alike, and reallocates engineering toward what the evidence supports.</t>
         </is>
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
           <t>Depth: Shapes how the company creates value through technical products.
-Evidenced by: Shapes how the company invests in AI based on demonstrated value, with numbers that survive diligence at board level.
-Scope: company.</t>
+Evidenced by: Shapes how the company invests in AI based on demonstrated value, with numbers that survive diligence at board level.</t>
         </is>
       </c>
     </row>
@@ -3399,43 +3189,37 @@
       <c r="G37" s="4" t="inlineStr">
         <is>
           <t>Depth: Learns to estimate; surfaces blockers; plans own tasks with guidance.
-Evidenced by: Breaks their work into small verifiable increments and flags early — with evidence — when the model can't do what the task assumed, instead of grinding silently.
-Scope: task.</t>
+Evidenced by: Breaks their work into small verifiable increments and flags early — with evidence — when the model can't do what the task assumed, instead of grinding silently.</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
           <t>Depth: Estimates scoped work realistically; plans own 1-3 week projects.
-Evidenced by: Plans feature work as a de-risking sequence — timeboxed feasibility spike, eval baseline, then build — giving estimates as ranges with stated confidence.
-Scope: component.</t>
+Evidenced by: Plans feature work as a de-risking sequence — timeboxed feasibility spike, eval baseline, then build — giving estimates as ranges with stated confidence.</t>
         </is>
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
           <t>Depth: Plans quarter-scale, multi-workstream efforts including dependencies.
-Evidenced by: Structures a capability's roadmap around its riskiest unknowns — feasibility gates before commitments, kill criteria stated before the spike starts and honored when triggered.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Structures a capability's roadmap around its riskiest unknowns — feasibility gates before commitments, kill criteria stated before the spike starts and honored when triggered.</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert at planning large programs; anticipates risk early.
-Evidenced by: Teaches teams to plan AI work honestly — separating engineering certainty from model uncertainty in commitments leaders can rely on — and de-risks the org's biggest AI commitments personally.
-Scope: multiple teams.</t>
+Evidenced by: Teaches teams to plan AI work honestly — separating engineering certainty from model uncertainty in commitments leaders can rely on — and de-risks the org's biggest AI commitments personally.</t>
         </is>
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
           <t>Depth: Plans org-level programs across quarters/years.
-Evidenced by: Shapes the org's portfolio of AI bets, balancing near-certain delivery against high-variance exploration and keeping leadership expectations calibrated to what evals actually show.
-Scope: organization.</t>
+Evidenced by: Shapes the org's portfolio of AI bets, balancing near-certain delivery against high-variance exploration and keeping leadership expectations calibrated to what evals actually show.</t>
         </is>
       </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
           <t>Depth: Shapes how the company plans major technical change.
-Evidenced by: Times company bets against the model-capability curve — what to build now versus wait for — and is accountable for the calls.
-Scope: company.</t>
+Evidenced by: Times company bets against the model-capability curve — what to build now versus wait for — and is accountable for the calls.</t>
         </is>
       </c>
     </row>
@@ -3473,43 +3257,37 @@
       <c r="G38" s="4" t="inlineStr">
         <is>
           <t>Depth: Follows the release process exactly — flags, staged rollout steps, verification checklists — verifies their change in production, and rolls back with guidance.
-Evidenced by: Ships work in small reviewable increments behind flags as directed and rolls back their own change cleanly when asked.
-Scope: task.</t>
+Evidenced by: Ships work in small reviewable increments behind flags as directed and rolls back their own change cleanly when asked.</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
           <t>Depth: Ships behind flags with a rollback plan by default, monitors rollouts and reverts on their own judgment when signals degrade, and writes changes that tolerate both versions running during rollout.
-Evidenced by: Designs a component's rollout as canary -&gt; percentage -&gt; full, watching evals and telemetry at each stage and rolling back on their own signal.
-Scope: component.</t>
+Evidenced by: Designs a component's rollout as canary -&gt; percentage -&gt; full, watching evals and telemetry at each stage and rolling back on their own signal.</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
           <t>Depth: Designs the rollout for risky changes — canary criteria, migration sequencing, flag lifecycle, kill switches — and reviews others' rollout plans for blast radius; the person teams ask how to ship something safely.
-Evidenced by: Owns progressive-delivery strategy for a capability — shadow modes for new models, reversible-by-design changes, automated rollback triggers — and their launches are uneventful.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Owns progressive-delivery strategy for a capability — shadow modes for new models, reversible-by-design changes, automated rollback triggers — and their launches are uneventful.</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
           <t>Depth: Builds progressive-delivery machinery multiple teams release through (flag platforms, automated canary analysis, automated rollback), retiring deploy patterns that cause repeat incidents and measurably raising deploy frequency.
-Evidenced by: Builds the progressive-delivery machinery multiple teams use for AI changes — flag conventions, automated rollback on eval regression.
-Scope: multiple teams.</t>
+Evidenced by: Builds the progressive-delivery machinery multiple teams use for AI changes — flag conventions, automated rollback on eval regression.</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
           <t>Depth: Owns release policy for an organization and its delivery metrics — rollout standards, freeze rules, environment strategy — dismantling ceremony that adds no safety.
-Evidenced by: Sets the org's release-engineering direction for AI products and its risk appetite per surface.
-Scope: organization.</t>
+Evidenced by: Sets the org's release-engineering direction for AI products and its risk appetite per surface.</t>
         </is>
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets how an entire company's software reaches customers — the risk posture products ship under — and defends it to executives, auditors, and regulators.
-Evidenced by: Makes safe iteration speed a company capability competitors can't easily copy.
-Scope: company.</t>
+Evidenced by: Makes safe iteration speed a company capability competitors can't easily copy.</t>
         </is>
       </c>
     </row>
@@ -3547,43 +3325,37 @@
       <c r="G39" s="4" t="inlineStr">
         <is>
           <t>Depth: Takes ownership of assigned tasks; honest about progress and blockers.
-Evidenced by: Tells their lead two days early that the eval-harness ticket will slip because the golden dataset isn't ready, instead of going quiet until standup.
-Scope: task.</t>
+Evidenced by: Tells their lead two days early that the eval-harness ticket will slip because the golden dataset isn't ready, instead of going quiet until standup.</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
           <t>Depth: Owns components end-to-end; delivers committed work reliably.
-Evidenced by: Delivers the retrieval-reranking component on the date they committed to, having flagged and absorbed a provider API change mid-sprint without missing the deadline.
-Scope: component.</t>
+Evidenced by: Delivers the retrieval-reranking component on the date they committed to, having flagged and absorbed a provider API change mid-sprint without missing the deadline.</t>
         </is>
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
           <t>Depth: Owns a domain; lands multi-week efforts without surprises; pushes back on unrealistic scope with reasons.
-Evidenced by: Owns the chatbot capability through a six-week model migration with no surprise regressions, and talks product out of a two-week scope add with a written cost estimate.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Owns the chatbot capability through a six-week model migration with no surprise regressions, and talks product out of a two-week scope add with a written cost estimate.</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
           <t>Depth: Owns cross-team initiatives; unblocks teams; kills failing approaches early.
-Evidenced by: Runs the cross-team migration off the deprecated embedding model, unblocking two teams stuck on the same provider quota issue and cutting a doomed fine-tuning effort before it burns another sprint.
-Scope: multiple teams.</t>
+Evidenced by: Runs the cross-team migration off the deprecated embedding model, unblocking two teams stuck on the same provider quota issue and cutting a doomed fine-tuning effort before it burns another sprint.</t>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
           <t>Depth: Owns an org-level portfolio of bets; sets direction others follow.
-Evidenced by: Owns the org's portfolio of AI reliability bets for the year, and three other teams plan their roadmaps around the sequencing they set.
-Scope: organization.</t>
+Evidenced by: Owns the org's portfolio of AI reliability bets for the year, and three other teams plan their roadmaps around the sequencing they set.</t>
         </is>
       </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
           <t>Depth: The go-to when something company-critical must land.
-Evidenced by: Is who leadership calls in when the flagship AI feature's launch is at risk two weeks out, and lands it.
-Scope: company.</t>
+Evidenced by: Is who leadership calls in when the flagship AI feature's launch is at risk two weeks out, and lands it.</t>
         </is>
       </c>
     </row>
@@ -3621,43 +3393,37 @@
       <c r="G40" s="4" t="inlineStr">
         <is>
           <t>Depth: Communicates status clearly; documentation is accurate.
-Evidenced by: Writes clear task updates, commit messages, and questions with enough context that responders don't have to ask for it, summarizing eval results without overstating them.
-Scope: task.</t>
+Evidenced by: Writes clear task updates, commit messages, and questions with enough context that responders don't have to ask for it, summarizing eval results without overstating them.</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
           <t>Depth: Writes clear design notes, runbooks and PRs; explains trade-offs without overselling.
-Evidenced by: Writes design notes and runbooks peers act on without follow-up questions, and explains model behavior and its limits to non-experts without jargon or overclaiming.
-Scope: component.</t>
+Evidenced by: Writes design notes and runbooks peers act on without follow-up questions, and explains model behavior and its limits to non-experts without jargon or overclaiming.</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
           <t>Depth: Writes design docs that drive decisions; translates technical risk for non-technical stakeholders.
-Evidenced by: Writes the docs that settle decisions and translates eval results and AI trade-offs so accurately that product decisions built on their word hold up.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Writes the docs that settle decisions and translates eval results and AI trade-offs so accurately that product decisions built on their word hold up.</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert at making complex capability/risk legible to executives without dumbing it down; RFCs align orgs.
-Evidenced by: Aligns multiple teams through writing — RFCs, strategies, decision records cited months later as the reference — and presents AI capability and risk to leadership without dumbing it down.
-Scope: multiple teams.</t>
+Evidenced by: Aligns multiple teams through writing — RFCs, strategies, decision records cited months later as the reference — and presents AI capability and risk to leadership without dumbing it down.</t>
         </is>
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
           <t>Depth: Strategy memos leadership acts on; org-wide and external reach.
-Evidenced by: Communicates org-level technical direction upward and outward, translating between executive and engineering registers without loss, including bad news early.
-Scope: organization.</t>
+Evidenced by: Communicates org-level technical direction upward and outward, translating between executive and engineering registers without loss, including bad news early.</t>
         </is>
       </c>
       <c r="L40" s="4" t="inlineStr">
         <is>
           <t>Depth: A clarifying voice at company scale; externally recognized.
-Evidenced by: Is the company's technical voice on AI internally and externally — talks, publications, customer and regulator conversations that move the company's position.
-Scope: company.</t>
+Evidenced by: Is the company's technical voice on AI internally and externally — talks, publications, customer and regulator conversations that move the company's position.</t>
         </is>
       </c>
     </row>
@@ -3695,43 +3461,37 @@
       <c r="G41" s="4" t="inlineStr">
         <is>
           <t>Depth: Responsive to feedback; pairs willingly; asks for help appropriately.
-Evidenced by: Works effectively with designer and PM counterparts on task details, surfacing AI-specific constraints — latency, failure modes — early, and incorporates feedback without churn.
-Scope: task.</t>
+Evidenced by: Works effectively with designer and PM counterparts on task details, surfacing AI-specific constraints — latency, failure modes — early, and incorporates feedback without churn.</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
           <t>Depth: Collaborates smoothly with adjacent functions; handles disagreement constructively.
-Evidenced by: Partners with product and design on what the model can and can't support, involving them before the prompt is final and prototyping to resolve disagreements with evidence.
-Scope: component.</t>
+Evidenced by: Partners with product and design on what the model can and can't support, involving them before the prompt is final and prototyping to resolve disagreements with evidence.</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
           <t>Depth: Builds strong cross-team relationships; resolves friction directly.
-Evidenced by: Runs the cross-functional process for a capability — brings legal, security, and support in before launch, turns product intent into evaluable requirements — and resolves conflicts between functions without escalation.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Runs the cross-functional process for a capability — brings legal, security, and support in before launch, turns product intent into evaluable requirements — and resolves conflicts between functions without escalation.</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
           <t>Depth: Expert at aligning teams with competing priorities; mediates disputes between senior people.
-Evidenced by: Fixes broken cross-team interfaces — ownership gaps, handoff friction — building the review forums, interface agreements, and shared vocabularies several teams use.
-Scope: multiple teams.</t>
+Evidenced by: Fixes broken cross-team interfaces — ownership gaps, handoff friction — building the review forums, interface agreements, and shared vocabularies several teams use.</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
           <t>Depth: Creates the forums and processes through which collaboration happens.
-Evidenced by: Builds the org's operating model between AI engineering and other functions — data, platform, trust, product — so work flows without heroics.
-Scope: organization.</t>
+Evidenced by: Builds the org's operating model between AI engineering and other functions — data, platform, trust, product — so work flows without heroics.</t>
         </is>
       </c>
       <c r="L41" s="4" t="inlineStr">
         <is>
           <t>Depth: Builds coalitions at company scale and externally.
-Evidenced by: Brokers company-level alignment on AI initiatives across executive functions with durable results.
-Scope: company.</t>
+Evidenced by: Brokers company-level alignment on AI initiatives across executive functions with durable results.</t>
         </is>
       </c>
     </row>
@@ -3769,43 +3529,37 @@
       <c r="G42" s="4" t="inlineStr">
         <is>
           <t>Depth: Shares what they learn; keeps their docs accurate.
-Evidenced by: Keeps the docs for what they build current — setup, known limits, gotchas — and files gaps they find in others'.
-Scope: task.</t>
+Evidenced by: Keeps the docs for what they build current — setup, known limits, gotchas — and files gaps they find in others'.</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
           <t>Depth: Documents their area well; proactively shares techniques with the team.
-Evidenced by: Documents a feature's behavior contract — intended use, eval results, failure modes, escalation paths — findable by the next engineer without asking.
-Scope: component.</t>
+Evidenced by: Documents a feature's behavior contract — intended use, eval results, failure modes, escalation paths — findable by the next engineer without asking.</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
           <t>Depth: Creates documentation and forums that raise a whole domain's understanding.
-Evidenced by: Maintains the canonical documentation for a capability — architecture, prompt rationale, eval history, runbooks — and prunes stale docs as ruthlessly as stale code.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Maintains the canonical documentation for a capability — architecture, prompt rationale, eval history, runbooks — and prunes stale docs as ruthlessly as stale code.</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
           <t>Depth: Builds knowledge-sharing systems adopted across teams.
-Evidenced by: Drives documentation standards for AI systems across teams — behavior cards, decision records — and reviews for compliance.
-Scope: multiple teams.</t>
+Evidenced by: Drives documentation standards for AI systems across teams — behavior cards, decision records — and reviews for compliance.</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
           <t>Depth: Defines how the org captures and spreads knowledge.
-Evidenced by: Builds the org's AI knowledge base as infrastructure, making internal expertise discoverable.
-Scope: organization.</t>
+Evidenced by: Builds the org's AI knowledge base as infrastructure, making internal expertise discoverable.</t>
         </is>
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
           <t>Depth: Shapes industry-facing knowledge practice.
-Evidenced by: Externalizes company knowledge deliberately — publications, standards participation — where it compounds the company's position.
-Scope: company.</t>
+Evidenced by: Externalizes company knowledge deliberately — publications, standards participation — where it compounds the company's position.</t>
         </is>
       </c>
     </row>
@@ -3843,43 +3597,37 @@
       <c r="G43" s="4" t="inlineStr">
         <is>
           <t>Depth: Receptive to mentoring; shares what they learn.
-Evidenced by: Asks for help effectively and pays it forward, documenting what they learned where the next person will find it.
-Scope: task.</t>
+Evidenced by: Asks for help effectively and pays it forward, documenting what they learned where the next person will find it.</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
           <t>Depth: Helps onboard teammates; informally mentors juniors.
-Evidenced by: Onboards new teammates onto the AI stack and pairs generously, turning their own review comments and repeated questions into reusable explanations.
-Scope: component.</t>
+Evidenced by: Onboards new teammates onto the AI stack and pairs generously, turning their own review comments and repeated questions into reusable explanations.</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
           <t>Depth: Coaches engineers with growth-oriented feedback; measurably improves a team's skill.
-Evidenced by: Mentors engineers deliberately — stretch tasks matched to gaps, feedback that names behavior and impact — and levels a team up on AI-specific craft it didn't have before; mentees ship independently sooner.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Mentors engineers deliberately — stretch tasks matched to gaps, feedback that names behavior and impact — and levels a team up on AI-specific craft it didn't have before; mentees ship independently sooner.</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
           <t>Depth: Develops future leads across teams; shapes hiring and onboarding.
-Evidenced by: Grows senior engineers across teams, sponsoring others into leading work they would have led, and builds the guilds and curricula that scale beyond one-on-ones.
-Scope: multiple teams.</t>
+Evidenced by: Grows senior engineers across teams, sponsoring others into leading work they would have led, and builds the guilds and curricula that scale beyond one-on-ones.</t>
         </is>
       </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
           <t>Depth: Develops senior engineers and leaders; builds culture deliberately.
-Evidenced by: Builds the org's AI-engineering bench — hiring bar, growth paths, promotion evidence, succession for critical systems.
-Scope: organization.</t>
+Evidenced by: Builds the org's AI-engineering bench — hiring bar, growth paths, promotion evidence, succession for critical systems.</t>
         </is>
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
           <t>Depth: Develops the next generation of top talent; legacy outlasts tenure.
-Evidenced by: Develops the company's next generation of principal-level technical leaders, largely through others, and shapes how the company is known to candidates.
-Scope: company.</t>
+Evidenced by: Develops the company's next generation of principal-level technical leaders, largely through others, and shapes how the company is known to candidates.</t>
         </is>
       </c>
     </row>
@@ -3917,43 +3665,37 @@
       <c r="G44" s="4" t="inlineStr">
         <is>
           <t>Depth: Contributes informed opinions in technical discussions.
-Evidenced by: Volunteers for unglamorous work that unblocks others and raises risks early instead of waiting to be asked.
-Scope: task.</t>
+Evidenced by: Volunteers for unglamorous work that unblocks others and raises risks early instead of waiting to be asked.</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
           <t>Depth: Influences component-level decisions through credibility.
-Evidenced by: Leads small technical efforts end to end — a migration, an integration — coordinating the people involved without formal authority or escalation.
-Scope: component.</t>
+Evidenced by: Leads small technical efforts end to end — a migration, an integration — coordinating the people involved without formal authority or escalation.</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
           <t>Depth: Sets technical direction for a domain; others align to their calls.
-Evidenced by: Sets technical direction for a capability — making and documenting the contentious calls, taking responsibility when wrong — and is the engineer others seek out when an AI decision is stuck.
-Scope: capability / domain (terminal level).</t>
+Evidenced by: Sets technical direction for a capability — making and documenting the contentious calls, taking responsibility when wrong — and is the engineer others seek out when an AI decision is stuck.</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
           <t>Depth: Shapes how multiple teams approach problems; trusted tiebreaker.
-Evidenced by: Creates alignment across teams that don't report to them, landing multi-team initiatives — platform migrations, model transitions — through writing, relationships, and demonstrated judgment.
-Scope: multiple teams.</t>
+Evidenced by: Creates alignment across teams that don't report to them, landing multi-team initiatives — platform migrations, model transitions — through writing, relationships, and demonstrated judgment.</t>
         </is>
       </c>
       <c r="K44" s="4" t="inlineStr">
         <is>
           <t>Depth: Influences org-wide technical strategy.
-Evidenced by: Drives the org's technical strategy for AI, choosing the few bets that matter and getting leadership and teams genuinely behind them.
-Scope: organization.</t>
+Evidenced by: Drives the org's technical strategy for AI, choosing the few bets that matter and getting leadership and teams genuinely behind them.</t>
         </is>
       </c>
       <c r="L44" s="4" t="inlineStr">
         <is>
           <t>Depth: Influences company strategic direction through insight.
-Evidenced by: Sets the company's long-term technical direction for AI, accountable for the bets years before they resolve.
-Scope: company.</t>
+Evidenced by: Sets the company's long-term technical direction for AI, accountable for the bets years before they resolve.</t>
         </is>
       </c>
     </row>

</xml_diff>